<commit_message>
Add Playground page with 2 mock projects
- New section #playground: same project card format as Projects,
  no category tabs, with search and pagination
- Extract buildProjectCard() helper shared by Projects and Playground
- Playground sheet in data.xlsx: Portfolio Website, Test Report Generator
- i18n keys for EN/TH; section-desc styling; dark mode support
- config.js: playground: true between projects and join

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Certifications" sheetId="7" r:id="rId7"/>
     <sheet name="Awards" sheetId="8" r:id="rId8"/>
     <sheet name="Tools" sheetId="9" r:id="rId9"/>
+    <sheet name="Playground" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -453,8 +454,8 @@
         <v>QA Lead with 14+ years across game development and software testing. ISTQB CTFL certified, passionate about quality, automation, and growing teams.</v>
       </c>
       <c r="D2" t="str" xml:space="preserve">
-        <v xml:space="preserve">I have over 10 years of experience in game development across various roles, including Production Manager, and more than 8 years in Quality Assurance with a current focus on software testing. While I am now primarily involved in non-gaming software projects, I maintain a strong passion for the gaming industry and bring a solid understanding of both game production pipelines and modern software development practices, including CI/CD processes._x000d__x000d__x000d__x000d_
-_x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">I have over 10 years of experience in game development across various roles, including Production Manager, and more than 8 years in Quality Assurance with a current focus on software testing. While I am now primarily involved in non-gaming software projects, I maintain a strong passion for the gaming industry and bring a solid understanding of both game production pipelines and modern software development practices, including CI/CD processes._x000d__x000d__x000d__x000d__x000d_
+_x000d__x000d__x000d__x000d__x000d_
 In addition to my technical expertise, I actively mentor team members and take pride in sharing knowledge to help others grow. I believe in building strong, collaborative teams and creating an environment that supports continuous learning. I have been certified with ISTQB CTFL since 2019 and as an Agile Tester (AT) in 2024.</v>
       </c>
       <c r="E2" t="str">
@@ -470,8 +471,8 @@
         <v>QA Lead ที่คลุกคลีกับวงการพัฒนาเกมและทดสอบซอฟต์แวร์มากว่า 14 ปี ได้รับการรับรอง ISTQB CTFL ชอบงานที่เกี่ยวกับคุณภาพ ระบบทดสอบอัตโนมัติ และการพาทีมเติบโตไปด้วยกัน</v>
       </c>
       <c r="I2" t="str" xml:space="preserve">
-        <v xml:space="preserve">ทำงานในวงการเกมมากว่า 10 ปี ผ่านหลายบทบาท รวมถึงตำแหน่ง Production Manager และมีประสบการณ์ด้าน QA อีกกว่า 8 ปี ปัจจุบันโฟกัสที่งานทดสอบซอฟต์แวร์เป็นหลัก แม้จะย้ายมาทำสายซอฟต์แวร์ทั่วไปแล้ว แต่ยังหลงรักวงการเกมอยู่เสมอ และเข้าใจทั้งกระบวนการผลิตเกมและการพัฒนาซอฟต์แวร์สมัยใหม่ รวมถึงงานสาย CI/CD เป็นอย่างดี_x000d__x000d__x000d__x000d_
-_x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">ทำงานในวงการเกมมากว่า 10 ปี ผ่านหลายบทบาท รวมถึงตำแหน่ง Production Manager และมีประสบการณ์ด้าน QA อีกกว่า 8 ปี ปัจจุบันโฟกัสที่งานทดสอบซอฟต์แวร์เป็นหลัก แม้จะย้ายมาทำสายซอฟต์แวร์ทั่วไปแล้ว แต่ยังหลงรักวงการเกมอยู่เสมอ และเข้าใจทั้งกระบวนการผลิตเกมและการพัฒนาซอฟต์แวร์สมัยใหม่ รวมถึงงานสาย CI/CD เป็นอย่างดี_x000d__x000d__x000d__x000d__x000d_
+_x000d__x000d__x000d__x000d__x000d_
 นอกจากเรื่องเทคนิคแล้ว ยังชอบทำหน้าที่เป็น Mentor ให้น้องๆ ในทีม และยินดีแบ่งปันความรู้เพื่อให้ทุกคนเก่งขึ้นไปด้วยกัน เชื่อในเรื่องการสร้างทีมที่แข็งแรงและบรรยากาศที่เอื้อให้ทุกคนได้เรียนรู้ตลอดเวลา ได้รับการรับรอง ISTQB CTFL ตั้งแต่ปี 2019 และ Agile Tester (AT) ในปี 2024</v>
       </c>
       <c r="J2" t="str">
@@ -485,6 +486,113 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Project name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Project name_TH</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Duration</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Project URL</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Project overview</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Project overview_TH</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Roles and Responsibility</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Skills and Tools</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Image_Folder</v>
+      </c>
+      <c r="J1" t="str">
+        <v>YouTube</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Portfolio Website</v>
+      </c>
+      <c r="B2" t="str">
+        <v>เว็บ Portfolio</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2025</v>
+      </c>
+      <c r="D2" t="str">
+        <v>https://monwork.onrender.com</v>
+      </c>
+      <c r="E2" t="str">
+        <v>A personal portfolio website built with vanilla HTML, CSS, and JavaScript — no frameworks. All data is managed through a single Excel file and rendered client-side using SheetJS. Features SPA routing, bilingual support, dark mode, contact form via Formspree, and project gallery.</v>
+      </c>
+      <c r="F2" t="str">
+        <v>เว็บ portfolio ส่วนตัวที่สร้างด้วย HTML, CSS และ JavaScript ล้วน ไม่ใช้ framework ข้อมูลทั้งหมดจัดการผ่าน Excel อ่านค่าฝั่ง client ด้วย SheetJS รองรับ 2 ภาษา dark mode และ gallery รูปภาพ</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>HTML, CSS, JavaScript, SheetJS, Formspree, Git, GitHub, Render.com</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Test Report Generator</v>
+      </c>
+      <c r="B3" t="str">
+        <v>สคริปต์สร้างรายงานทดสอบ</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2024</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>A Python script that reads test execution results from an Excel workbook and automatically generates a formatted HTML report. Includes pass/fail summary, defect counts by severity, and a coverage breakdown by test area.</v>
+      </c>
+      <c r="F3" t="str">
+        <v>สคริปต์ Python ที่อ่านผลการทดสอบจาก Excel แล้วสร้างรายงาน HTML อัตโนมัติ รวมสรุป pass/fail จำนวน defect แยกตาม severity และสัดส่วน coverage ของแต่ละ area</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Python, openpyxl, pandas, Jinja2, HTML, CSS</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -719,9 +827,9 @@
         <v>Lotus's is a major retail chain in Thailand, formerly known as Tesco Lotus, operating a wide range of store formats including hypermarkets, supermarkets, and convenience stores. Lotus's Web (Lotus's Shop Online) is their official online shopping platform, allowing customers to order groceries and household goods through its website or mobile app.</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Manage products and inventory system to meet the requirements_x000d_
-• Manage test plan, design and execute test cases_x000d_
-• Transfer knowledge and provide documents to team_x000d_
+        <v xml:space="preserve">• Manage products and inventory system to meet the requirements_x000d__x000d_
+• Manage test plan, design and execute test cases_x000d__x000d_
+• Transfer knowledge and provide documents to team_x000d__x000d_
 • Collaborate supporting between teams and investigate issue and root cause.</v>
       </c>
       <c r="G2" t="str">
@@ -742,8 +850,11 @@
       <c r="L2" t="str">
         <v>Lotus's เป็นเชนค้าปลีกรายใหญ่ของไทย เดิมชื่อ Tesco Lotus มีร้านหลายรูปแบบ ทั้งไฮเปอร์มาร์เก็ต ซูเปอร์มาร์เก็ต และร้านสะดวกซื้อ ส่วน Lotus's Web (Lotus's Shop Online) คือแพลตฟอร์มช้อปออนไลน์อย่างเป็นทางการ ให้ลูกค้าสั่งของกินของใช้ผ่านเว็บไซต์หรือแอปได้สะดวกๆ</v>
       </c>
-      <c r="M2" t="str">
-        <v>• ดูแลระบบสินค้าและสต็อกให้ตรงตามที่ทีมต้องการ • วาง Test Plan ออกแบบและรัน Test Case • ถ่ายทอดความรู้และทำเอกสารให้ทีม • ประสานงานข้ามทีมและสืบหาต้นตอของปัญหา</v>
+      <c r="M2" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ดูแลระบบสินค้าและสต็อกให้ตรงตามที่ทีมต้องการ_x000d__x000d_
+• วาง Test Plan ออกแบบและรัน Test Case_x000d__x000d_
+• ถ่ายทอดความรู้และทำเอกสารให้ทีม_x000d__x000d_
+• ประสานงานข้ามทีมและสืบหาต้นตอของปัญหา</v>
       </c>
       <c r="N2" t="str">
         <v>Software</v>
@@ -766,9 +877,9 @@
         <v>Manao Meals is a web and mobile application that allows company members to order lunch meals as a company benefit. Admins can assign restaurant details and menus, and employees use the app to order food, adjust add-ons, and submit to admin for processing to the restaurant.</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Define test plan, approaches, template and strategy for test coverage_x000d__x000d__x000d_
-• Define automation test plan, template and contribute documentation_x000d__x000d__x000d_
-• Perform functional test and test case design_x000d__x000d__x000d_
+        <v xml:space="preserve">• Define test plan, approaches, template and strategy for test coverage_x000d__x000d__x000d__x000d_
+• Define automation test plan, template and contribute documentation_x000d__x000d__x000d__x000d_
+• Perform functional test and test case design_x000d__x000d__x000d__x000d_
 • Communicate between developer, QA and project owner.</v>
       </c>
       <c r="G3" t="str">
@@ -789,8 +900,11 @@
       <c r="L3" t="str">
         <v>Manao Meals เป็นเว็บและแอปสำหรับสั่งข้าวกลางวันในออฟฟิศเป็นสวัสดิการพนักงาน แอดมินตั้งร้านและเมนูได้ พนักงานก็เข้าแอปไปสั่ง เลือก add-on แล้วส่งให้แอดมินรวบรวมไปสั่งร้านต่อ</v>
       </c>
-      <c r="M3" t="str">
-        <v>• วางแผน Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม • วาง Automation Test Plan พร้อมเทมเพลตและช่วยทำเอกสาร • ทำ Functional Test และออกแบบ Test Case • ประสานงานระหว่าง Dev, QA และ Project Owner</v>
+      <c r="M3" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม_x000d__x000d_
+• วาง Automation Test Plan พร้อมเทมเพลตและช่วยทำเอกสาร_x000d__x000d_
+• ทำ Functional Test และออกแบบ Test Case_x000d__x000d_
+• ประสานงานระหว่าง Dev, QA และ Project Owner</v>
       </c>
       <c r="N3" t="str">
         <v>Software</v>
@@ -813,9 +927,9 @@
         <v>Seller Center is an E-commerce web application and inventory system that allows vendors (sellers) to join and manage their teams, orders, campaigns, and products. It separates into an admin site (managing other admins, sellers, and transactions) and a seller site (managing shop products and order transactions).</v>
       </c>
       <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Manage and contribute documentation_x000d__x000d__x000d_
-• Define test plan, approaches, template and strategy for test coverage_x000d__x000d__x000d_
-• Perform functional test and test case design_x000d__x000d__x000d_
+        <v xml:space="preserve">• Manage and contribute documentation_x000d__x000d__x000d__x000d_
+• Define test plan, approaches, template and strategy for test coverage_x000d__x000d__x000d__x000d_
+• Perform functional test and test case design_x000d__x000d__x000d__x000d_
 • Communicate between developer, QA and project owner.</v>
       </c>
       <c r="G4" t="str">
@@ -836,8 +950,11 @@
       <c r="L4" t="str">
         <v>Seller Center เป็นเว็บ E-commerce และระบบสต็อกที่ให้ผู้ขาย (Seller) เข้ามาจัดการทีม ออเดอร์ แคมเปญ และสินค้าได้ แบ่งเป็นฝั่ง Admin (จัดการแอดมินอื่น ผู้ขาย และธุรกรรม) กับฝั่ง Seller (จัดการสินค้าในร้านและออเดอร์)</v>
       </c>
-      <c r="M4" t="str">
-        <v>• ดูแลและช่วยจัดทำเอกสาร • วาง Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม • ทำ Functional Test และออกแบบ Test Case • ประสานงานระหว่าง Dev, QA และ Project Owner</v>
+      <c r="M4" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ดูแลและช่วยจัดทำเอกสาร_x000d__x000d_
+• วาง Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม_x000d__x000d_
+• ทำ Functional Test และออกแบบ Test Case_x000d__x000d_
+• ประสานงานระหว่าง Dev, QA และ Project Owner</v>
       </c>
       <c r="N4" t="str">
         <v>Software</v>
@@ -860,7 +977,7 @@
         <v>PTT Digital is a finance application for PTT, requiring Quality Assurance standards and DevSecOps processes to ensure secure and reliable transactions.</v>
       </c>
       <c r="F5" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Contribute documentation for Standard Quality Assurance, covering DevSecOps process with user acceptance criteria_x000d__x000d__x000d_
+        <v xml:space="preserve">• Contribute documentation for Standard Quality Assurance, covering DevSecOps process with user acceptance criteria_x000d__x000d__x000d__x000d_
 • Communicate between developer, QA and project owner.</v>
       </c>
       <c r="G5" t="str">
@@ -881,8 +998,9 @@
       <c r="L5" t="str">
         <v>PTT Digital เป็นแอปด้านการเงินของ ปตท. ที่ต้องการมาตรฐาน QA และกระบวนการ DevSecOps เพื่อให้ทุกธุรกรรมปลอดภัยและเชื่อถือได้</v>
       </c>
-      <c r="M5" t="str">
-        <v>• จัดทำเอกสารมาตรฐาน QA ครอบคลุมกระบวนการ DevSecOps พร้อมเงื่อนไขการรับมอบงานจากผู้ใช้ • ประสานงานระหว่าง Dev, QA และ Project Owner</v>
+      <c r="M5" t="str" xml:space="preserve">
+        <v xml:space="preserve">• จัดทำเอกสารมาตรฐาน QA ครอบคลุมกระบวนการ DevSecOps พร้อมเงื่อนไขการรับมอบงานจากผู้ใช้_x000d__x000d_
+• ประสานงานระหว่าง Dev, QA และ Project Owner</v>
       </c>
       <c r="N5" t="str">
         <v>Software</v>
@@ -905,9 +1023,9 @@
         <v>True Online Store is an E-commerce website by True Corporation, providing True products and services for customers and True membership.</v>
       </c>
       <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, analysis and design to cover business requirements_x000d__x000d__x000d_
-• Test case design and execution from day-to-day basis_x000d__x000d__x000d_
-• Generate test data and test script for manual and automation testing_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, analysis and design to cover business requirements_x000d__x000d__x000d__x000d_
+• Test case design and execution from day-to-day basis_x000d__x000d__x000d__x000d_
+• Generate test data and test script for manual and automation testing_x000d__x000d__x000d__x000d_
 • Perform static and dynamic testing to cover acceptances.</v>
       </c>
       <c r="G6" t="str">
@@ -928,8 +1046,11 @@
       <c r="L6" t="str">
         <v>True Online Store เป็นเว็บ E-commerce ของ True Corporation ขายสินค้าและบริการของทรู รวมถึงสิทธิประโยชน์สำหรับสมาชิก True</v>
       </c>
-      <c r="M6" t="str">
-        <v>• วางแผน วิเคราะห์ และออกแบบการทดสอบให้ครอบคลุม Business Requirement • ออกแบบและรัน Test Case ในงานประจำวัน • เตรียม Test Data และเขียน Test Script ทั้งแบบ Manual และ Automation • ทำทั้ง Static และ Dynamic Testing เพื่อให้ผ่านเกณฑ์รับมอบ</v>
+      <c r="M6" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน วิเคราะห์ และออกแบบการทดสอบให้ครอบคลุม Business Requirement_x000d__x000d_
+• ออกแบบและรัน Test Case ในงานประจำวัน_x000d__x000d_
+• เตรียม Test Data และเขียน Test Script ทั้งแบบ Manual และ Automation_x000d__x000d_
+• ทำทั้ง Static และ Dynamic Testing เพื่อให้ผ่านเกณฑ์รับมอบ</v>
       </c>
       <c r="N6" t="str">
         <v>Software</v>
@@ -952,8 +1073,8 @@
         <v>Linage W is a global scale MMORPG where players fight for their glories, set 150 years after the original Lineage story in the Aden World. Players can pick a story among lord, knight, fairy, and mage to explore a dark fantasy world.</v>
       </c>
       <c r="F7" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Define test scope, plan, data and documentation to cover test standard_x000d__x000d__x000d_
-• Maintenance testing, investigate and analyze issues_x000d__x000d__x000d_
+        <v xml:space="preserve">• Define test scope, plan, data and documentation to cover test standard_x000d__x000d__x000d__x000d_
+• Maintenance testing, investigate and analyze issues_x000d__x000d__x000d__x000d_
 • Playthrough testing as end-user on production environment.</v>
       </c>
       <c r="G7" t="str">
@@ -974,8 +1095,10 @@
       <c r="L7" t="str">
         <v>Lineage W เป็นเกม MMORPG ระดับโลก ซึ่งผู้เล่นต้องต่อสู้เพื่อชื่อเสียงของตัวเอง ดำเนินเรื่องหลังจาก Lineage ภาคแรก 150 ปี ในโลก Aden ผู้เล่นสามารถเลือกเล่นเป็นขุนนาง อัศวิน นางฟ้า หรือพ่อมด เพื่อผจญภัยในโลกแฟนตาซีลึกลับ</v>
       </c>
-      <c r="M7" t="str">
-        <v>• กำหนดขอบเขตการทดสอบ Test Plan ข้อมูล และเอกสารให้ตรงตามมาตรฐาน • ทำ Maintenance Testing ตรวจสอบและวิเคราะห์ปัญหา • เล่นจริงในมุมมองผู้ใช้งานบน Production</v>
+      <c r="M7" t="str" xml:space="preserve">
+        <v xml:space="preserve">• กำหนดขอบเขตการทดสอบ Test Plan ข้อมูล และเอกสารให้ตรงตามมาตรฐาน_x000d__x000d_
+• ทำ Maintenance Testing ตรวจสอบและวิเคราะห์ปัญหา_x000d__x000d_
+• เล่นจริงในมุมมองผู้ใช้งานบน Production</v>
       </c>
       <c r="N7" t="str">
         <v>Game</v>
@@ -998,9 +1121,9 @@
         <v>The project focused on the 'ALL member' 7-Eleven membership program via the 7App. This program allows users to get discounts, earn coupons, check, redeem, and transfer ALL points, and pay with credit cards via Truemoney Wallet at 7-Eleven stores, 7Delivery service, and All Online.</v>
       </c>
       <c r="F8" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Supervision and coordinate between teams, developers, internal and external QA_x000d__x000d__x000d_
-• Test analysis, planning and management_x000d__x000d__x000d_
-• Manage QA processes for new campaigns and features for each release_x000d__x000d__x000d_
+        <v xml:space="preserve">• Supervision and coordinate between teams, developers, internal and external QA_x000d__x000d__x000d__x000d_
+• Test analysis, planning and management_x000d__x000d__x000d__x000d_
+• Manage QA processes for new campaigns and features for each release_x000d__x000d__x000d__x000d_
 • Transfer testing tool knowledge to teams.</v>
       </c>
       <c r="G8" t="str">
@@ -1021,8 +1144,11 @@
       <c r="L8" t="str">
         <v>โปรเจกต์นี้เน้นที่ระบบสมาชิก 'ALL Member' ผ่านแอป 7App ผู้ใช้รับส่วนลด เก็บคูปอง เช็ค แลก และโอนคะแนน ALL Point รวมถึงจ่ายผ่านบัตรเครดิตผ่าน TrueMoney Wallet ที่ร้าน 7-Eleven, บริการ 7Delivery และ All Online</v>
       </c>
-      <c r="M8" t="str">
-        <v>• ดูแลและประสานงานระหว่างทีม Dev และทีม QA ทั้งภายในและภายนอก • วิเคราะห์ วางแผน และบริหารจัดการงานทดสอบ • ดูแลกระบวนการ QA สำหรับแคมเปญและฟีเจอร์ใหม่ในแต่ละ Release • ถ่ายทอดความรู้เรื่องเครื่องมือทดสอบให้ทีม</v>
+      <c r="M8" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ดูแลและประสานงานระหว่างทีม Dev และทีม QA ทั้งภายในและภายนอก_x000d__x000d_
+• วิเคราะห์ วางแผน และบริหารจัดการงานทดสอบ_x000d__x000d_
+• ดูแลกระบวนการ QA สำหรับแคมเปญและฟีเจอร์ใหม่ในแต่ละ Release_x000d__x000d_
+• ถ่ายทอดความรู้เรื่องเครื่องมือทดสอบให้ทีม</v>
       </c>
       <c r="N8" t="str">
         <v>Software</v>
@@ -1045,9 +1171,9 @@
         <v>Aliveunited is a digital platform that focuses on UI/UX design and system flow for end users, with consultation between project owner and design team.</v>
       </c>
       <c r="F9" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d_
-• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d_
-• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d__x000d_
+• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d__x000d_
 • Design, UI and UX consultant with Project Owner to analyze the whole system.</v>
       </c>
       <c r="G9" t="str">
@@ -1068,8 +1194,11 @@
       <c r="L9" t="str">
         <v>Aliveunited เป็นแพลตฟอร์มดิจิทัลที่เน้นการออกแบบ UI/UX และ System Flow สำหรับผู้ใช้ ผ่านการปรึกษาระหว่าง Project Owner กับทีมดีไซน์</v>
       </c>
-      <c r="M9" t="str">
-        <v>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager • ให้คำปรึกษาด้าน Design, UI และ UX ร่วมกับ Project Owner เพื่อวิเคราะห์ระบบทั้งหมด</v>
+      <c r="M9" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ_x000d__x000d_
+• ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester_x000d__x000d_
+• รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager_x000d__x000d_
+• ให้คำปรึกษาด้าน Design, UI และ UX ร่วมกับ Project Owner เพื่อวิเคราะห์ระบบทั้งหมด</v>
       </c>
       <c r="N9" t="str">
         <v>etc.</v>
@@ -1092,8 +1221,8 @@
         <v>The Curaprox App (iOS, Android) is designed to help users stay motivated in their daily dental routines, ensuring preventive dental care year-round. It allows connection with dental professionals and access to lectures, articles, and products.</v>
       </c>
       <c r="F10" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d_
-• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d__x000d_
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers.</v>
       </c>
       <c r="G10" t="str">
@@ -1114,8 +1243,10 @@
       <c r="L10" t="str">
         <v>แอป Curaprox (iOS, Android) ช่วยสร้างแรงจูงใจในการดูแลสุขภาพฟันประจำวัน เพื่อการดูแลฟันเชิงป้องกันตลอดปี สามารถเชื่อมต่อกับทันตแพทย์ อ่านบทความ และเข้าถึงผลิตภัณฑ์ได้ผ่านแอป</v>
       </c>
-      <c r="M10" t="str">
-        <v>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager</v>
+      <c r="M10" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ_x000d__x000d_
+• ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester_x000d__x000d_
+• รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager</v>
       </c>
       <c r="N10" t="str">
         <v>Software</v>
@@ -1138,8 +1269,8 @@
         <v>The Curaprox Pro App (iOS Android) aims to help dental professionals motivate patients and communicate and support them throughout the year emphasizing daily dental care over quick fixes.</v>
       </c>
       <c r="F11" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d_
-• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d__x000d_
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers.</v>
       </c>
       <c r="G11" t="str">
@@ -1160,8 +1291,10 @@
       <c r="L11" t="str">
         <v>แอป Curaprox Pro (iOS, Android) ออกแบบมาเพื่อช่วยทันตแพทย์สร้างแรงบันดาลใจและสื่อสารกับคนไข้ตลอดปี เน้นการดูแลฟันในชีวิตประจำวันมากกว่าการแก้ปัญหาเฉพาะหน้า</v>
       </c>
-      <c r="M11" t="str">
-        <v>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager</v>
+      <c r="M11" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ_x000d__x000d_
+• ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester_x000d__x000d_
+• รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager</v>
       </c>
       <c r="N11" t="str">
         <v>Software</v>
@@ -1184,10 +1317,10 @@
         <v>Hotel Life: A Resort Simulator is a simulation game where players build and manage their own resort, designing rooms, attractions, and services to attract guests.</v>
       </c>
       <c r="F12" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d_
-• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d_
-• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d_
-• Coordinated developer team to request test tools for game level testing and improve QA processes_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d__x000d_
+• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d__x000d_
+• Coordinated developer team to request test tools for game level testing and improve QA processes_x000d__x000d__x000d__x000d_
 • Research PC and console guidelines and pass information to the team to understand more about specific requirements and limitations for submission.</v>
       </c>
       <c r="G12" t="str">
@@ -1208,8 +1341,12 @@
       <c r="L12" t="str">
         <v>Hotel Life: A Resort Simulator เป็นเกมแนวสร้างและบริหารรีสอร์ตของตัวเอง ผู้เล่นออกแบบห้องพัก สิ่งอำนวยความสะดวก และสถานที่ท่องเที่ยวต่างๆ เพื่อดึงดูดลูกค้า</v>
       </c>
-      <c r="M12" t="str">
-        <v>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager • ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA • ศึกษา Guideline ของ PC และ Console แล้วส่งต่อให้ทีม เพื่อรองรับรีควอเรมนต์และข้อจำกัดของแต่ละแพลตฟอร์มสำหรับ Submission</v>
+      <c r="M12" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ_x000d__x000d_
+• ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester_x000d__x000d_
+• รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager_x000d__x000d_
+• ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA_x000d__x000d_
+• ศึกษา Guideline ของ PC และ Console แล้วส่งต่อให้ทีม เพื่อรองรับรีควอเรมนต์และข้อจำกัดของแต่ละแพลตฟอร์มสำหรับ Submission</v>
       </c>
       <c r="N12" t="str">
         <v>Game</v>
@@ -1229,14 +1366,14 @@
         <v/>
       </c>
       <c r="E13" t="str" xml:space="preserve">
-        <v xml:space="preserve">Lumen. is a puzzle game on Apple Arcade where players solve levels using lights lenses and mirrors_x000d__x000d__x000d__x000d_
+        <v xml:space="preserve">Lumen. is a puzzle game on Apple Arcade where players solve levels using lights lenses and mirrors_x000d__x000d__x000d__x000d__x000d_
   discovering a mysterious antique box.</v>
       </c>
       <c r="F13" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d_
-• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d_
-• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d_
-• Coordinated developer team to request test tools for game level testing and improve QA processes_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, monitoring, analysis and design_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d__x000d_
+• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d__x000d_
+• Coordinated developer team to request test tools for game level testing and improve QA processes_x000d__x000d__x000d__x000d_
 • Research PC and console guidelines and pass information to the team to understand more about specific requirements and limitations for submission.</v>
       </c>
       <c r="G13" t="str">
@@ -1257,8 +1394,12 @@
       <c r="L13" t="str">
         <v>Lumen. เป็นเกมปริศนาบน Apple Arcade ผู้เล่นไขปริศนาแต่ละด่านด้วยแสง เลนส์ และกระจก พร้อมไขปริศนาของกล่องโบราณลึกลับ</v>
       </c>
-      <c r="M13" t="str">
-        <v>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager • ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA • ศึกษา Guideline ของ PC และ Console แล้วส่งต่อให้ทีม เพื่อรองรับรีควอเรมนต์และข้อจำกัดของแต่ละแพลตฟอร์มสำหรับ Submission</v>
+      <c r="M13" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ_x000d__x000d_
+• ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester_x000d__x000d_
+• รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager_x000d__x000d_
+• ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA_x000d__x000d_
+• ศึกษา Guideline ของ PC และ Console แล้วส่งต่อให้ทีม เพื่อรองรับรีควอเรมนต์และข้อจำกัดของแต่ละแพลตฟอร์มสำหรับ Submission</v>
       </c>
       <c r="N13" t="str">
         <v>Game</v>
@@ -1281,7 +1422,7 @@
         <v>Pick is a mobile application that connects with hardware devices, allowing users to synchronize and control device functions through the app.</v>
       </c>
       <c r="F14" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Coordinated with the external production and passed testing criteria to external tester teams_x000d__x000d__x000d_
+        <v xml:space="preserve">• Coordinated with the external production and passed testing criteria to external tester teams_x000d__x000d__x000d__x000d_
 • Functional, and API testing between software and hardware remotely to ensure app can synchronize as client acceptance.</v>
       </c>
       <c r="G14" t="str">
@@ -1302,8 +1443,9 @@
       <c r="L14" t="str">
         <v>Pick เป็นแอปมือถือที่เชื่อมต่อกับ Hardware ผู้ใช้สามารถซิงโครไนซ์และควบคุมการทำงานของอุปกรณ์ผ่านแอปได้</v>
       </c>
-      <c r="M14" t="str">
-        <v>• ประสานงานกับผู้ผลิตภายนอก และส่งต่อ Test Criteria ให้ทีม Tester ภายนอก • ทำ Functional Test และ API Test ระหว่าง Software กับ Hardware แบบ Remote เพื่อยืนยันว่าแอปซิงโครไนซ์ได้ตามที่ลูกค้าต้องการ</v>
+      <c r="M14" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ประสานงานกับผู้ผลิตภายนอก และส่งต่อ Test Criteria ให้ทีม Tester ภายนอก_x000d__x000d_
+• ทำ Functional Test และ API Test ระหว่าง Software กับ Hardware แบบ Remote เพื่อยืนยันว่าแอปซิงโครไนซ์ได้ตามที่ลูกค้าต้องการ</v>
       </c>
       <c r="N14" t="str">
         <v>Software</v>
@@ -1326,10 +1468,10 @@
         <v>City of Games is an app allowing free play of classic and no-commission baccarat modes, featuring 3D card squeezing, available on iOS, Android, and Chinese Android.</v>
       </c>
       <c r="F15" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Release control, submit application to Apple and Google stores_x000d__x000d__x000d_
-• Test planning, monitoring, analysis and design_x000d__x000d__x000d_
-• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d_
-• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d_
+        <v xml:space="preserve">• Release control, submit application to Apple and Google stores_x000d__x000d__x000d__x000d_
+• Test planning, monitoring, analysis and design_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing, collected requirements and passed on information to the tester team_x000d__x000d__x000d__x000d_
+• Document review, managed test scenarios and coordinated with the developer team, tester team and managers_x000d__x000d__x000d__x000d_
 • Coordinated developer team to request test tools for game level testing and improve QA processes.</v>
       </c>
       <c r="G15" t="str">
@@ -1350,8 +1492,12 @@
       <c r="L15" t="str">
         <v>City of Games เป็นแอปที่ให้เล่นบาคาร่าแบบคลาสสิกและไร้ค่าคอมมิชชั่น ฟรี มีระบบเปิดไพ่สามมิติ รองรับทั้ง iOS, Android และ Android ของจีน</v>
       </c>
-      <c r="M15" t="str">
-        <v>• ดูแล Release Control และ Submit แอปขึ้น Apple และ Google Store • วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager • ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA</v>
+      <c r="M15" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ดูแล Release Control และ Submit แอปขึ้น Apple และ Google Store_x000d__x000d_
+• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ_x000d__x000d_
+• ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester_x000d__x000d_
+• รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager_x000d__x000d_
+• ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA</v>
       </c>
       <c r="N15" t="str">
         <v>Game</v>
@@ -1374,9 +1520,9 @@
         <v>Tint. is a mobile and console game available on iOS, MacOS, and TvOS, designed to work with and without peripheral game controllers.</v>
       </c>
       <c r="F16" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Coordinated with the external production and passed testing criteria and other game information to external tester teams_x000d__x000d__x000d_
-• Functional testing of new features and playthrough testing to ensure the game can progress correctly as expected with new integrated contents_x000d__x000d__x000d_
-• Monitoring external teams closely from the regression process to cover client and store acceptance_x000d__x000d__x000d_
+        <v xml:space="preserve">• Coordinated with the external production and passed testing criteria and other game information to external tester teams_x000d__x000d__x000d__x000d_
+• Functional testing of new features and playthrough testing to ensure the game can progress correctly as expected with new integrated contents_x000d__x000d__x000d__x000d_
+• Monitoring external teams closely from the regression process to cover client and store acceptance_x000d__x000d__x000d__x000d_
 • Device coverage testing, to ensure app can work correctly on MacOS, TvOS and iOS devices with and without peripheral game controllers.</v>
       </c>
       <c r="G16" t="str">
@@ -1397,8 +1543,11 @@
       <c r="L16" t="str">
         <v>Tint. เป็นเกมบนมือถือและคอนโซล รองรับทั้ง iOS, MacOS และ tvOS ออกแบบมาให้เล่นได้ทั้งแบบใช้และไม่ใช้ Game Controller เสริม</v>
       </c>
-      <c r="M16" t="str">
-        <v>• ประสานงานกับผู้ผลิตภายนอก ส่งต่อ Test Criteria และข้อมูลเกมให้ทีม Tester ภายนอก • Functional Test ฟีเจอร์ใหม่ และ Playthrough เพื่อให้มั่นใจว่าเกมเล่นได้ต่อเนื่องตามที่คาดหวังหลังรวม Content ใหม่ • ติดตามทีมภายนอกอย่างใกล้ชิดตอนทำ Regression เพื่อรองรับรีควอเรมนต์ของลูกค้าและ Store • ทดสอบการรองรับอุปกรณ์ให้แอปทำงานได้บน MacOS, tvOS และ iOS ทั้งแบบใช้และไม่ใช้ Game Controller</v>
+      <c r="M16" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ประสานงานกับผู้ผลิตภายนอก ส่งต่อ Test Criteria และข้อมูลเกมให้ทีม Tester ภายนอก_x000d__x000d_
+• Functional Test ฟีเจอร์ใหม่ และ Playthrough เพื่อให้มั่นใจว่าเกมเล่นได้ต่อเนื่องตามที่คาดหวังหลังรวม Content ใหม่_x000d__x000d_
+• ติดตามทีมภายนอกอย่างใกล้ชิดตอนทำ Regression เพื่อรองรับรีควอเรมนต์ของลูกค้าและ Store_x000d__x000d_
+• ทดสอบการรองรับอุปกรณ์ให้แอปทำงานได้บน MacOS, tvOS และ iOS ทั้งแบบใช้และไม่ใช้ Game Controller</v>
       </c>
       <c r="N16" t="str">
         <v>Game</v>
@@ -1421,9 +1570,9 @@
         <v>Panya is a mobile application designed to work reliably across various network conditions, with a focus on stability and performance for end users.</v>
       </c>
       <c r="F17" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Test planning, gathered new requirements from clients directly and passed on information to the tester team_x000d__x000d__x000d_
-• Test suite control, created, updated, prioritized and defined test cases from test suite for regression testing to reach client acceptance_x000d__x000d__x000d_
-• Handled responsibility for test tools, implemented processes for automation to prepare test data, and created technical documents for internal purposes_x000d__x000d__x000d_
+        <v xml:space="preserve">• Test planning, gathered new requirements from clients directly and passed on information to the tester team_x000d__x000d__x000d__x000d_
+• Test suite control, created, updated, prioritized and defined test cases from test suite for regression testing to reach client acceptance_x000d__x000d__x000d__x000d_
+• Handled responsibility for test tools, implemented processes for automation to prepare test data, and created technical documents for internal purposes_x000d__x000d__x000d__x000d_
 • Investigated network link conditions to perform stability testing, making sure the app works to various network status.</v>
       </c>
       <c r="G17" t="str">
@@ -1444,8 +1593,11 @@
       <c r="L17" t="str">
         <v>Panya เป็นแอปมือถือที่ออกแบบมาให้ทำงานได้อย่างเสถียรบนสภาพเครือข่ายที่หลากหลาย มุ่งเน้นความเสถียรและประสิทธิภาพสำหรับผู้ใช้</v>
       </c>
-      <c r="M17" t="str">
-        <v>• วางแผนการทดสอบ รับ Requirement จากลูกค้าโดยตรงและส่งต่อให้ทีม Tester • จัดการ Test Suite — สร้าง อัปเดต จัดลำดับความสำคัญ และกำหนด Test Case สำหรับ Regression ให้ตรงตามที่ลูกค้ายอมรับ • ดูแล Test Tools วางแนวทาง Automation สำหรับจัดเตรียม Test Data พร้อมทำเอกสารทางเทคนิคภายใน • ตรวจสภาพเครือข่ายเพื่อทำ Stability Testing ให้มั่นใจว่าแอปทำงานได้ในทุกสภาพเน็ตเวิร์ก</v>
+      <c r="M17" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผนการทดสอบ รับ Requirement จากลูกค้าโดยตรงและส่งต่อให้ทีม Tester_x000d__x000d_
+• จัดการ Test Suite — สร้าง อัปเดต จัดลำดับความสำคัญ และกำหนด Test Case สำหรับ Regression ให้ตรงตามที่ลูกค้ายอมรับ_x000d__x000d_
+• ดูแล Test Tools วางแนวทาง Automation สำหรับจัดเตรียม Test Data พร้อมทำเอกสารทางเทคนิคภายใน_x000d__x000d_
+• ตรวจสภาพเครือข่ายเพื่อทำ Stability Testing ให้มั่นใจว่าแอปทำงานได้ในทุกสภาพเน็ตเวิร์ก</v>
       </c>
       <c r="N17" t="str">
         <v>Software</v>
@@ -1512,10 +1664,10 @@
         <v>ImaginMe Beauty and the Beast is a personalized interactive storybook app where users customize their character to star in the Beauty and the Beast story, featuring mini-games and animated scenes.</v>
       </c>
       <c r="F19" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance_x000d__x000d__x000d_
-• Art Asset management, designed specification, limitation and performed optimization for device coverage_x000d__x000d__x000d_
-• Level designing with Unity to generate mini games and performed own unit, integration and system testing to meet requirements_x000d__x000d__x000d_
-• Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing_x000d__x000d__x000d_
+        <v xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance_x000d__x000d__x000d__x000d_
+• Art Asset management, designed specification, limitation and performed optimization for device coverage_x000d__x000d__x000d__x000d_
+• Level designing with Unity to generate mini games and performed own unit, integration and system testing to meet requirements_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing_x000d__x000d__x000d__x000d_
 • Game version controlling and submitting game builds via Google Play Console and iTunes Connect.</v>
       </c>
       <c r="G19" t="str">
@@ -1536,8 +1688,12 @@
       <c r="L19" t="str">
         <v>เป็นแอปหนังสือนิทานส่วนตัวที่ผู้ใช้ปรับแต่งตัวละครได้เอง ร่วมผจญภัยในเรื่องโฉมงามกับเจ้าชายอสูร พร้อมมินิเกมและฉากแอนิเมชัน</v>
       </c>
-      <c r="M19" t="str">
-        <v>• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า • จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย • ทำ Level Design ด้วย Unity สร้าง Mini Game พร้อม Unit, Integration และ System Test ของตัวเองให้ตรงตาม Requirement • ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop • คุม Game Version และ Submit Build ผ่าน Google Play Console และ iTunes Connect</v>
+      <c r="M19" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า_x000d__x000d_
+• จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย_x000d__x000d_
+• ทำ Level Design ด้วย Unity สร้าง Mini Game พร้อม Unit, Integration และ System Test ของตัวเองให้ตรงตาม Requirement_x000d__x000d_
+• ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop_x000d__x000d_
+• คุม Game Version และ Submit Build ผ่าน Google Play Console และ iTunes Connect</v>
       </c>
       <c r="N19" t="str">
         <v>Game</v>
@@ -1560,10 +1716,10 @@
         <v>ImaginMe Dragons is a personalized interactive storybook app where users customize their character to star in a dragon-themed adventure, featuring mini-games with patterns and obstacles.</v>
       </c>
       <c r="F20" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance_x000d__x000d__x000d_
-• Art Asset management, designed specification, limitation and performed optimization for device coverage_x000d__x000d__x000d_
-• Level designing with Unity to generate pattern and obstacles and performed own unit, integration and system testing to meet requirements_x000d__x000d__x000d_
-• Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing_x000d__x000d__x000d_
+        <v xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance_x000d__x000d__x000d__x000d_
+• Art Asset management, designed specification, limitation and performed optimization for device coverage_x000d__x000d__x000d__x000d_
+• Level designing with Unity to generate pattern and obstacles and performed own unit, integration and system testing to meet requirements_x000d__x000d__x000d__x000d_
+• Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing_x000d__x000d__x000d__x000d_
 • Game version controlling and submitting game builds via Google Play Console and iTunes Connect.</v>
       </c>
       <c r="G20" t="str">
@@ -1584,8 +1740,12 @@
       <c r="L20" t="str">
         <v>หนังสือนิทานส่วนตัวธีมมังกร ที่ผู้ใช้ปรับแต่งตัวละครได้เอง ร่วมผจญภัยผ่านมินิเกมที่มีรูปแบบและอุปสรรคหลากหลาย</v>
       </c>
-      <c r="M20" t="str">
-        <v>• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า • จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย • ทำ Level Design ด้วย Unity สร้างรูปแบบและอุปสรรค พร้อม Unit, Integration และ System Test • ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop • คุม Game Version และ Submit Build ผ่าน Google Play Console และ iTunes Connect</v>
+      <c r="M20" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า_x000d__x000d_
+• จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย_x000d__x000d_
+• ทำ Level Design ด้วย Unity สร้างรูปแบบและอุปสรรค พร้อม Unit, Integration และ System Test_x000d__x000d_
+• ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop_x000d__x000d_
+• คุม Game Version และ Submit Build ผ่าน Google Play Console และ iTunes Connect</v>
       </c>
       <c r="N20" t="str">
         <v>Game</v>
@@ -1696,9 +1856,9 @@
         <v>Tesco Lotus Shopping Spree is a promotional infinite running game for Tesco Lotus, designed for low-end mobile devices, where players run through stages to collect items and rewards.</v>
       </c>
       <c r="F23" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Built on client concepts to design promotional infinite running games to meet client acceptance_x000d__x000d__x000d_
-• Designed specification, limitation and optimization to cover low end devices_x000d__x000d__x000d_
-• Level designing with Unity to generate stage patterns and perform own unit, integration and system testing_x000d__x000d__x000d_
+        <v xml:space="preserve">• Built on client concepts to design promotional infinite running games to meet client acceptance_x000d__x000d__x000d__x000d_
+• Designed specification, limitation and optimization to cover low end devices_x000d__x000d__x000d__x000d_
+• Level designing with Unity to generate stage patterns and perform own unit, integration and system testing_x000d__x000d__x000d__x000d_
 • Handling responsibility for test tools and developing improvement processes.</v>
       </c>
       <c r="G23" t="str">
@@ -1719,8 +1879,11 @@
       <c r="L23" t="str">
         <v>เกมประชาสัมพันธ์แนว Infinite Running ของเทสโก้โลตัส ทำงานได้บนมือถือสเป็กต่ำ ผู้เล่นวิ่งผ่านด่านต่างๆ เพื่อเก็บไอเท็มและรางวัล</v>
       </c>
-      <c r="M23" t="str">
-        <v>• ออกแบบเกม Promotional Infinite Running ตามคอนเซ็ปต์ของลูกค้า • ออกแบบ Spec ข้อจำกัด และ Optimize ให้รองรับมือถือ Spec ต่ำ • ทำ Level Design ด้วย Unity สร้าง Stage Pattern พร้อม Unit, Integration และ System Test • ดูแล Test Tools และพัฒนาปรับปรุงกระบวนการ</v>
+      <c r="M23" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบเกม Promotional Infinite Running ตามคอนเซ็ปต์ของลูกค้า_x000d__x000d_
+• ออกแบบ Spec ข้อจำกัด และ Optimize ให้รองรับมือถือ Spec ต่ำ_x000d__x000d_
+• ทำ Level Design ด้วย Unity สร้าง Stage Pattern พร้อม Unit, Integration และ System Test_x000d__x000d_
+• ดูแล Test Tools และพัฒนาปรับปรุงกระบวนการ</v>
       </c>
       <c r="N23" t="str">
         <v>Game</v>
@@ -1743,9 +1906,9 @@
         <v>Totem Defender is a free-to-play tower defense game for mobile, where players use totems to defend against waves of enemies across multiple stages and difficulty levels.</v>
       </c>
       <c r="F24" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Project planning, built on client concepts to design games contents from scratch to be the final product to meet client acceptance_x000d__x000d__x000d_
-• Researched and designed monetization for F2P games, targeted to both free and paid mobile users_x000d__x000d__x000d_
-• Level designing with Unity to generate stage patterns, level progress, difficulty level and perform own unit, integration and system testing to cover low end devices_x000d__x000d__x000d_
+        <v xml:space="preserve">• Project planning, built on client concepts to design games contents from scratch to be the final product to meet client acceptance_x000d__x000d__x000d__x000d_
+• Researched and designed monetization for F2P games, targeted to both free and paid mobile users_x000d__x000d__x000d__x000d_
+• Level designing with Unity to generate stage patterns, level progress, difficulty level and perform own unit, integration and system testing to cover low end devices_x000d__x000d__x000d__x000d_
 • Coordinated with the production team closely and managed sprint goal planning.</v>
       </c>
       <c r="G24" t="str">
@@ -1766,8 +1929,11 @@
       <c r="L24" t="str">
         <v>Totem Defender เป็นเกม Tower Defense แบบ Free-to-Play บนมือถือ ผู้เล่นใช้โทเท็มป้องกันศัตรูที่บุกเข้ามาเป็นระลอกไปในหลายด่านและหลายระดับความยาก</v>
       </c>
-      <c r="M24" t="str">
-        <v>• วางแผนโปรเจกต์ ออกแบบเนื้อหาเกมตั้งแต่ต้นจนถึง Final Product ตามคอนเซ็ปต์ลูกค้า • วิจัยและออกแบบระบบ Monetization สำหรับเกม F2P รองรับทั้งผู้เล่นฟรีและจ่ายเงิน • ทำ Level Design ด้วย Unity สร้าง Stage Pattern, Level Progress และ Difficulty พร้อมทดสอบให้รองรับมือถือ Spec ต่ำ • ประสานงานกับทีม Production อย่างใกล้ชิด และจัดการ Sprint Goal Planning</v>
+      <c r="M24" t="str" xml:space="preserve">
+        <v xml:space="preserve">• วางแผนโปรเจกต์ ออกแบบเนื้อหาเกมตั้งแต่ต้นจนถึง Final Product ตามคอนเซ็ปต์ลูกค้า_x000d__x000d_
+• วิจัยและออกแบบระบบ Monetization สำหรับเกม F2P รองรับทั้งผู้เล่นฟรีและจ่ายเงิน_x000d__x000d_
+• ทำ Level Design ด้วย Unity สร้าง Stage Pattern, Level Progress และ Difficulty พร้อมทดสอบให้รองรับมือถือ Spec ต่ำ_x000d__x000d_
+• ประสานงานกับทีม Production อย่างใกล้ชิด และจัดการ Sprint Goal Planning</v>
       </c>
       <c r="N24" t="str">
         <v>Game</v>
@@ -1790,8 +1956,8 @@
         <v>Mes Comptines for 3DS is a children's music game on Nintendo 3DS that combines karaoke and rhythm tap gameplay, helping kids sing along to French nursery rhymes.</v>
       </c>
       <c r="F25" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Built on client concepts to design additional game play from karaoke to rhythm tap game to meet client acceptance_x000d__x000d__x000d_
-• Level designing, improved learning curve to cover more target players and replayability with various difficulty levels_x000d__x000d__x000d_
+        <v xml:space="preserve">• Built on client concepts to design additional game play from karaoke to rhythm tap game to meet client acceptance_x000d__x000d__x000d__x000d_
+• Level designing, improved learning curve to cover more target players and replayability with various difficulty levels_x000d__x000d__x000d__x000d_
 • Game version controlling and submitting game builds via Nintendo with LotCheck guidelines.</v>
       </c>
       <c r="G25" t="str">
@@ -1812,8 +1978,10 @@
       <c r="L25" t="str">
         <v>Mes Comptines for 3DS เป็นเกมดนตรีสำหรับเด็กบน Nintendo 3DS ผสมผสานระหว่างคาราโอเกะกับเกมจังหวะตามจังหวะ ช่วยให้เด็กร้องตามเพลงกล่อมเด็กภาษาฝรั่งเศส</v>
       </c>
-      <c r="M25" t="str">
-        <v>• ออกแบบ Gameplay เพิ่มเติมจากคาราโอเกะไปสู่เกมจังหวะตามจังหวะ ตามคอนเซ็ปต์ของลูกค้า • ปรับปรุง Learning Curve ให้ครอบคลุมผู้เล่นหลายกลุ่ม และเพิ่ม Replayability ด้วยระดับความยากหลายระดับ • คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</v>
+      <c r="M25" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบ Gameplay เพิ่มเติมจากคาราโอเกะไปสู่เกมจังหวะตามจังหวะ ตามคอนเซ็ปต์ของลูกค้า_x000d__x000d_
+• ปรับปรุง Learning Curve ให้ครอบคลุมผู้เล่นหลายกลุ่ม และเพิ่ม Replayability ด้วยระดับความยากหลายระดับ_x000d__x000d_
+• คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</v>
       </c>
       <c r="N25" t="str">
         <v>Game</v>
@@ -1924,7 +2092,7 @@
         <v>Lolirock is a music and karaoke game based on the Lolirock animated series, featuring character and stage customization with mini-games synced to the show's vocal lines.</v>
       </c>
       <c r="F28" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Level designing, design karaoke pitch level and synced to vocal line_x000d__x000d__x000d_
+        <v xml:space="preserve">• Level designing, design karaoke pitch level and synced to vocal line_x000d__x000d__x000d__x000d_
 • Functional and regression testing to mini game, character and stage customization.</v>
       </c>
       <c r="G28" t="str">
@@ -1945,8 +2113,9 @@
       <c r="L28" t="str">
         <v>เกมดนตรีและคาราโอเกะที่อิงจากการ์ตูน Lolirock มี Mini Game ซิงกับเสียงร้อง พร้อมออกแบบตัวละครและเวที</v>
       </c>
-      <c r="M28" t="str">
-        <v>• ออกแบบ Karaoke Pitch Level ให้ซิงค์กับ Vocal • ทำ Functional และ Regression Test ให้กับ Mini Game รวมถึงระบบตัวละครและเวที</v>
+      <c r="M28" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบ Karaoke Pitch Level ให้ซิงค์กับ Vocal_x000d__x000d_
+• ทำ Functional และ Regression Test ให้กับ Mini Game รวมถึงระบบตัวละครและเวที</v>
       </c>
       <c r="N28" t="str">
         <v>Game</v>
@@ -1969,8 +2138,8 @@
         <v>Meine ersten Mitsing-Lieder for WiiU is a children's karaoke game on Nintendo WiiU (remastered from the Wii version), featuring German nursery rhymes with peripheral device support.</v>
       </c>
       <c r="F29" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Remastering from Wii to WiiU version, functional and regression testing with peripheral devices_x000d__x000d__x000d_
-• Customer supporting and services_x000d__x000d__x000d_
+        <v xml:space="preserve">• Remastering from Wii to WiiU version, functional and regression testing with peripheral devices_x000d__x000d__x000d__x000d_
+• Customer supporting and services_x000d__x000d__x000d__x000d_
 • Game version controlling and submitting game builds via Nintendo with LotCheck guidelines.</v>
       </c>
       <c r="G29" t="str">
@@ -1991,8 +2160,10 @@
       <c r="L29" t="str">
         <v>เกมคาราโอเกะสำหรับเด็กบน Nintendo Wii U (ปรับจากเวอร์ชัน Wii) ร้องเพลงกล่อมเด็กภาษาเยอรมัน พร้อมรองรับอุปกรณ์เสริม</v>
       </c>
-      <c r="M29" t="str">
-        <v>• ปรับ Wii ไปเป็นเวอร์ชัน Wii U พร้อมทำ Functional และ Regression Test ร่วมกับอุปกรณ์เสริม • สนับสนุนลูกค้า • คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</v>
+      <c r="M29" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ปรับ Wii ไปเป็นเวอร์ชัน Wii U พร้อมทำ Functional และ Regression Test ร่วมกับอุปกรณ์เสริม_x000d__x000d_
+• สนับสนุนลูกค้า_x000d__x000d_
+• คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</v>
       </c>
       <c r="N29" t="str">
         <v>Game</v>
@@ -2103,11 +2274,11 @@
         <v>AeternoBlade for 3DS is a 2D side-scrolling action game on Nintendo 3DS where players control Freyja, who uses a magical blade to manipulate time and battle enemies across multiple stages.</v>
       </c>
       <c r="F32" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Handling responsibility for test tools and QA improvement processes_x000d__x000d__x000d_
-• Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly_x000d__x000d__x000d_
-• Handling responsibility for test tools and developing improvement processes for testing and generating game cutscenes_x000d__x000d__x000d_
-• Level designing and difficulty control, fine tuning effects and particles_x000d__x000d__x000d_
-• Game version controlling and submitting game builds and DLC to Nintendo US, EU and JP regions_x000d__x000d__x000d_
+        <v xml:space="preserve">• Handling responsibility for test tools and QA improvement processes_x000d__x000d__x000d__x000d_
+• Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly_x000d__x000d__x000d__x000d_
+• Handling responsibility for test tools and developing improvement processes for testing and generating game cutscenes_x000d__x000d__x000d__x000d_
+• Level designing and difficulty control, fine tuning effects and particles_x000d__x000d__x000d__x000d_
+• Game version controlling and submitting game builds and DLC to Nintendo US, EU and JP regions_x000d__x000d__x000d__x000d_
 • Created video trailer for promotional purposes.</v>
       </c>
       <c r="G32" t="str">
@@ -2128,8 +2299,13 @@
       <c r="L32" t="str">
         <v>AeternoBlade for 3DS เป็นเกมแอ็กชั่นแบบ 2D Side-Scrolling บน Nintendo 3DS ผู้เล่นบังคับ Freyja ที่ใช้ดาบเวทมนต์บิดผันเวลาบุกออกต่อสู้ศัตรูผ่านหลายด่าน</v>
       </c>
-      <c r="M32" t="str">
-        <v>• ดูแล Test Tools และปรับปรุงกระบวนการ QA • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตามที่ออกแบบไว้ • พัฒนา Test Tools สำหรับทดสอบและสร้าง Cutscene ของเกม • ทำ Level Design และ Difficulty Control รวมถึง Fine-Tune Effect และ Particle • คุม Game Version และ Submit Build พร้อม DLC ไป Nintendo ทั้ง US, EU และ JP • ตัดต่อ Trailer สำหรับงานโปรโมต</v>
+      <c r="M32" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ดูแล Test Tools และปรับปรุงกระบวนการ QA_x000d__x000d_
+• ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตามที่ออกแบบไว้_x000d__x000d_
+• พัฒนา Test Tools สำหรับทดสอบและสร้าง Cutscene ของเกม_x000d__x000d_
+• ทำ Level Design และ Difficulty Control รวมถึง Fine-Tune Effect และ Particle_x000d__x000d_
+• คุม Game Version และ Submit Build พร้อม DLC ไป Nintendo ทั้ง US, EU และ JP_x000d__x000d_
+• ตัดต่อ Trailer สำหรับงานโปรโมต</v>
       </c>
       <c r="N32" t="str">
         <v>Game</v>
@@ -2152,7 +2328,7 @@
         <v>Deadly Premonition: The Director's Cut for Steam is a survival horror mystery game on Steam (built from the PS3 version), where players investigate a series of murders in a small American town.</v>
       </c>
       <c r="F33" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Built on PS3 and Steam versions, designed additional contents, character control and customization to match with client, Steam submission requirements_x000d__x000d__x000d_
+        <v xml:space="preserve">• Built on PS3 and Steam versions, designed additional contents, character control and customization to match with client, Steam submission requirements_x000d__x000d__x000d__x000d_
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly as requirements.</v>
       </c>
       <c r="G33" t="str">
@@ -2173,8 +2349,9 @@
       <c r="L33" t="str">
         <v>เกม Survival Horror แนวสืบสวนบน Steam (พอร์ตมาจากเวอร์ชัน PS3) ผู้เล่นสืบสวนคดีฝาต่อเนื่องในเมืองเล็กของอเมริกา</v>
       </c>
-      <c r="M33" t="str">
-        <v>• พอร์ตจากเวอร์ชัน PS3 ไป Steam ออกแบบ Content เพิ่ม ระบบ Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Steam Submission • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตาม Requirement</v>
+      <c r="M33" t="str" xml:space="preserve">
+        <v xml:space="preserve">• พอร์ตจากเวอร์ชัน PS3 ไป Steam ออกแบบ Content เพิ่ม ระบบ Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Steam Submission_x000d__x000d_
+• ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตาม Requirement</v>
       </c>
       <c r="N33" t="str">
         <v>Game</v>
@@ -2197,7 +2374,7 @@
         <v>Deadly Premonition: Director's Cut for PS3 is a survival horror mystery game on PlayStation 3 (remastered from Xbox 360), with added content, character controls, and customization.</v>
       </c>
       <c r="F34" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Remastering from XBOX360 to PS3 version, designed additional contents, character control and customization to match with client, Sony submission requirements_x000d__x000d__x000d_
+        <v xml:space="preserve">• Remastering from XBOX360 to PS3 version, designed additional contents, character control and customization to match with client, Sony submission requirements_x000d__x000d__x000d__x000d_
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly as requirements.</v>
       </c>
       <c r="G34" t="str">
@@ -2218,8 +2395,9 @@
       <c r="L34" t="str">
         <v>เกม Survival Horror แนวสืบสวนบน PlayStation 3 (รีมาสเตอร์จากเวอร์ชัน Xbox 360) เพิ่ม Content ระบบ Control และ Customization</v>
       </c>
-      <c r="M34" t="str">
-        <v>• รีมาสเตอร์จาก Xbox 360 ไป PS3 ออกแบบ Content, Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Sony Submission • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content</v>
+      <c r="M34" t="str" xml:space="preserve">
+        <v xml:space="preserve">• รีมาสเตอร์จาก Xbox 360 ไป PS3 ออกแบบ Content, Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Sony Submission_x000d__x000d_
+• ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content</v>
       </c>
       <c r="N34" t="str">
         <v>Game</v>
@@ -2242,8 +2420,8 @@
         <v>Wicked Monster BLAST! for PS3 is a casual arcade shooting game on PlayStation 3, where players blast monsters across colorful stages with party-style multiplayer gameplay.</v>
       </c>
       <c r="F35" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Game, level designing and art asset control, produced from the beginning to final product_x000d__x000d__x000d_
-• Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly_x000d__x000d__x000d_
+        <v xml:space="preserve">• Game, level designing and art asset control, produced from the beginning to final product_x000d__x000d__x000d__x000d_
+• Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly_x000d__x000d__x000d__x000d_
 • Game version controlling and submitting game builds and to Sony PlayStation.</v>
       </c>
       <c r="G35" t="str">
@@ -2264,8 +2442,10 @@
       <c r="L35" t="str">
         <v>เกมยิงปีศาจแนวอาร์เคดบน PlayStation 3 ผู้เล่นยิงมอนสเตอร์ผ่านสเตจสีสัน รองรับ Multiplayer สไตล์ปาร์ตี้</v>
       </c>
-      <c r="M35" t="str">
-        <v>• ออกแบบเกม Level Design และควบคุม Art Asset ตั้งแต่ต้นจน Final Product • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content • คุม Game Version และ Submit Build ไป Sony PlayStation</v>
+      <c r="M35" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบเกม Level Design และควบคุม Art Asset ตั้งแต่ต้นจน Final Product_x000d__x000d_
+• ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content_x000d__x000d_
+• คุม Game Version และ Submit Build ไป Sony PlayStation</v>
       </c>
       <c r="N35" t="str">
         <v>Game</v>
@@ -2288,8 +2468,8 @@
         <v>Crazy Strike Bowling for PS3 is a casual bowling game on PlayStation 3 released in US, EU, and Asia regions, featuring fun pin layouts, obstacles, and physics-based gameplay.</v>
       </c>
       <c r="F36" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Functional, regression and playthrough testing to ensure player can go through to all area_x000d__x000d__x000d_
-• Handling responsibility for test tools and developing improvement processes for testing, pin, obstacle and physic editor_x000d__x000d__x000d_
+        <v xml:space="preserve">• Functional, regression and playthrough testing to ensure player can go through to all area_x000d__x000d__x000d__x000d_
+• Handling responsibility for test tools and developing improvement processes for testing, pin, obstacle and physic editor_x000d__x000d__x000d__x000d_
 • Game version controlling and submitting game builds Sony PlayStation US, EU, and Asia.</v>
       </c>
       <c r="G36" t="str">
@@ -2310,8 +2490,10 @@
       <c r="L36" t="str">
         <v>เกมโบวลิ่งแนวแคชวลบน PlayStation 3 วางจำหน่ายใน US, EU และ เอเชีย มีรูปแบบ Pin อุปสรรค และ Gameplay อิง Physic สนุกสนาน</v>
       </c>
-      <c r="M36" t="str">
-        <v>• ทำ Functional, Regression และ Playthrough Testing ให้ผู้เล่นสามารถผ่านไปได้ทุกพื้นที่ของเกม • ดูแล Test Tools และพัฒนา Pin, Obstacle และ Physic Editor • คุม Game Version และ Submit Build ไป Sony PlayStation US, EU และ Asia</v>
+      <c r="M36" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ทำ Functional, Regression และ Playthrough Testing ให้ผู้เล่นสามารถผ่านไปได้ทุกพื้นที่ของเกม_x000d__x000d_
+• ดูแล Test Tools และพัฒนา Pin, Obstacle และ Physic Editor_x000d__x000d_
+• คุม Game Version และ Submit Build ไป Sony PlayStation US, EU และ Asia</v>
       </c>
       <c r="N36" t="str">
         <v>Game</v>
@@ -2334,8 +2516,8 @@
         <v>Wicked Monsters Type! is a Google HTML5 typing game made for promotional purposes, reusing art assets from the original Wicked Monsters shooting game in a typing-based format.</v>
       </c>
       <c r="F37" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Created game design for promotional purposes as a Google HTML5 game_x000d__x000d__x000d_
-• Transfer art assets from the original shooting game to typing game_x000d__x000d__x000d_
+        <v xml:space="preserve">• Created game design for promotional purposes as a Google HTML5 game_x000d__x000d__x000d__x000d_
+• Transfer art assets from the original shooting game to typing game_x000d__x000d__x000d__x000d_
 • Functional and regression testing to ensure the game meets google game acceptance.</v>
       </c>
       <c r="G37" t="str">
@@ -2356,8 +2538,10 @@
       <c r="L37" t="str">
         <v>เกมฝึกพิมพ์บน Google HTML5 สร้างขึ้นเพื่องานโปรโมต โดยนำ Art Asset จาก Wicked Monsters ต้นฉบับมาปรับให้เป็นเกมแนวพิมพ์ดีด</v>
       </c>
-      <c r="M37" t="str">
-        <v>• ออกแบบเกมสำหรับ Google HTML5 เพื่องานโปรโมต • ย้าย Art Asset จากเกมต้นฉบับมาสู่เกมแนวพิมพ์ • ทำ Functional และ Regression Test ให้ผ่านตามมาตรฐานของ Google Game</v>
+      <c r="M37" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ออกแบบเกมสำหรับ Google HTML5 เพื่องานโปรโมต_x000d__x000d_
+• ย้าย Art Asset จากเกมต้นฉบับมาสู่เกมแนวพิมพ์_x000d__x000d_
+• ทำ Functional และ Regression Test ให้ผ่านตามมาตรฐานของ Google Game</v>
       </c>
       <c r="N37" t="str">
         <v>Game</v>
@@ -2380,7 +2564,7 @@
         <v>B-Units: Build It! is a 2D casual construction game where players complete mini-games to build structures, featuring colorful characters and quick tasks. The project involved functional and playthrough testing, game level controlling, and handling test tools for process improvement.</v>
       </c>
       <c r="F38" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Functional and playthrough testing and game level controlling_x000d__x000d__x000d_
+        <v xml:space="preserve">• Functional and playthrough testing and game level controlling_x000d__x000d__x000d__x000d_
 • Handling responsibility for test tools and developing improvement process for testing, managed script editor for level control.</v>
       </c>
       <c r="G38" t="str">
@@ -2401,8 +2585,9 @@
       <c r="L38" t="str">
         <v>B-Units: Build It! เป็นเกมก่อสร้างแนวแคชวลแบบ 2D ผู้เล่นต้องผ่าน Mini Game เพื่อสร้างสิ่งปลูกสร้างต่างๆ มีตัวละครสีสันและภารกิจรวดเร็ว</v>
       </c>
-      <c r="M38" t="str">
-        <v>• ทำ Functional และ Playthrough Testing พร้อมควบคุม Game Level • ดูแล Test Tools และพัฒนากระบวนการทดสอบ รวมถึง Script Editor สำหรับ Level Control</v>
+      <c r="M38" t="str" xml:space="preserve">
+        <v xml:space="preserve">• ทำ Functional และ Playthrough Testing พร้อมควบคุม Game Level_x000d__x000d_
+• ดูแล Test Tools และพัฒนากระบวนการทดสอบ รวมถึง Script Editor สำหรับ Level Control</v>
       </c>
       <c r="N38" t="str">
         <v>Game</v>
@@ -2425,9 +2610,9 @@
         <v>Wicked Monsters BLAST! is a 2D casual shooting game developed by Thai studio Corecell Technology, supporting up to 4 players with fast-paced, arcade-style mini-games.</v>
       </c>
       <c r="F39" t="str" xml:space="preserve">
-        <v xml:space="preserve">• Level designer_x000d__x000d__x000d_
-• Quality assurance_x000d__x000d__x000d_
-• Lead Tester_x000d__x000d__x000d_
+        <v xml:space="preserve">• Level designer_x000d__x000d__x000d__x000d_
+• Quality assurance_x000d__x000d__x000d__x000d_
+• Lead Tester_x000d__x000d__x000d__x000d_
 • Release Control.</v>
       </c>
       <c r="G39" t="str">
@@ -2448,8 +2633,11 @@
       <c r="L39" t="str">
         <v>Wicked Monsters BLAST! เป็นเกมยิงแนว 2D พัฒนาโดยสตูดิโอไทย Corecell Technology รองรับผู้เล่นสูงสุด 4 คน มาพร้อม Mini Game สไตล์อาร์เคดสนุกๆ</v>
       </c>
-      <c r="M39" t="str">
-        <v>• Level Designer • Quality Assurance • Lead Tester • Release Control</v>
+      <c r="M39" t="str" xml:space="preserve">
+        <v xml:space="preserve">• Level Designer_x000d__x000d_
+• Quality Assurance_x000d__x000d_
+• Lead Tester_x000d__x000d_
+• Release Control</v>
       </c>
       <c r="N39" t="str">
         <v>Game</v>

</xml_diff>

<commit_message>
Add header styling to data.xlsx; add style-xlsx.js script
- style-xlsx.js: applies dark-blue header row (bold, white text, frozen,
  auto-filter) and sets column widths on every sheet; also normalises
  line breaks in data cells and enables wrapText — replaces format-xlsx.js
  for day-to-day use
- format-xlsx.js: fix require path (xlsx reinstalled as devDependency)
- package.json / package-lock.json: add exceljs and xlsx as devDependencies

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,30 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\practice\portfolio4\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBA0CC4-E320-4AD4-AAD3-431326172CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Profile" sheetId="1" r:id="rId1"/>
-    <sheet name="Skills" sheetId="2" r:id="rId2"/>
-    <sheet name="Project" sheetId="3" r:id="rId3"/>
-    <sheet name="Contact" sheetId="4" r:id="rId4"/>
-    <sheet name="Experience" sheetId="5" r:id="rId5"/>
-    <sheet name="Education" sheetId="6" r:id="rId6"/>
-    <sheet name="Certifications" sheetId="7" r:id="rId7"/>
-    <sheet name="Awards" sheetId="8" r:id="rId8"/>
-    <sheet name="Tools" sheetId="9" r:id="rId9"/>
-    <sheet name="Playground" sheetId="10" r:id="rId10"/>
+    <sheet sheetId="1" name="Profile" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Skills" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Project" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Contact" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Experience" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Education" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Certifications" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Awards" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Tools" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Playground" state="visible" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -73,7 +67,7 @@
     <t>QA Lead with 14+ years across game development and software testing. ISTQB CTFL certified, passionate about quality, automation, and growing teams.</t>
   </si>
   <si>
-    <t>I have over 10 years of experience in game development across various roles, including Production Manager, and more than 8 years in Quality Assurance with a current focus on software testing. While I am now primarily involved in non-gaming software projects, I maintain a strong passion for the gaming industry and bring a solid understanding of both game production pipelines and modern software development practices, including CI/CD processes.
+    <t xml:space="preserve">I have over 10 years of experience in game development across various roles, including Production Manager, and more than 8 years in Quality Assurance with a current focus on software testing. While I am now primarily involved in non-gaming software projects, I maintain a strong passion for the gaming industry and bring a solid understanding of both game production pipelines and modern software development practices, including CI/CD processes.
 In addition to my technical expertise, I actively mentor team members and take pride in sharing knowledge to help others grow. I believe in building strong, collaborative teams and creating an environment that supports continuous learning. I have been certified with ISTQB CTFL since 2019 and as an Agile Tester (AT) in 2024.</t>
   </si>
   <si>
@@ -89,7 +83,7 @@
     <t>QA Lead ที่คลุกคลีกับวงการพัฒนาเกมและทดสอบซอฟต์แวร์มากว่า 14 ปี ได้รับการรับรอง ISTQB CTFL ชอบงานที่เกี่ยวกับคุณภาพ ระบบทดสอบอัตโนมัติ และการพาทีมเติบโตไปด้วยกัน</t>
   </si>
   <si>
-    <t>ทำงานในวงการเกมมากว่า 10 ปี ผ่านหลายบทบาท รวมถึงตำแหน่ง Production Manager และมีประสบการณ์ด้าน QA อีกกว่า 8 ปี ปัจจุบันโฟกัสที่งานทดสอบซอฟต์แวร์เป็นหลัก แม้จะย้ายมาทำสายซอฟต์แวร์ทั่วไปแล้ว แต่ยังหลงรักวงการเกมอยู่เสมอ และเข้าใจทั้งกระบวนการผลิตเกมและการพัฒนาซอฟต์แวร์สมัยใหม่ รวมถึงงานสาย CI/CD เป็นอย่างดี
+    <t xml:space="preserve">ทำงานในวงการเกมมากว่า 10 ปี ผ่านหลายบทบาท รวมถึงตำแหน่ง Production Manager และมีประสบการณ์ด้าน QA อีกกว่า 8 ปี ปัจจุบันโฟกัสที่งานทดสอบซอฟต์แวร์เป็นหลัก แม้จะย้ายมาทำสายซอฟต์แวร์ทั่วไปแล้ว แต่ยังหลงรักวงการเกมอยู่เสมอ และเข้าใจทั้งกระบวนการผลิตเกมและการพัฒนาซอฟต์แวร์สมัยใหม่ รวมถึงงานสาย CI/CD เป็นอย่างดี
 นอกจากเรื่องเทคนิคแล้ว ยังชอบทำหน้าที่เป็น Mentor ให้น้องๆ ในทีม และยินดีแบ่งปันความรู้เพื่อให้ทุกคนเก่งขึ้นไปด้วยกัน เชื่อในเรื่องการสร้างทีมที่แข็งแรงและบรรยากาศที่เอื้อให้ทุกคนได้เรียนรู้ตลอดเวลา ได้รับการรับรอง ISTQB CTFL ตั้งแต่ปี 2019 และ Agile Tester (AT) ในปี 2024</t>
   </si>
   <si>
@@ -240,7 +234,7 @@
     <t>Lotus's is a major retail chain in Thailand, formerly known as Tesco Lotus, operating a wide range of store formats including hypermarkets, supermarkets, and convenience stores. Lotus's Web (Lotus's Shop Online) is their official online shopping platform, allowing customers to order groceries and household goods through its website or mobile app.</t>
   </si>
   <si>
-    <t>• Manage products and inventory system to meet the requirements
+    <t xml:space="preserve">• Manage products and inventory system to meet the requirements
 • Manage test plan, design and execute test cases
 • Transfer knowledge and provide documents to team
 • Collaborate supporting between teams and investigate issue and root cause.</t>
@@ -258,7 +252,7 @@
     <t>Lotus's เป็นเชนค้าปลีกรายใหญ่ของไทย เดิมชื่อ Tesco Lotus มีร้านหลายรูปแบบ ทั้งไฮเปอร์มาร์เก็ต ซูเปอร์มาร์เก็ต และร้านสะดวกซื้อ ส่วน Lotus's Web (Lotus's Shop Online) คือแพลตฟอร์มช้อปออนไลน์อย่างเป็นทางการ ให้ลูกค้าสั่งของกินของใช้ผ่านเว็บไซต์หรือแอปได้สะดวกๆ</t>
   </si>
   <si>
-    <t>• ดูแลระบบสินค้าและสต็อกให้ตรงตามที่ทีมต้องการ
+    <t xml:space="preserve">• ดูแลระบบสินค้าและสต็อกให้ตรงตามที่ทีมต้องการ
 • วาง Test Plan ออกแบบและรัน Test Case
 • ถ่ายทอดความรู้และทำเอกสารให้ทีม
 • ประสานงานข้ามทีมและสืบหาต้นตอของปัญหา</t>
@@ -282,7 +276,7 @@
     <t>Manao Meals is a web and mobile application that allows company members to order lunch meals as a company benefit. Admins can assign restaurant details and menus, and employees use the app to order food, adjust add-ons, and submit to admin for processing to the restaurant.</t>
   </si>
   <si>
-    <t>• Define test plan, approaches, template and strategy for test coverage
+    <t xml:space="preserve">• Define test plan, approaches, template and strategy for test coverage
 • Define automation test plan, template and contribute documentation
 • Perform functional test and test case design
 • Communicate between developer, QA and project owner.</t>
@@ -294,7 +288,7 @@
     <t>Manao Meals เป็นเว็บและแอปสำหรับสั่งข้าวกลางวันในออฟฟิศเป็นสวัสดิการพนักงาน แอดมินตั้งร้านและเมนูได้ พนักงานก็เข้าแอปไปสั่ง เลือก add-on แล้วส่งให้แอดมินรวบรวมไปสั่งร้านต่อ</t>
   </si>
   <si>
-    <t>• วางแผน Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม
+    <t xml:space="preserve">• วางแผน Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม
 • วาง Automation Test Plan พร้อมเทมเพลตและช่วยทำเอกสาร
 • ทำ Functional Test และออกแบบ Test Case
 • ประสานงานระหว่าง Dev, QA และ Project Owner</t>
@@ -312,7 +306,7 @@
     <t>Seller Center is an E-commerce web application and inventory system that allows vendors (sellers) to join and manage their teams, orders, campaigns, and products. It separates into an admin site (managing other admins, sellers, and transactions) and a seller site (managing shop products and order transactions).</t>
   </si>
   <si>
-    <t>• Manage and contribute documentation
+    <t xml:space="preserve">• Manage and contribute documentation
 • Define test plan, approaches, template and strategy for test coverage
 • Perform functional test and test case design
 • Communicate between developer, QA and project owner.</t>
@@ -324,7 +318,7 @@
     <t>Seller Center เป็นเว็บ E-commerce และระบบสต็อกที่ให้ผู้ขาย (Seller) เข้ามาจัดการทีม ออเดอร์ แคมเปญ และสินค้าได้ แบ่งเป็นฝั่ง Admin (จัดการแอดมินอื่น ผู้ขาย และธุรกรรม) กับฝั่ง Seller (จัดการสินค้าในร้านและออเดอร์)</t>
   </si>
   <si>
-    <t>• ดูแลและช่วยจัดทำเอกสาร
+    <t xml:space="preserve">• ดูแลและช่วยจัดทำเอกสาร
 • วาง Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม
 • ทำ Functional Test และออกแบบ Test Case
 • ประสานงานระหว่าง Dev, QA และ Project Owner</t>
@@ -339,7 +333,7 @@
     <t>PTT Digital is a finance application for PTT, requiring Quality Assurance standards and DevSecOps processes to ensure secure and reliable transactions.</t>
   </si>
   <si>
-    <t>• Contribute documentation for Standard Quality Assurance, covering DevSecOps process with user acceptance criteria
+    <t xml:space="preserve">• Contribute documentation for Standard Quality Assurance, covering DevSecOps process with user acceptance criteria
 • Communicate between developer, QA and project owner.</t>
   </si>
   <si>
@@ -349,7 +343,7 @@
     <t>PTT Digital เป็นแอปด้านการเงินของ ปตท. ที่ต้องการมาตรฐาน QA และกระบวนการ DevSecOps เพื่อให้ทุกธุรกรรมปลอดภัยและเชื่อถือได้</t>
   </si>
   <si>
-    <t>• จัดทำเอกสารมาตรฐาน QA ครอบคลุมกระบวนการ DevSecOps พร้อมเงื่อนไขการรับมอบงานจากผู้ใช้
+    <t xml:space="preserve">• จัดทำเอกสารมาตรฐาน QA ครอบคลุมกระบวนการ DevSecOps พร้อมเงื่อนไขการรับมอบงานจากผู้ใช้
 • ประสานงานระหว่าง Dev, QA และ Project Owner</t>
   </si>
   <si>
@@ -365,7 +359,7 @@
     <t>True Online Store is an E-commerce website by True Corporation, providing True products and services for customers and True membership.</t>
   </si>
   <si>
-    <t>• Test planning, analysis and design to cover business requirements
+    <t xml:space="preserve">• Test planning, analysis and design to cover business requirements
 • Test case design and execution from day-to-day basis
 • Generate test data and test script for manual and automation testing
 • Perform static and dynamic testing to cover acceptances.</t>
@@ -377,7 +371,7 @@
     <t>True Online Store เป็นเว็บ E-commerce ของ True Corporation ขายสินค้าและบริการของทรู รวมถึงสิทธิประโยชน์สำหรับสมาชิก True</t>
   </si>
   <si>
-    <t>• วางแผน วิเคราะห์ และออกแบบการทดสอบให้ครอบคลุม Business Requirement
+    <t xml:space="preserve">• วางแผน วิเคราะห์ และออกแบบการทดสอบให้ครอบคลุม Business Requirement
 • ออกแบบและรัน Test Case ในงานประจำวัน
 • เตรียม Test Data และเขียน Test Script ทั้งแบบ Manual และ Automation
 • ทำทั้ง Static และ Dynamic Testing เพื่อให้ผ่านเกณฑ์รับมอบ</t>
@@ -398,7 +392,7 @@
     <t>Linage W is a global scale MMORPG where players fight for their glories, set 150 years after the original Lineage story in the Aden World. Players can pick a story among lord, knight, fairy, and mage to explore a dark fantasy world.</t>
   </si>
   <si>
-    <t>• Define test scope, plan, data and documentation to cover test standard
+    <t xml:space="preserve">• Define test scope, plan, data and documentation to cover test standard
 • Maintenance testing, investigate and analyze issues
 • Playthrough testing as end-user on production environment.</t>
   </si>
@@ -415,7 +409,7 @@
     <t>Lineage W เป็นเกม MMORPG ระดับโลก ซึ่งผู้เล่นต้องต่อสู้เพื่อชื่อเสียงของตัวเอง ดำเนินเรื่องหลังจาก Lineage ภาคแรก 150 ปี ในโลก Aden ผู้เล่นสามารถเลือกเล่นเป็นขุนนาง อัศวิน นางฟ้า หรือพ่อมด เพื่อผจญภัยในโลกแฟนตาซีลึกลับ</t>
   </si>
   <si>
-    <t>• กำหนดขอบเขตการทดสอบ Test Plan ข้อมูล และเอกสารให้ตรงตามมาตรฐาน
+    <t xml:space="preserve">• กำหนดขอบเขตการทดสอบ Test Plan ข้อมูล และเอกสารให้ตรงตามมาตรฐาน
 • ทำ Maintenance Testing ตรวจสอบและวิเคราะห์ปัญหา
 • เล่นจริงในมุมมองผู้ใช้งานบน Production</t>
   </si>
@@ -438,7 +432,7 @@
     <t>The project focused on the 'ALL member' 7-Eleven membership program via the 7App. This program allows users to get discounts, earn coupons, check, redeem, and transfer ALL points, and pay with credit cards via Truemoney Wallet at 7-Eleven stores, 7Delivery service, and All Online.</t>
   </si>
   <si>
-    <t>• Supervision and coordinate between teams, developers, internal and external QA
+    <t xml:space="preserve">• Supervision and coordinate between teams, developers, internal and external QA
 • Test analysis, planning and management
 • Manage QA processes for new campaigns and features for each release
 • Transfer testing tool knowledge to teams.</t>
@@ -453,7 +447,7 @@
     <t>โปรเจกต์นี้เน้นที่ระบบสมาชิก 'ALL Member' ผ่านแอป 7App ผู้ใช้รับส่วนลด เก็บคูปอง เช็ค แลก และโอนคะแนน ALL Point รวมถึงจ่ายผ่านบัตรเครดิตผ่าน TrueMoney Wallet ที่ร้าน 7-Eleven, บริการ 7Delivery และ All Online</t>
   </si>
   <si>
-    <t>• ดูแลและประสานงานระหว่างทีม Dev และทีม QA ทั้งภายในและภายนอก
+    <t xml:space="preserve">• ดูแลและประสานงานระหว่างทีม Dev และทีม QA ทั้งภายในและภายนอก
 • วิเคราะห์ วางแผน และบริหารจัดการงานทดสอบ
 • ดูแลกระบวนการ QA สำหรับแคมเปญและฟีเจอร์ใหม่ในแต่ละ Release
 • ถ่ายทอดความรู้เรื่องเครื่องมือทดสอบให้ทีม</t>
@@ -471,7 +465,7 @@
     <t>Aliveunited is a digital platform that focuses on UI/UX design and system flow for end users, with consultation between project owner and design team.</t>
   </si>
   <si>
-    <t>• Test planning, monitoring, analysis and design
+    <t xml:space="preserve">• Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers
 • Design, UI and UX consultant with Project Owner to analyze the whole system.</t>
@@ -483,7 +477,7 @@
     <t>Aliveunited เป็นแพลตฟอร์มดิจิทัลที่เน้นการออกแบบ UI/UX และ System Flow สำหรับผู้ใช้ ผ่านการปรึกษาระหว่าง Project Owner กับทีมดีไซน์</t>
   </si>
   <si>
-    <t>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
+    <t xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager
 • ให้คำปรึกษาด้าน Design, UI และ UX ร่วมกับ Project Owner เพื่อวิเคราะห์ระบบทั้งหมด</t>
@@ -501,7 +495,7 @@
     <t>The Curaprox App (iOS, Android) is designed to help users stay motivated in their daily dental routines, ensuring preventive dental care year-round. It allows connection with dental professionals and access to lectures, articles, and products.</t>
   </si>
   <si>
-    <t>• Test planning, monitoring, analysis and design
+    <t xml:space="preserve">• Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers.</t>
   </si>
@@ -509,7 +503,7 @@
     <t>แอป Curaprox (iOS, Android) ช่วยสร้างแรงจูงใจในการดูแลสุขภาพฟันประจำวัน เพื่อการดูแลฟันเชิงป้องกันตลอดปี สามารถเชื่อมต่อกับทันตแพทย์ อ่านบทความ และเข้าถึงผลิตภัณฑ์ได้ผ่านแอป</t>
   </si>
   <si>
-    <t>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
+    <t xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager</t>
   </si>
@@ -538,7 +532,7 @@
     <t>Hotel Life: A Resort Simulator is a simulation game where players build and manage their own resort, designing rooms, attractions, and services to attract guests.</t>
   </si>
   <si>
-    <t>• Test planning, monitoring, analysis and design
+    <t xml:space="preserve">• Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers
 • Coordinated developer team to request test tools for game level testing and improve QA processes
@@ -551,7 +545,7 @@
     <t>Hotel Life: A Resort Simulator เป็นเกมแนวสร้างและบริหารรีสอร์ตของตัวเอง ผู้เล่นออกแบบห้องพัก สิ่งอำนวยความสะดวก และสถานที่ท่องเที่ยวต่างๆ เพื่อดึงดูดลูกค้า</t>
   </si>
   <si>
-    <t>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
+    <t xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager
 • ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA
@@ -564,10 +558,13 @@
     <t>Lumen.</t>
   </si>
   <si>
-    <t>Lumen. is a puzzle game on Apple Arcade where players solve levels using lights lenses and mirrors
+    <t xml:space="preserve">Lumen. is a puzzle game on Apple Arcade where players solve levels using lights lenses and mirrors
   discovering a mysterious antique box.</t>
   </si>
   <si>
+    <t>Lumen</t>
+  </si>
+  <si>
     <t>Lumen. เป็นเกมปริศนาบน Apple Arcade ผู้เล่นไขปริศนาแต่ละด่านด้วยแสง เลนส์ และกระจก พร้อมไขปริศนาของกล่องโบราณลึกลับ</t>
   </si>
   <si>
@@ -583,7 +580,7 @@
     <t>Pick is a mobile application that connects with hardware devices, allowing users to synchronize and control device functions through the app.</t>
   </si>
   <si>
-    <t>• Coordinated with the external production and passed testing criteria to external tester teams
+    <t xml:space="preserve">• Coordinated with the external production and passed testing criteria to external tester teams
 • Functional, and API testing between software and hardware remotely to ensure app can synchronize as client acceptance.</t>
   </si>
   <si>
@@ -593,7 +590,7 @@
     <t>Pick เป็นแอปมือถือที่เชื่อมต่อกับ Hardware ผู้ใช้สามารถซิงโครไนซ์และควบคุมการทำงานของอุปกรณ์ผ่านแอปได้</t>
   </si>
   <si>
-    <t>• ประสานงานกับผู้ผลิตภายนอก และส่งต่อ Test Criteria ให้ทีม Tester ภายนอก
+    <t xml:space="preserve">• ประสานงานกับผู้ผลิตภายนอก และส่งต่อ Test Criteria ให้ทีม Tester ภายนอก
 • ทำ Functional Test และ API Test ระหว่าง Software กับ Hardware แบบ Remote เพื่อยืนยันว่าแอปซิงโครไนซ์ได้ตามที่ลูกค้าต้องการ</t>
   </si>
   <si>
@@ -609,7 +606,7 @@
     <t>City of Games is an app allowing free play of classic and no-commission baccarat modes, featuring 3D card squeezing, available on iOS, Android, and Chinese Android.</t>
   </si>
   <si>
-    <t>• Release control, submit application to Apple and Google stores
+    <t xml:space="preserve">• Release control, submit application to Apple and Google stores
 • Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers
@@ -622,7 +619,7 @@
     <t>City of Games เป็นแอปที่ให้เล่นบาคาร่าแบบคลาสสิกและไร้ค่าคอมมิชชั่น ฟรี มีระบบเปิดไพ่สามมิติ รองรับทั้ง iOS, Android และ Android ของจีน</t>
   </si>
   <si>
-    <t>• ดูแล Release Control และ Submit แอปขึ้น Apple และ Google Store
+    <t xml:space="preserve">• ดูแล Release Control และ Submit แอปขึ้น Apple และ Google Store
 • วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager
@@ -641,7 +638,7 @@
     <t>Tint. is a mobile and console game available on iOS, MacOS, and TvOS, designed to work with and without peripheral game controllers.</t>
   </si>
   <si>
-    <t>• Coordinated with the external production and passed testing criteria and other game information to external tester teams
+    <t xml:space="preserve">• Coordinated with the external production and passed testing criteria and other game information to external tester teams
 • Functional testing of new features and playthrough testing to ensure the game can progress correctly as expected with new integrated contents
 • Monitoring external teams closely from the regression process to cover client and store acceptance
 • Device coverage testing, to ensure app can work correctly on MacOS, TvOS and iOS devices with and without peripheral game controllers.</t>
@@ -653,7 +650,7 @@
     <t>Tint. เป็นเกมบนมือถือและคอนโซล รองรับทั้ง iOS, MacOS และ tvOS ออกแบบมาให้เล่นได้ทั้งแบบใช้และไม่ใช้ Game Controller เสริม</t>
   </si>
   <si>
-    <t>• ประสานงานกับผู้ผลิตภายนอก ส่งต่อ Test Criteria และข้อมูลเกมให้ทีม Tester ภายนอก
+    <t xml:space="preserve">• ประสานงานกับผู้ผลิตภายนอก ส่งต่อ Test Criteria และข้อมูลเกมให้ทีม Tester ภายนอก
 • Functional Test ฟีเจอร์ใหม่ และ Playthrough เพื่อให้มั่นใจว่าเกมเล่นได้ต่อเนื่องตามที่คาดหวังหลังรวม Content ใหม่
 • ติดตามทีมภายนอกอย่างใกล้ชิดตอนทำ Regression เพื่อรองรับรีควอเรมนต์ของลูกค้าและ Store
 • ทดสอบการรองรับอุปกรณ์ให้แอปทำงานได้บน MacOS, tvOS และ iOS ทั้งแบบใช้และไม่ใช้ Game Controller</t>
@@ -671,7 +668,7 @@
     <t>Panya is a mobile application designed to work reliably across various network conditions, with a focus on stability and performance for end users.</t>
   </si>
   <si>
-    <t>• Test planning, gathered new requirements from clients directly and passed on information to the tester team
+    <t xml:space="preserve">• Test planning, gathered new requirements from clients directly and passed on information to the tester team
 • Test suite control, created, updated, prioritized and defined test cases from test suite for regression testing to reach client acceptance
 • Handled responsibility for test tools, implemented processes for automation to prepare test data, and created technical documents for internal purposes
 • Investigated network link conditions to perform stability testing, making sure the app works to various network status.</t>
@@ -683,7 +680,7 @@
     <t>Panya เป็นแอปมือถือที่ออกแบบมาให้ทำงานได้อย่างเสถียรบนสภาพเครือข่ายที่หลากหลาย มุ่งเน้นความเสถียรและประสิทธิภาพสำหรับผู้ใช้</t>
   </si>
   <si>
-    <t>• วางแผนการทดสอบ รับ Requirement จากลูกค้าโดยตรงและส่งต่อให้ทีม Tester
+    <t xml:space="preserve">• วางแผนการทดสอบ รับ Requirement จากลูกค้าโดยตรงและส่งต่อให้ทีม Tester
 • จัดการ Test Suite — สร้าง อัปเดต จัดลำดับความสำคัญ และกำหนด Test Case สำหรับ Regression ให้ตรงตามที่ลูกค้ายอมรับ
 • ดูแล Test Tools วางแนวทาง Automation สำหรับจัดเตรียม Test Data พร้อมทำเอกสารทางเทคนิคภายใน
 • ตรวจสภาพเครือข่ายเพื่อทำ Stability Testing ให้มั่นใจว่าแอปทำงานได้ในทุกสภาพเน็ตเวิร์ก</t>
@@ -722,7 +719,7 @@
     <t>ImaginMe Beauty and the Beast is a personalized interactive storybook app where users customize their character to star in the Beauty and the Beast story, featuring mini-games and animated scenes.</t>
   </si>
   <si>
-    <t>• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
+    <t xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
 • Art Asset management, designed specification, limitation and performed optimization for device coverage
 • Level designing with Unity to generate mini games and performed own unit, integration and system testing to meet requirements
 • Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing
@@ -735,7 +732,7 @@
     <t>เป็นแอปหนังสือนิทานส่วนตัวที่ผู้ใช้ปรับแต่งตัวละครได้เอง ร่วมผจญภัยในเรื่องโฉมงามกับเจ้าชายอสูร พร้อมมินิเกมและฉากแอนิเมชัน</t>
   </si>
   <si>
-    <t>• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
+    <t xml:space="preserve">• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
 • จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย
 • ทำ Level Design ด้วย Unity สร้าง Mini Game พร้อม Unit, Integration และ System Test ของตัวเองให้ตรงตาม Requirement
 • ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop
@@ -751,7 +748,7 @@
     <t>ImaginMe Dragons is a personalized interactive storybook app where users customize their character to star in a dragon-themed adventure, featuring mini-games with patterns and obstacles.</t>
   </si>
   <si>
-    <t>• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
+    <t xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
 • Art Asset management, designed specification, limitation and performed optimization for device coverage
 • Level designing with Unity to generate pattern and obstacles and performed own unit, integration and system testing to meet requirements
 • Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing
@@ -764,7 +761,7 @@
     <t>หนังสือนิทานส่วนตัวธีมมังกร ที่ผู้ใช้ปรับแต่งตัวละครได้เอง ร่วมผจญภัยผ่านมินิเกมที่มีรูปแบบและอุปสรรคหลากหลาย</t>
   </si>
   <si>
-    <t>• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
+    <t xml:space="preserve">• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
 • จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย
 • ทำ Level Design ด้วย Unity สร้างรูปแบบและอุปสรรค พร้อม Unit, Integration และ System Test
 • ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop
@@ -819,7 +816,7 @@
     <t>Tesco Lotus Shopping Spree is a promotional infinite running game for Tesco Lotus, designed for low-end mobile devices, where players run through stages to collect items and rewards.</t>
   </si>
   <si>
-    <t>• Built on client concepts to design promotional infinite running games to meet client acceptance
+    <t xml:space="preserve">• Built on client concepts to design promotional infinite running games to meet client acceptance
 • Designed specification, limitation and optimization to cover low end devices
 • Level designing with Unity to generate stage patterns and perform own unit, integration and system testing
 • Handling responsibility for test tools and developing improvement processes.</t>
@@ -831,7 +828,7 @@
     <t>เกมประชาสัมพันธ์แนว Infinite Running ของเทสโก้โลตัส ทำงานได้บนมือถือสเป็กต่ำ ผู้เล่นวิ่งผ่านด่านต่างๆ เพื่อเก็บไอเท็มและรางวัล</t>
   </si>
   <si>
-    <t>• ออกแบบเกม Promotional Infinite Running ตามคอนเซ็ปต์ของลูกค้า
+    <t xml:space="preserve">• ออกแบบเกม Promotional Infinite Running ตามคอนเซ็ปต์ของลูกค้า
 • ออกแบบ Spec ข้อจำกัด และ Optimize ให้รองรับมือถือ Spec ต่ำ
 • ทำ Level Design ด้วย Unity สร้าง Stage Pattern พร้อม Unit, Integration และ System Test
 • ดูแล Test Tools และพัฒนาปรับปรุงกระบวนการ</t>
@@ -849,7 +846,7 @@
     <t>Totem Defender is a free-to-play tower defense game for mobile, where players use totems to defend against waves of enemies across multiple stages and difficulty levels.</t>
   </si>
   <si>
-    <t>• Project planning, built on client concepts to design games contents from scratch to be the final product to meet client acceptance
+    <t xml:space="preserve">• Project planning, built on client concepts to design games contents from scratch to be the final product to meet client acceptance
 • Researched and designed monetization for F2P games, targeted to both free and paid mobile users
 • Level designing with Unity to generate stage patterns, level progress, difficulty level and perform own unit, integration and system testing to cover low end devices
 • Coordinated with the production team closely and managed sprint goal planning.</t>
@@ -861,7 +858,7 @@
     <t>Totem Defender เป็นเกม Tower Defense แบบ Free-to-Play บนมือถือ ผู้เล่นใช้โทเท็มป้องกันศัตรูที่บุกเข้ามาเป็นระลอกไปในหลายด่านและหลายระดับความยาก</t>
   </si>
   <si>
-    <t>• วางแผนโปรเจกต์ ออกแบบเนื้อหาเกมตั้งแต่ต้นจนถึง Final Product ตามคอนเซ็ปต์ลูกค้า
+    <t xml:space="preserve">• วางแผนโปรเจกต์ ออกแบบเนื้อหาเกมตั้งแต่ต้นจนถึง Final Product ตามคอนเซ็ปต์ลูกค้า
 • วิจัยและออกแบบระบบ Monetization สำหรับเกม F2P รองรับทั้งผู้เล่นฟรีและจ่ายเงิน
 • ทำ Level Design ด้วย Unity สร้าง Stage Pattern, Level Progress และ Difficulty พร้อมทดสอบให้รองรับมือถือ Spec ต่ำ
 • ประสานงานกับทีม Production อย่างใกล้ชิด และจัดการ Sprint Goal Planning</t>
@@ -879,7 +876,7 @@
     <t>Mes Comptines for 3DS is a children's music game on Nintendo 3DS that combines karaoke and rhythm tap gameplay, helping kids sing along to French nursery rhymes.</t>
   </si>
   <si>
-    <t>• Built on client concepts to design additional game play from karaoke to rhythm tap game to meet client acceptance
+    <t xml:space="preserve">• Built on client concepts to design additional game play from karaoke to rhythm tap game to meet client acceptance
 • Level designing, improved learning curve to cover more target players and replayability with various difficulty levels
 • Game version controlling and submitting game builds via Nintendo with LotCheck guidelines.</t>
   </si>
@@ -890,7 +887,7 @@
     <t>Mes Comptines for 3DS เป็นเกมดนตรีสำหรับเด็กบน Nintendo 3DS ผสมผสานระหว่างคาราโอเกะกับเกมจังหวะตามจังหวะ ช่วยให้เด็กร้องตามเพลงกล่อมเด็กภาษาฝรั่งเศส</t>
   </si>
   <si>
-    <t>• ออกแบบ Gameplay เพิ่มเติมจากคาราโอเกะไปสู่เกมจังหวะตามจังหวะ ตามคอนเซ็ปต์ของลูกค้า
+    <t xml:space="preserve">• ออกแบบ Gameplay เพิ่มเติมจากคาราโอเกะไปสู่เกมจังหวะตามจังหวะ ตามคอนเซ็ปต์ของลูกค้า
 • ปรับปรุง Learning Curve ให้ครอบคลุมผู้เล่นหลายกลุ่ม และเพิ่ม Replayability ด้วยระดับความยากหลายระดับ
 • คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</t>
   </si>
@@ -949,7 +946,7 @@
     <t>Lolirock is a music and karaoke game based on the Lolirock animated series, featuring character and stage customization with mini-games synced to the show's vocal lines.</t>
   </si>
   <si>
-    <t>• Level designing, design karaoke pitch level and synced to vocal line
+    <t xml:space="preserve">• Level designing, design karaoke pitch level and synced to vocal line
 • Functional and regression testing to mini game, character and stage customization.</t>
   </si>
   <si>
@@ -959,7 +956,7 @@
     <t>เกมดนตรีและคาราโอเกะที่อิงจากการ์ตูน Lolirock มี Mini Game ซิงกับเสียงร้อง พร้อมออกแบบตัวละครและเวที</t>
   </si>
   <si>
-    <t>• ออกแบบ Karaoke Pitch Level ให้ซิงค์กับ Vocal
+    <t xml:space="preserve">• ออกแบบ Karaoke Pitch Level ให้ซิงค์กับ Vocal
 • ทำ Functional และ Regression Test ให้กับ Mini Game รวมถึงระบบตัวละครและเวที</t>
   </si>
   <si>
@@ -975,7 +972,7 @@
     <t>Meine ersten Mitsing-Lieder for WiiU is a children's karaoke game on Nintendo WiiU (remastered from the Wii version), featuring German nursery rhymes with peripheral device support.</t>
   </si>
   <si>
-    <t>• Remastering from Wii to WiiU version, functional and regression testing with peripheral devices
+    <t xml:space="preserve">• Remastering from Wii to WiiU version, functional and regression testing with peripheral devices
 • Customer supporting and services
 • Game version controlling and submitting game builds via Nintendo with LotCheck guidelines.</t>
   </si>
@@ -986,7 +983,7 @@
     <t>เกมคาราโอเกะสำหรับเด็กบน Nintendo Wii U (ปรับจากเวอร์ชัน Wii) ร้องเพลงกล่อมเด็กภาษาเยอรมัน พร้อมรองรับอุปกรณ์เสริม</t>
   </si>
   <si>
-    <t>• ปรับ Wii ไปเป็นเวอร์ชัน Wii U พร้อมทำ Functional และ Regression Test ร่วมกับอุปกรณ์เสริม
+    <t xml:space="preserve">• ปรับ Wii ไปเป็นเวอร์ชัน Wii U พร้อมทำ Functional และ Regression Test ร่วมกับอุปกรณ์เสริม
 • สนับสนุนลูกค้า
 • คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</t>
   </si>
@@ -1045,7 +1042,7 @@
     <t>AeternoBlade for 3DS is a 2D side-scrolling action game on Nintendo 3DS where players control Freyja, who uses a magical blade to manipulate time and battle enemies across multiple stages.</t>
   </si>
   <si>
-    <t>• Handling responsibility for test tools and QA improvement processes
+    <t xml:space="preserve">• Handling responsibility for test tools and QA improvement processes
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly
 • Handling responsibility for test tools and developing improvement processes for testing and generating game cutscenes
 • Level designing and difficulty control, fine tuning effects and particles
@@ -1059,7 +1056,7 @@
     <t>AeternoBlade for 3DS เป็นเกมแอ็กชั่นแบบ 2D Side-Scrolling บน Nintendo 3DS ผู้เล่นบังคับ Freyja ที่ใช้ดาบเวทมนต์บิดผันเวลาบุกออกต่อสู้ศัตรูผ่านหลายด่าน</t>
   </si>
   <si>
-    <t>• ดูแล Test Tools และปรับปรุงกระบวนการ QA
+    <t xml:space="preserve">• ดูแล Test Tools และปรับปรุงกระบวนการ QA
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตามที่ออกแบบไว้
 • พัฒนา Test Tools สำหรับทดสอบและสร้าง Cutscene ของเกม
 • ทำ Level Design และ Difficulty Control รวมถึง Fine-Tune Effect และ Particle
@@ -1079,7 +1076,7 @@
     <t>Deadly Premonition: The Director's Cut for Steam is a survival horror mystery game on Steam (built from the PS3 version), where players investigate a series of murders in a small American town.</t>
   </si>
   <si>
-    <t>• Built on PS3 and Steam versions, designed additional contents, character control and customization to match with client, Steam submission requirements
+    <t xml:space="preserve">• Built on PS3 and Steam versions, designed additional contents, character control and customization to match with client, Steam submission requirements
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly as requirements.</t>
   </si>
   <si>
@@ -1089,7 +1086,7 @@
     <t>เกม Survival Horror แนวสืบสวนบน Steam (พอร์ตมาจากเวอร์ชัน PS3) ผู้เล่นสืบสวนคดีฝาต่อเนื่องในเมืองเล็กของอเมริกา</t>
   </si>
   <si>
-    <t>• พอร์ตจากเวอร์ชัน PS3 ไป Steam ออกแบบ Content เพิ่ม ระบบ Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Steam Submission
+    <t xml:space="preserve">• พอร์ตจากเวอร์ชัน PS3 ไป Steam ออกแบบ Content เพิ่ม ระบบ Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Steam Submission
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตาม Requirement</t>
   </si>
   <si>
@@ -1105,14 +1102,14 @@
     <t>Deadly Premonition: Director's Cut for PS3 is a survival horror mystery game on PlayStation 3 (remastered from Xbox 360), with added content, character controls, and customization.</t>
   </si>
   <si>
-    <t>• Remastering from XBOX360 to PS3 version, designed additional contents, character control and customization to match with client, Sony submission requirements
+    <t xml:space="preserve">• Remastering from XBOX360 to PS3 version, designed additional contents, character control and customization to match with client, Sony submission requirements
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly as requirements.</t>
   </si>
   <si>
     <t>เกม Survival Horror แนวสืบสวนบน PlayStation 3 (รีมาสเตอร์จากเวอร์ชัน Xbox 360) เพิ่ม Content ระบบ Control และ Customization</t>
   </si>
   <si>
-    <t>• รีมาสเตอร์จาก Xbox 360 ไป PS3 ออกแบบ Content, Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Sony Submission
+    <t xml:space="preserve">• รีมาสเตอร์จาก Xbox 360 ไป PS3 ออกแบบ Content, Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Sony Submission
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content</t>
   </si>
   <si>
@@ -1128,7 +1125,7 @@
     <t>Puzzle game for promotional purpose</t>
   </si>
   <si>
-    <t>• Created game design for promotional purposes
+    <t xml:space="preserve">• Created game design for promotional purposes
 • Functional, level design and regression testing</t>
   </si>
   <si>
@@ -1138,7 +1135,7 @@
     <t>เกมพัซเซิลใช้ในการโปรโมทสินค้า</t>
   </si>
   <si>
-    <t>• ออกแบบเกมสำหรับ เพื่องานโปรโมต
+    <t xml:space="preserve">• ออกแบบเกมสำหรับ เพื่องานโปรโมต
 • ทำ Functional level design และ Regression Test</t>
   </si>
   <si>
@@ -1154,7 +1151,7 @@
     <t>Wicked Monster BLAST! for PS3 is a casual arcade shooting game on PlayStation 3, where players blast monsters across colorful stages with party-style multiplayer gameplay.</t>
   </si>
   <si>
-    <t>• Game, level designing and art asset control, produced from the beginning to final product
+    <t xml:space="preserve">• Game, level designing and art asset control, produced from the beginning to final product
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly
 • Game version controlling and submitting game builds and to Sony PlayStation.</t>
   </si>
@@ -1165,7 +1162,7 @@
     <t>เกมยิงปีศาจแนวอาร์เคดบน PlayStation 3 ผู้เล่นยิงมอนสเตอร์ผ่านสเตจสีสัน รองรับ Multiplayer สไตล์ปาร์ตี้</t>
   </si>
   <si>
-    <t>• ออกแบบเกม Level Design และควบคุม Art Asset ตั้งแต่ต้นจน Final Product
+    <t xml:space="preserve">• ออกแบบเกม Level Design และควบคุม Art Asset ตั้งแต่ต้นจน Final Product
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content
 • คุม Game Version และ Submit Build ไป Sony PlayStation</t>
   </si>
@@ -1182,7 +1179,7 @@
     <t>Crazy Strike Bowling for PS3 is a casual bowling game on PlayStation 3 released in US, EU, and Asia regions, featuring fun pin layouts, obstacles, and physics-based gameplay.</t>
   </si>
   <si>
-    <t>• Functional, regression and playthrough testing to ensure player can go through to all area
+    <t xml:space="preserve">• Functional, regression and playthrough testing to ensure player can go through to all area
 • Handling responsibility for test tools and developing improvement processes for testing, pin, obstacle and physic editor
 • Game version controlling and submitting game builds Sony PlayStation US, EU, and Asia.</t>
   </si>
@@ -1193,7 +1190,7 @@
     <t>เกมโบวลิ่งแนวแคชวลบน PlayStation 3 วางจำหน่ายใน US, EU และ เอเชีย มีรูปแบบ Pin อุปสรรค และ Gameplay อิง Physic สนุกสนาน</t>
   </si>
   <si>
-    <t>• ทำ Functional, Regression และ Playthrough Testing ให้ผู้เล่นสามารถผ่านไปได้ทุกพื้นที่ของเกม
+    <t xml:space="preserve">• ทำ Functional, Regression และ Playthrough Testing ให้ผู้เล่นสามารถผ่านไปได้ทุกพื้นที่ของเกม
 • ดูแล Test Tools และพัฒนา Pin, Obstacle และ Physic Editor
 • คุม Game Version และ Submit Build ไป Sony PlayStation US, EU และ Asia</t>
   </si>
@@ -1210,7 +1207,7 @@
     <t>Wicked Monsters Type! is a Google HTML5 typing game made for promotional purposes, reusing art assets from the original Wicked Monsters shooting game in a typing-based format.</t>
   </si>
   <si>
-    <t>• Created game design for promotional purposes as a Google HTML5 game
+    <t xml:space="preserve">• Created game design for promotional purposes as a Google HTML5 game
 • Transfer art assets from the original shooting game to typing game
 • Functional and regression testing to ensure the game meets google game acceptance.</t>
   </si>
@@ -1221,7 +1218,7 @@
     <t>เกมฝึกพิมพ์บน Google HTML5 สร้างขึ้นเพื่องานโปรโมต โดยนำ Art Asset จาก Wicked Monsters ต้นฉบับมาปรับให้เป็นเกมแนวพิมพ์ดีด</t>
   </si>
   <si>
-    <t>• ออกแบบเกมสำหรับ Google HTML5 เพื่องานโปรโมต
+    <t xml:space="preserve">• ออกแบบเกมสำหรับ Google HTML5 เพื่องานโปรโมต
 • ย้าย Art Asset จากเกมต้นฉบับมาสู่เกมแนวพิมพ์
 • ทำ Functional และ Regression Test ให้ผ่านตามมาตรฐานของ Google Game</t>
   </si>
@@ -1238,7 +1235,7 @@
     <t>B-Units: Build It! is a 2D casual construction game where players complete mini-games to build structures, featuring colorful characters and quick tasks. The project involved functional and playthrough testing, game level controlling, and handling test tools for process improvement.</t>
   </si>
   <si>
-    <t>• Functional and playthrough testing and game level controlling
+    <t xml:space="preserve">• Functional and playthrough testing and game level controlling
 • Handling responsibility for test tools and developing improvement process for testing, managed script editor for level control.</t>
   </si>
   <si>
@@ -1248,7 +1245,7 @@
     <t>B-Units: Build It! เป็นเกมก่อสร้างแนวแคชวลแบบ 2D ผู้เล่นต้องผ่าน Mini Game เพื่อสร้างสิ่งปลูกสร้างต่างๆ มีตัวละครสีสันและภารกิจรวดเร็ว</t>
   </si>
   <si>
-    <t>• ทำ Functional และ Playthrough Testing พร้อมควบคุม Game Level
+    <t xml:space="preserve">• ทำ Functional และ Playthrough Testing พร้อมควบคุม Game Level
 • ดูแล Test Tools และพัฒนากระบวนการทดสอบ รวมถึง Script Editor สำหรับ Level Control</t>
   </si>
   <si>
@@ -1264,7 +1261,7 @@
     <t>Wicked Monsters BLAST! is a 2D casual shooting game developed by Thai studio Corecell Technology, supporting up to 4 players with fast-paced, arcade-style mini-games.</t>
   </si>
   <si>
-    <t>• Level designer
+    <t xml:space="preserve">• Level designer
 • Quality assurance
 • Lead Tester
 • Release Control.</t>
@@ -1276,7 +1273,7 @@
     <t>Wicked Monsters BLAST! เป็นเกมยิงแนว 2D พัฒนาโดยสตูดิโอไทย Corecell Technology รองรับผู้เล่นสูงสุด 4 คน มาพร้อม Mini Game สไตล์อาร์เคดสนุกๆ</t>
   </si>
   <si>
-    <t>• Level Designer
+    <t xml:space="preserve">• Level Designer
 • Quality Assurance
 • Lead Tester
 • Release Control</t>
@@ -1330,7 +1327,7 @@
     <t>MegaXGame is a Thai gaming magazine known for its comprehensive coverage, expert walkthroughs, and deep dives into the gaming world.</t>
   </si>
   <si>
-    <t>• Fast and simple updates on new releases.
+    <t xml:space="preserve">• Fast and simple updates on new releases.
 • Honest opinions and gameplay breakdowns.
 • Deep dives into combos and fighting mechanics.
 • Selecting visuals and engaging with the community.</t>
@@ -1345,7 +1342,7 @@
     <t>MegaXGame เป็นนิตยสารที่อยู่คู่เกมเมอร์ไทยมานาน เน้นเนื้อหาที่เข้มข้น ครบเครื่อง ทั้งข่าวสาร บทสรุป และบทวิเคราะห์ที่เข้าถึงง่าย</t>
   </si>
   <si>
-    <t>• สรุปข่าวเกมใหม่แบบสั้นง่าย ทันเหตุการณ์
+    <t xml:space="preserve">• สรุปข่าวเกมใหม่แบบสั้นง่าย ทันเหตุการณ์
 • รีวิวจากที่เล่นจริง บอกจุดดีจุดด้อยให้คนอ่าน
 • เจาะลึกสูตร คอมโบ และเทคนิคเฉพาะทางเกมต่อสู้</t>
   </si>
@@ -1383,7 +1380,7 @@
     <t>Website</t>
   </si>
   <si>
-    <t>Freshy Golf
+    <t xml:space="preserve">Freshy Golf
 Wicked Monster Blast
 Wicked Monster Type
 Crazy Strike Bowling</t>
@@ -1828,33 +1825,41 @@
   </si>
   <si>
     <t>Python, openpyxl, pandas, Jinja2, HTML, CSS</t>
-  </si>
-  <si>
-    <t>Lumen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F5597"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1862,18 +1867,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1E3A6E"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2206,46 +2226,57 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="4" width="60" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="9" width="60" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="11" width="25" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2255,7 +2286,7 @@
       <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" t="s">
@@ -2270,7 +2301,7 @@
       <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="J2" t="s">
@@ -2281,74 +2312,81 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:K2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="7" width="55" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B2" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C2" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D2" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F2" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G2" t="s">
         <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
@@ -2357,30 +2395,30 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B3" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F3" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="G3" t="s">
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="I3" t="s">
         <v>15</v>
@@ -2390,36 +2428,41 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:J3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -2436,7 +2479,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -2453,7 +2496,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -2470,7 +2513,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -2487,7 +2530,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -2504,7 +2547,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -2521,7 +2564,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -2538,7 +2581,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -2556,77 +2599,76 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:E9" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:XFD45"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.75" customWidth="1"/>
-    <col min="2" max="2" width="17.375" customWidth="1"/>
-    <col min="3" max="4" width="9" customWidth="1"/>
-    <col min="5" max="5" width="41.75" customWidth="1"/>
-    <col min="6" max="6" width="25.375" customWidth="1"/>
-    <col min="7" max="7" width="9" customWidth="1"/>
-    <col min="8" max="8" width="8.5" customWidth="1"/>
-    <col min="9" max="11" width="9" customWidth="1"/>
-    <col min="12" max="12" width="39.875" customWidth="1"/>
-    <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="8.625" customWidth="1"/>
-    <col min="15" max="16384" width="9" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="6" width="55" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="11" max="11" width="32" customWidth="1"/>
+    <col min="12" max="13" width="55" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="16384" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:16384" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>64</v>
       </c>
@@ -2642,7 +2684,7 @@
       <c r="E2" t="s">
         <v>68</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="G2" t="s">
@@ -2663,14 +2705,14 @@
       <c r="L2" t="s">
         <v>73</v>
       </c>
-      <c r="M2" t="s">
+      <c r="M2" s="2" t="s">
         <v>74</v>
       </c>
       <c r="N2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="220.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -2686,7 +2728,7 @@
       <c r="E3" t="s">
         <v>80</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="2" t="s">
         <v>81</v>
       </c>
       <c r="G3" t="s">
@@ -2707,14 +2749,14 @@
       <c r="L3" t="s">
         <v>83</v>
       </c>
-      <c r="M3" t="s">
+      <c r="M3" s="2" t="s">
         <v>84</v>
       </c>
       <c r="N3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="189" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -2730,7 +2772,7 @@
       <c r="E4" t="s">
         <v>88</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>89</v>
       </c>
       <c r="G4" t="s">
@@ -2751,14 +2793,14 @@
       <c r="L4" t="s">
         <v>91</v>
       </c>
-      <c r="M4" t="s">
+      <c r="M4" s="2" t="s">
         <v>92</v>
       </c>
       <c r="N4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -2774,7 +2816,7 @@
       <c r="E5" t="s">
         <v>95</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="2" t="s">
         <v>96</v>
       </c>
       <c r="G5" t="s">
@@ -2795,14 +2837,14 @@
       <c r="L5" t="s">
         <v>98</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="2" t="s">
         <v>99</v>
       </c>
       <c r="N5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="252" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="252" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -2818,7 +2860,7 @@
       <c r="E6" t="s">
         <v>103</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="2" t="s">
         <v>104</v>
       </c>
       <c r="G6" t="s">
@@ -2839,14 +2881,14 @@
       <c r="L6" t="s">
         <v>106</v>
       </c>
-      <c r="M6" t="s">
+      <c r="M6" s="2" t="s">
         <v>107</v>
       </c>
       <c r="N6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>108</v>
       </c>
@@ -2862,7 +2904,7 @@
       <c r="E7" t="s">
         <v>112</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="2" t="s">
         <v>113</v>
       </c>
       <c r="G7" t="s">
@@ -2883,14 +2925,14 @@
       <c r="L7" t="s">
         <v>117</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="2" t="s">
         <v>118</v>
       </c>
       <c r="N7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>120</v>
       </c>
@@ -2906,7 +2948,7 @@
       <c r="E8" t="s">
         <v>124</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="2" t="s">
         <v>125</v>
       </c>
       <c r="G8" t="s">
@@ -2927,14 +2969,14 @@
       <c r="L8" t="s">
         <v>128</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="2" t="s">
         <v>129</v>
       </c>
       <c r="N8" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="267.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="267.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>130</v>
       </c>
@@ -2950,7 +2992,7 @@
       <c r="E9" t="s">
         <v>133</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>134</v>
       </c>
       <c r="G9" t="s">
@@ -2971,14 +3013,14 @@
       <c r="L9" t="s">
         <v>136</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="2" t="s">
         <v>137</v>
       </c>
       <c r="N9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="189" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>138</v>
       </c>
@@ -2994,7 +3036,7 @@
       <c r="E10" t="s">
         <v>141</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>142</v>
       </c>
       <c r="G10" t="s">
@@ -3015,14 +3057,14 @@
       <c r="L10" t="s">
         <v>143</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="2" t="s">
         <v>144</v>
       </c>
       <c r="N10" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="189" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="189" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>145</v>
       </c>
@@ -3038,7 +3080,7 @@
       <c r="E11" t="s">
         <v>147</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>142</v>
       </c>
       <c r="G11" t="s">
@@ -3059,14 +3101,14 @@
       <c r="L11" t="s">
         <v>148</v>
       </c>
-      <c r="M11" t="s">
+      <c r="M11" s="2" t="s">
         <v>144</v>
       </c>
       <c r="N11" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="393.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="393.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>149</v>
       </c>
@@ -3082,7 +3124,7 @@
       <c r="E12" t="s">
         <v>152</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2" t="s">
         <v>153</v>
       </c>
       <c r="G12" t="s">
@@ -3103,14 +3145,14 @@
       <c r="L12" t="s">
         <v>155</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M12" s="2" t="s">
         <v>156</v>
       </c>
       <c r="N12" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="393.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="393.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>157</v>
       </c>
@@ -3123,10 +3165,10 @@
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>153</v>
       </c>
       <c r="G13" t="s">
@@ -3136,7 +3178,7 @@
         <v>15</v>
       </c>
       <c r="I13" t="s">
-        <v>546</v>
+        <v>160</v>
       </c>
       <c r="J13" t="s">
         <v>15</v>
@@ -3145,241 +3187,241 @@
         <v>158</v>
       </c>
       <c r="L13" t="s">
-        <v>160</v>
-      </c>
-      <c r="M13" t="s">
+        <v>161</v>
+      </c>
+      <c r="M13" s="2" t="s">
         <v>156</v>
       </c>
       <c r="N13" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="173.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="173.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C14" t="s">
         <v>15</v>
       </c>
       <c r="D14" t="s">
+        <v>164</v>
+      </c>
+      <c r="E14" t="s">
+        <v>165</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" t="s">
+        <v>167</v>
+      </c>
+      <c r="J14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K14" t="s">
         <v>163</v>
       </c>
-      <c r="E14" t="s">
-        <v>164</v>
-      </c>
-      <c r="F14" t="s">
-        <v>165</v>
-      </c>
-      <c r="G14" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" t="s">
-        <v>166</v>
-      </c>
-      <c r="J14" t="s">
-        <v>15</v>
-      </c>
-      <c r="K14" t="s">
-        <v>162</v>
-      </c>
       <c r="L14" t="s">
-        <v>167</v>
-      </c>
-      <c r="M14" t="s">
         <v>168</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>169</v>
       </c>
       <c r="N14" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="330.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="330.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C15" t="s">
         <v>15</v>
       </c>
       <c r="D15" t="s">
+        <v>172</v>
+      </c>
+      <c r="E15" t="s">
+        <v>173</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>175</v>
+      </c>
+      <c r="J15" t="s">
+        <v>15</v>
+      </c>
+      <c r="K15" t="s">
         <v>171</v>
       </c>
-      <c r="E15" t="s">
-        <v>172</v>
-      </c>
-      <c r="F15" t="s">
-        <v>173</v>
-      </c>
-      <c r="G15" t="s">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" t="s">
-        <v>174</v>
-      </c>
-      <c r="J15" t="s">
-        <v>15</v>
-      </c>
-      <c r="K15" t="s">
-        <v>170</v>
-      </c>
       <c r="L15" t="s">
-        <v>175</v>
-      </c>
-      <c r="M15" t="s">
         <v>176</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>177</v>
       </c>
       <c r="N15" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="378" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="378" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B16" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
       </c>
       <c r="D16" t="s">
+        <v>180</v>
+      </c>
+      <c r="E16" t="s">
+        <v>181</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" t="s">
+        <v>183</v>
+      </c>
+      <c r="J16" t="s">
+        <v>15</v>
+      </c>
+      <c r="K16" t="s">
         <v>179</v>
       </c>
-      <c r="E16" t="s">
-        <v>180</v>
-      </c>
-      <c r="F16" t="s">
-        <v>181</v>
-      </c>
-      <c r="G16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s">
-        <v>15</v>
-      </c>
-      <c r="I16" t="s">
-        <v>182</v>
-      </c>
-      <c r="J16" t="s">
-        <v>15</v>
-      </c>
-      <c r="K16" t="s">
-        <v>178</v>
-      </c>
       <c r="L16" t="s">
-        <v>183</v>
-      </c>
-      <c r="M16" t="s">
         <v>184</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>185</v>
       </c>
       <c r="N16" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="378" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="378" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C17" t="s">
         <v>15</v>
       </c>
       <c r="D17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E17" t="s">
+        <v>189</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" t="s">
+        <v>191</v>
+      </c>
+      <c r="J17" t="s">
+        <v>15</v>
+      </c>
+      <c r="K17" t="s">
         <v>187</v>
       </c>
-      <c r="E17" t="s">
-        <v>188</v>
-      </c>
-      <c r="F17" t="s">
-        <v>189</v>
-      </c>
-      <c r="G17" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" t="s">
-        <v>190</v>
-      </c>
-      <c r="J17" t="s">
-        <v>15</v>
-      </c>
-      <c r="K17" t="s">
-        <v>186</v>
-      </c>
       <c r="L17" t="s">
-        <v>191</v>
-      </c>
-      <c r="M17" t="s">
         <v>192</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>193</v>
       </c>
       <c r="N17" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="110.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C18" t="s">
         <v>15</v>
       </c>
       <c r="D18" t="s">
+        <v>196</v>
+      </c>
+      <c r="E18" t="s">
+        <v>197</v>
+      </c>
+      <c r="F18" t="s">
+        <v>198</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" t="s">
+        <v>199</v>
+      </c>
+      <c r="J18" t="s">
+        <v>15</v>
+      </c>
+      <c r="K18" t="s">
         <v>195</v>
       </c>
-      <c r="E18" t="s">
-        <v>196</v>
-      </c>
-      <c r="F18" t="s">
-        <v>197</v>
-      </c>
-      <c r="G18" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s">
-        <v>15</v>
-      </c>
-      <c r="I18" t="s">
-        <v>198</v>
-      </c>
-      <c r="J18" t="s">
-        <v>15</v>
-      </c>
-      <c r="K18" t="s">
-        <v>194</v>
-      </c>
       <c r="L18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N18" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="409.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C19" t="s">
         <v>15</v>
@@ -3388,42 +3430,42 @@
         <v>15</v>
       </c>
       <c r="E19" t="s">
+        <v>204</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" t="s">
+        <v>206</v>
+      </c>
+      <c r="J19" t="s">
+        <v>15</v>
+      </c>
+      <c r="K19" t="s">
         <v>203</v>
       </c>
-      <c r="F19" t="s">
-        <v>204</v>
-      </c>
-      <c r="G19" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s">
-        <v>15</v>
-      </c>
-      <c r="I19" t="s">
-        <v>205</v>
-      </c>
-      <c r="J19" t="s">
-        <v>15</v>
-      </c>
-      <c r="K19" t="s">
-        <v>202</v>
-      </c>
       <c r="L19" t="s">
-        <v>206</v>
-      </c>
-      <c r="M19" t="s">
         <v>207</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>208</v>
       </c>
       <c r="N19" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="409.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B20" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C20" t="s">
         <v>15</v>
@@ -3432,42 +3474,42 @@
         <v>15</v>
       </c>
       <c r="E20" t="s">
+        <v>211</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" t="s">
+        <v>213</v>
+      </c>
+      <c r="J20" t="s">
+        <v>15</v>
+      </c>
+      <c r="K20" t="s">
         <v>210</v>
       </c>
-      <c r="F20" t="s">
-        <v>211</v>
-      </c>
-      <c r="G20" t="s">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s">
-        <v>15</v>
-      </c>
-      <c r="I20" t="s">
-        <v>212</v>
-      </c>
-      <c r="J20" t="s">
-        <v>15</v>
-      </c>
-      <c r="K20" t="s">
-        <v>209</v>
-      </c>
       <c r="L20" t="s">
-        <v>213</v>
-      </c>
-      <c r="M20" t="s">
         <v>214</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>215</v>
       </c>
       <c r="N20" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B21" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C21" t="s">
         <v>15</v>
@@ -3476,878 +3518,878 @@
         <v>15</v>
       </c>
       <c r="E21" t="s">
+        <v>218</v>
+      </c>
+      <c r="F21" t="s">
+        <v>219</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+      <c r="H21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" t="s">
+        <v>220</v>
+      </c>
+      <c r="J21" t="s">
+        <v>15</v>
+      </c>
+      <c r="K21" t="s">
         <v>217</v>
       </c>
-      <c r="F21" t="s">
-        <v>218</v>
-      </c>
-      <c r="G21" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" t="s">
-        <v>15</v>
-      </c>
-      <c r="I21" t="s">
-        <v>219</v>
-      </c>
-      <c r="J21" t="s">
-        <v>15</v>
-      </c>
-      <c r="K21" t="s">
-        <v>216</v>
-      </c>
       <c r="L21" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="M21" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="N21" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>223</v>
+      </c>
+      <c r="B22" t="s">
+        <v>224</v>
+      </c>
+      <c r="C22" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" t="s">
+        <v>225</v>
+      </c>
+      <c r="F22" t="s">
+        <v>219</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+      <c r="H22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" t="s">
+        <v>226</v>
+      </c>
+      <c r="J22" t="s">
+        <v>15</v>
+      </c>
+      <c r="K22" t="s">
+        <v>224</v>
+      </c>
+      <c r="L22" t="s">
+        <v>227</v>
+      </c>
+      <c r="M22" t="s">
         <v>222</v>
-      </c>
-      <c r="B22" t="s">
-        <v>223</v>
-      </c>
-      <c r="C22" t="s">
-        <v>15</v>
-      </c>
-      <c r="D22" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" t="s">
-        <v>224</v>
-      </c>
-      <c r="F22" t="s">
-        <v>218</v>
-      </c>
-      <c r="G22" t="s">
-        <v>15</v>
-      </c>
-      <c r="H22" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" t="s">
-        <v>225</v>
-      </c>
-      <c r="J22" t="s">
-        <v>15</v>
-      </c>
-      <c r="K22" t="s">
-        <v>223</v>
-      </c>
-      <c r="L22" t="s">
-        <v>226</v>
-      </c>
-      <c r="M22" t="s">
-        <v>221</v>
       </c>
       <c r="N22" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="252" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" ht="252" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B23" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C23" t="s">
         <v>15</v>
       </c>
       <c r="D23" t="s">
+        <v>230</v>
+      </c>
+      <c r="E23" t="s">
+        <v>231</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" t="s">
+        <v>233</v>
+      </c>
+      <c r="J23" t="s">
+        <v>15</v>
+      </c>
+      <c r="K23" t="s">
         <v>229</v>
       </c>
-      <c r="E23" t="s">
-        <v>230</v>
-      </c>
-      <c r="F23" t="s">
-        <v>231</v>
-      </c>
-      <c r="G23" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I23" t="s">
-        <v>232</v>
-      </c>
-      <c r="J23" t="s">
-        <v>15</v>
-      </c>
-      <c r="K23" t="s">
-        <v>228</v>
-      </c>
       <c r="L23" t="s">
-        <v>233</v>
-      </c>
-      <c r="M23" t="s">
         <v>234</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>235</v>
       </c>
       <c r="N23" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="330.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" ht="330.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B24" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C24" t="s">
         <v>15</v>
       </c>
       <c r="D24" t="s">
+        <v>238</v>
+      </c>
+      <c r="E24" t="s">
+        <v>239</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" t="s">
+        <v>241</v>
+      </c>
+      <c r="J24" t="s">
+        <v>15</v>
+      </c>
+      <c r="K24" t="s">
         <v>237</v>
       </c>
-      <c r="E24" t="s">
-        <v>238</v>
-      </c>
-      <c r="F24" t="s">
-        <v>239</v>
-      </c>
-      <c r="G24" t="s">
-        <v>15</v>
-      </c>
-      <c r="H24" t="s">
-        <v>15</v>
-      </c>
-      <c r="I24" t="s">
-        <v>240</v>
-      </c>
-      <c r="J24" t="s">
-        <v>15</v>
-      </c>
-      <c r="K24" t="s">
-        <v>236</v>
-      </c>
       <c r="L24" t="s">
-        <v>241</v>
-      </c>
-      <c r="M24" t="s">
         <v>242</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>243</v>
       </c>
       <c r="N24" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B25" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C25" t="s">
         <v>15</v>
       </c>
       <c r="D25" t="s">
+        <v>246</v>
+      </c>
+      <c r="E25" t="s">
+        <v>247</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" t="s">
+        <v>15</v>
+      </c>
+      <c r="I25" t="s">
+        <v>249</v>
+      </c>
+      <c r="J25" t="s">
+        <v>15</v>
+      </c>
+      <c r="K25" t="s">
         <v>245</v>
       </c>
-      <c r="E25" t="s">
-        <v>246</v>
-      </c>
-      <c r="F25" t="s">
-        <v>247</v>
-      </c>
-      <c r="G25" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" t="s">
-        <v>15</v>
-      </c>
-      <c r="I25" t="s">
-        <v>248</v>
-      </c>
-      <c r="J25" t="s">
-        <v>15</v>
-      </c>
-      <c r="K25" t="s">
-        <v>244</v>
-      </c>
       <c r="L25" t="s">
-        <v>249</v>
-      </c>
-      <c r="M25" t="s">
         <v>250</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>251</v>
       </c>
       <c r="N25" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B26" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C26" t="s">
         <v>15</v>
       </c>
       <c r="D26" t="s">
+        <v>254</v>
+      </c>
+      <c r="E26" t="s">
+        <v>255</v>
+      </c>
+      <c r="F26" t="s">
+        <v>256</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+      <c r="H26" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" t="s">
+        <v>257</v>
+      </c>
+      <c r="J26" t="s">
+        <v>15</v>
+      </c>
+      <c r="K26" t="s">
         <v>253</v>
       </c>
-      <c r="E26" t="s">
-        <v>254</v>
-      </c>
-      <c r="F26" t="s">
-        <v>255</v>
-      </c>
-      <c r="G26" t="s">
-        <v>15</v>
-      </c>
-      <c r="H26" t="s">
-        <v>15</v>
-      </c>
-      <c r="I26" t="s">
-        <v>256</v>
-      </c>
-      <c r="J26" t="s">
-        <v>15</v>
-      </c>
-      <c r="K26" t="s">
-        <v>252</v>
-      </c>
       <c r="L26" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="M26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="N26" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" ht="47.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>260</v>
+      </c>
+      <c r="B27" t="s">
+        <v>261</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" t="s">
+        <v>262</v>
+      </c>
+      <c r="E27" t="s">
+        <v>263</v>
+      </c>
+      <c r="F27" t="s">
+        <v>256</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+      <c r="H27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I27" t="s">
+        <v>264</v>
+      </c>
+      <c r="J27" t="s">
+        <v>15</v>
+      </c>
+      <c r="K27" t="s">
+        <v>261</v>
+      </c>
+      <c r="L27" t="s">
+        <v>265</v>
+      </c>
+      <c r="M27" t="s">
         <v>259</v>
-      </c>
-      <c r="B27" t="s">
-        <v>260</v>
-      </c>
-      <c r="C27" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" t="s">
-        <v>261</v>
-      </c>
-      <c r="E27" t="s">
-        <v>262</v>
-      </c>
-      <c r="F27" t="s">
-        <v>255</v>
-      </c>
-      <c r="G27" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" t="s">
-        <v>15</v>
-      </c>
-      <c r="I27" t="s">
-        <v>263</v>
-      </c>
-      <c r="J27" t="s">
-        <v>15</v>
-      </c>
-      <c r="K27" t="s">
-        <v>260</v>
-      </c>
-      <c r="L27" t="s">
-        <v>264</v>
-      </c>
-      <c r="M27" t="s">
-        <v>258</v>
       </c>
       <c r="N27" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="126" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" ht="126" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B28" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C28" t="s">
         <v>15</v>
       </c>
       <c r="D28" t="s">
+        <v>268</v>
+      </c>
+      <c r="E28" t="s">
+        <v>269</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+      <c r="H28" t="s">
+        <v>15</v>
+      </c>
+      <c r="I28" t="s">
+        <v>271</v>
+      </c>
+      <c r="J28" t="s">
+        <v>15</v>
+      </c>
+      <c r="K28" t="s">
         <v>267</v>
       </c>
-      <c r="E28" t="s">
-        <v>268</v>
-      </c>
-      <c r="F28" t="s">
-        <v>269</v>
-      </c>
-      <c r="G28" t="s">
-        <v>15</v>
-      </c>
-      <c r="H28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I28" t="s">
-        <v>270</v>
-      </c>
-      <c r="J28" t="s">
-        <v>15</v>
-      </c>
-      <c r="K28" t="s">
-        <v>266</v>
-      </c>
       <c r="L28" t="s">
-        <v>271</v>
-      </c>
-      <c r="M28" t="s">
         <v>272</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>273</v>
       </c>
       <c r="N28" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B29" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C29" t="s">
         <v>15</v>
       </c>
       <c r="D29" t="s">
+        <v>276</v>
+      </c>
+      <c r="E29" t="s">
+        <v>277</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+      <c r="H29" t="s">
+        <v>15</v>
+      </c>
+      <c r="I29" t="s">
+        <v>279</v>
+      </c>
+      <c r="J29" t="s">
+        <v>15</v>
+      </c>
+      <c r="K29" t="s">
         <v>275</v>
       </c>
-      <c r="E29" t="s">
-        <v>276</v>
-      </c>
-      <c r="F29" t="s">
-        <v>277</v>
-      </c>
-      <c r="G29" t="s">
-        <v>15</v>
-      </c>
-      <c r="H29" t="s">
-        <v>15</v>
-      </c>
-      <c r="I29" t="s">
-        <v>278</v>
-      </c>
-      <c r="J29" t="s">
-        <v>15</v>
-      </c>
-      <c r="K29" t="s">
-        <v>274</v>
-      </c>
       <c r="L29" t="s">
-        <v>279</v>
-      </c>
-      <c r="M29" t="s">
         <v>280</v>
+      </c>
+      <c r="M29" s="2" t="s">
+        <v>281</v>
       </c>
       <c r="N29" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C30" t="s">
         <v>15</v>
       </c>
       <c r="D30" t="s">
+        <v>284</v>
+      </c>
+      <c r="E30" t="s">
+        <v>285</v>
+      </c>
+      <c r="F30" t="s">
+        <v>256</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" t="s">
+        <v>15</v>
+      </c>
+      <c r="I30" t="s">
+        <v>286</v>
+      </c>
+      <c r="J30" t="s">
+        <v>15</v>
+      </c>
+      <c r="K30" t="s">
         <v>283</v>
       </c>
-      <c r="E30" t="s">
-        <v>284</v>
-      </c>
-      <c r="F30" t="s">
-        <v>255</v>
-      </c>
-      <c r="G30" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" t="s">
-        <v>15</v>
-      </c>
-      <c r="I30" t="s">
-        <v>285</v>
-      </c>
-      <c r="J30" t="s">
-        <v>15</v>
-      </c>
-      <c r="K30" t="s">
-        <v>282</v>
-      </c>
       <c r="L30" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="M30" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="N30" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B31" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C31" t="s">
         <v>15</v>
       </c>
       <c r="D31" t="s">
+        <v>290</v>
+      </c>
+      <c r="E31" t="s">
+        <v>291</v>
+      </c>
+      <c r="F31" t="s">
+        <v>292</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" t="s">
+        <v>15</v>
+      </c>
+      <c r="I31" t="s">
+        <v>293</v>
+      </c>
+      <c r="J31" t="s">
+        <v>15</v>
+      </c>
+      <c r="K31" t="s">
         <v>289</v>
       </c>
-      <c r="E31" t="s">
-        <v>290</v>
-      </c>
-      <c r="F31" t="s">
-        <v>291</v>
-      </c>
-      <c r="G31" t="s">
-        <v>15</v>
-      </c>
-      <c r="H31" t="s">
-        <v>15</v>
-      </c>
-      <c r="I31" t="s">
-        <v>292</v>
-      </c>
-      <c r="J31" t="s">
-        <v>15</v>
-      </c>
-      <c r="K31" t="s">
-        <v>288</v>
-      </c>
       <c r="L31" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="M31" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="N31" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="393.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" ht="393.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B32" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C32" t="s">
         <v>15</v>
       </c>
       <c r="D32" t="s">
+        <v>298</v>
+      </c>
+      <c r="E32" t="s">
+        <v>299</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" t="s">
+        <v>15</v>
+      </c>
+      <c r="I32" t="s">
+        <v>301</v>
+      </c>
+      <c r="J32" t="s">
+        <v>15</v>
+      </c>
+      <c r="K32" t="s">
         <v>297</v>
       </c>
-      <c r="E32" t="s">
-        <v>298</v>
-      </c>
-      <c r="F32" t="s">
-        <v>299</v>
-      </c>
-      <c r="G32" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" t="s">
-        <v>15</v>
-      </c>
-      <c r="I32" t="s">
-        <v>300</v>
-      </c>
-      <c r="J32" t="s">
-        <v>15</v>
-      </c>
-      <c r="K32" t="s">
-        <v>296</v>
-      </c>
       <c r="L32" t="s">
-        <v>301</v>
-      </c>
-      <c r="M32" t="s">
         <v>302</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>303</v>
       </c>
       <c r="N32" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B33" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C33" t="s">
         <v>15</v>
       </c>
       <c r="D33" t="s">
+        <v>306</v>
+      </c>
+      <c r="E33" t="s">
+        <v>307</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="G33" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" t="s">
+        <v>15</v>
+      </c>
+      <c r="I33" t="s">
+        <v>309</v>
+      </c>
+      <c r="J33" t="s">
+        <v>15</v>
+      </c>
+      <c r="K33" t="s">
         <v>305</v>
       </c>
-      <c r="E33" t="s">
-        <v>306</v>
-      </c>
-      <c r="F33" t="s">
-        <v>307</v>
-      </c>
-      <c r="G33" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" t="s">
-        <v>308</v>
-      </c>
-      <c r="J33" t="s">
-        <v>15</v>
-      </c>
-      <c r="K33" t="s">
-        <v>304</v>
-      </c>
       <c r="L33" t="s">
-        <v>309</v>
-      </c>
-      <c r="M33" t="s">
         <v>310</v>
+      </c>
+      <c r="M33" s="2" t="s">
+        <v>311</v>
       </c>
       <c r="N33" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" ht="220.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B34" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C34" t="s">
         <v>15</v>
       </c>
       <c r="D34" t="s">
+        <v>314</v>
+      </c>
+      <c r="E34" t="s">
+        <v>315</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+      <c r="H34" t="s">
+        <v>15</v>
+      </c>
+      <c r="I34" t="s">
+        <v>309</v>
+      </c>
+      <c r="J34" t="s">
+        <v>15</v>
+      </c>
+      <c r="K34" t="s">
         <v>313</v>
       </c>
-      <c r="E34" t="s">
-        <v>314</v>
-      </c>
-      <c r="F34" t="s">
-        <v>315</v>
-      </c>
-      <c r="G34" t="s">
-        <v>15</v>
-      </c>
-      <c r="H34" t="s">
-        <v>15</v>
-      </c>
-      <c r="I34" t="s">
-        <v>308</v>
-      </c>
-      <c r="J34" t="s">
-        <v>15</v>
-      </c>
-      <c r="K34" t="s">
-        <v>312</v>
-      </c>
       <c r="L34" t="s">
-        <v>316</v>
-      </c>
-      <c r="M34" t="s">
         <v>317</v>
+      </c>
+      <c r="M34" s="2" t="s">
+        <v>318</v>
       </c>
       <c r="N34" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" ht="78.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B35" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C35" t="s">
         <v>15</v>
       </c>
       <c r="D35" t="s">
+        <v>321</v>
+      </c>
+      <c r="E35" t="s">
+        <v>322</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" t="s">
+        <v>15</v>
+      </c>
+      <c r="I35" t="s">
+        <v>324</v>
+      </c>
+      <c r="J35" t="s">
+        <v>15</v>
+      </c>
+      <c r="K35" t="s">
         <v>320</v>
       </c>
-      <c r="E35" t="s">
-        <v>321</v>
-      </c>
-      <c r="F35" t="s">
-        <v>322</v>
-      </c>
-      <c r="G35" t="s">
-        <v>15</v>
-      </c>
-      <c r="H35" t="s">
-        <v>15</v>
-      </c>
-      <c r="I35" t="s">
-        <v>323</v>
-      </c>
-      <c r="J35" t="s">
-        <v>15</v>
-      </c>
-      <c r="K35" t="s">
-        <v>319</v>
-      </c>
       <c r="L35" t="s">
-        <v>324</v>
-      </c>
-      <c r="M35" t="s">
         <v>325</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>326</v>
       </c>
       <c r="N35" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="204.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" ht="204.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B36" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C36" t="s">
         <v>15</v>
       </c>
       <c r="D36" t="s">
+        <v>329</v>
+      </c>
+      <c r="E36" t="s">
+        <v>330</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" t="s">
+        <v>15</v>
+      </c>
+      <c r="I36" t="s">
+        <v>332</v>
+      </c>
+      <c r="J36" t="s">
+        <v>15</v>
+      </c>
+      <c r="K36" t="s">
         <v>328</v>
       </c>
-      <c r="E36" t="s">
-        <v>329</v>
-      </c>
-      <c r="F36" t="s">
-        <v>330</v>
-      </c>
-      <c r="G36" t="s">
-        <v>15</v>
-      </c>
-      <c r="H36" t="s">
-        <v>15</v>
-      </c>
-      <c r="I36" t="s">
-        <v>331</v>
-      </c>
-      <c r="J36" t="s">
-        <v>15</v>
-      </c>
-      <c r="K36" t="s">
-        <v>327</v>
-      </c>
       <c r="L36" t="s">
-        <v>332</v>
-      </c>
-      <c r="M36" t="s">
         <v>333</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>334</v>
       </c>
       <c r="N36" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="204.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" ht="204.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B37" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C37" t="s">
         <v>15</v>
       </c>
       <c r="D37" t="s">
+        <v>337</v>
+      </c>
+      <c r="E37" t="s">
+        <v>338</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+      <c r="H37" t="s">
+        <v>15</v>
+      </c>
+      <c r="I37" t="s">
+        <v>340</v>
+      </c>
+      <c r="J37" t="s">
+        <v>15</v>
+      </c>
+      <c r="K37" t="s">
         <v>336</v>
       </c>
-      <c r="E37" t="s">
-        <v>337</v>
-      </c>
-      <c r="F37" t="s">
-        <v>338</v>
-      </c>
-      <c r="G37" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" t="s">
-        <v>15</v>
-      </c>
-      <c r="I37" t="s">
-        <v>339</v>
-      </c>
-      <c r="J37" t="s">
-        <v>15</v>
-      </c>
-      <c r="K37" t="s">
-        <v>335</v>
-      </c>
       <c r="L37" t="s">
-        <v>340</v>
-      </c>
-      <c r="M37" t="s">
         <v>341</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>342</v>
       </c>
       <c r="N37" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B38" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C38" t="s">
         <v>15</v>
       </c>
       <c r="D38" t="s">
+        <v>345</v>
+      </c>
+      <c r="E38" t="s">
+        <v>346</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+      <c r="H38" t="s">
+        <v>15</v>
+      </c>
+      <c r="I38" t="s">
+        <v>348</v>
+      </c>
+      <c r="J38" t="s">
+        <v>15</v>
+      </c>
+      <c r="K38" t="s">
         <v>344</v>
       </c>
-      <c r="E38" t="s">
-        <v>345</v>
-      </c>
-      <c r="F38" t="s">
-        <v>346</v>
-      </c>
-      <c r="G38" t="s">
-        <v>15</v>
-      </c>
-      <c r="H38" t="s">
-        <v>15</v>
-      </c>
-      <c r="I38" t="s">
-        <v>347</v>
-      </c>
-      <c r="J38" t="s">
-        <v>15</v>
-      </c>
-      <c r="K38" t="s">
-        <v>343</v>
-      </c>
       <c r="L38" t="s">
-        <v>348</v>
-      </c>
-      <c r="M38" t="s">
         <v>349</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>350</v>
       </c>
       <c r="N38" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" ht="141.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B39" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C39" t="s">
         <v>15</v>
       </c>
       <c r="D39" t="s">
+        <v>353</v>
+      </c>
+      <c r="E39" t="s">
+        <v>354</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" t="s">
+        <v>15</v>
+      </c>
+      <c r="I39" t="s">
+        <v>356</v>
+      </c>
+      <c r="J39" t="s">
+        <v>15</v>
+      </c>
+      <c r="K39" t="s">
         <v>352</v>
       </c>
-      <c r="E39" t="s">
-        <v>353</v>
-      </c>
-      <c r="F39" t="s">
-        <v>354</v>
-      </c>
-      <c r="G39" t="s">
-        <v>15</v>
-      </c>
-      <c r="H39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I39" t="s">
-        <v>355</v>
-      </c>
-      <c r="J39" t="s">
-        <v>15</v>
-      </c>
-      <c r="K39" t="s">
-        <v>351</v>
-      </c>
       <c r="L39" t="s">
-        <v>356</v>
-      </c>
-      <c r="M39" t="s">
         <v>357</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>358</v>
       </c>
       <c r="N39" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B40" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C40" t="s">
         <v>15</v>
       </c>
       <c r="D40" t="s">
+        <v>361</v>
+      </c>
+      <c r="E40" t="s">
+        <v>362</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" t="s">
+        <v>15</v>
+      </c>
+      <c r="I40" t="s">
+        <v>364</v>
+      </c>
+      <c r="J40" t="s">
+        <v>15</v>
+      </c>
+      <c r="K40" t="s">
         <v>360</v>
       </c>
-      <c r="E40" t="s">
-        <v>361</v>
-      </c>
-      <c r="F40" t="s">
-        <v>362</v>
-      </c>
-      <c r="G40" t="s">
-        <v>15</v>
-      </c>
-      <c r="H40" t="s">
-        <v>15</v>
-      </c>
-      <c r="I40" t="s">
-        <v>363</v>
-      </c>
-      <c r="J40" t="s">
-        <v>15</v>
-      </c>
-      <c r="K40" t="s">
-        <v>359</v>
-      </c>
       <c r="L40" t="s">
-        <v>364</v>
-      </c>
-      <c r="M40" t="s">
         <v>365</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>366</v>
       </c>
       <c r="N40" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" ht="94.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B41" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C41" t="s">
         <v>15</v>
@@ -4356,42 +4398,42 @@
         <v>15</v>
       </c>
       <c r="E41" t="s">
+        <v>369</v>
+      </c>
+      <c r="F41" t="s">
+        <v>370</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+      <c r="H41" t="s">
+        <v>15</v>
+      </c>
+      <c r="I41" t="s">
+        <v>371</v>
+      </c>
+      <c r="J41" t="s">
+        <v>15</v>
+      </c>
+      <c r="K41" t="s">
         <v>368</v>
       </c>
-      <c r="F41" t="s">
-        <v>369</v>
-      </c>
-      <c r="G41" t="s">
-        <v>15</v>
-      </c>
-      <c r="H41" t="s">
-        <v>15</v>
-      </c>
-      <c r="I41" t="s">
+      <c r="L41" t="s">
+        <v>372</v>
+      </c>
+      <c r="M41" t="s">
         <v>370</v>
-      </c>
-      <c r="J41" t="s">
-        <v>15</v>
-      </c>
-      <c r="K41" t="s">
-        <v>367</v>
-      </c>
-      <c r="L41" t="s">
-        <v>371</v>
-      </c>
-      <c r="M41" t="s">
-        <v>369</v>
       </c>
       <c r="N41" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" ht="47.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B42" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C42" t="s">
         <v>15</v>
@@ -4400,895 +4442,914 @@
         <v>15</v>
       </c>
       <c r="E42" t="s">
+        <v>375</v>
+      </c>
+      <c r="F42" t="s">
+        <v>376</v>
+      </c>
+      <c r="G42" t="s">
+        <v>15</v>
+      </c>
+      <c r="H42" t="s">
+        <v>15</v>
+      </c>
+      <c r="I42" t="s">
+        <v>377</v>
+      </c>
+      <c r="J42" t="s">
+        <v>15</v>
+      </c>
+      <c r="K42" t="s">
         <v>374</v>
       </c>
-      <c r="F42" t="s">
-        <v>375</v>
-      </c>
-      <c r="G42" t="s">
-        <v>15</v>
-      </c>
-      <c r="H42" t="s">
-        <v>15</v>
-      </c>
-      <c r="I42" t="s">
-        <v>376</v>
-      </c>
-      <c r="J42" t="s">
-        <v>15</v>
-      </c>
-      <c r="K42" t="s">
-        <v>373</v>
-      </c>
       <c r="L42" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="M42" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="N42" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" ht="141.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B43" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E43" t="s">
-        <v>381</v>
-      </c>
-      <c r="F43" t="s">
         <v>382</v>
       </c>
+      <c r="F43" s="2" t="s">
+        <v>383</v>
+      </c>
       <c r="I43" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="K43" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="L43" t="s">
-        <v>385</v>
-      </c>
-      <c r="M43" t="s">
         <v>386</v>
       </c>
+      <c r="M43" s="2" t="s">
+        <v>387</v>
+      </c>
       <c r="N43" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="44" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>389</v>
+      </c>
+      <c r="B44" t="s">
+        <v>390</v>
+      </c>
+      <c r="E44" t="s">
+        <v>391</v>
+      </c>
+      <c r="F44" t="s">
+        <v>392</v>
+      </c>
+      <c r="I44" t="s">
+        <v>393</v>
+      </c>
+      <c r="K44" t="s">
+        <v>394</v>
+      </c>
+      <c r="L44" t="s">
+        <v>395</v>
+      </c>
+      <c r="M44" t="s">
+        <v>396</v>
+      </c>
+      <c r="N44" t="s">
         <v>388</v>
       </c>
-      <c r="B44" t="s">
-        <v>389</v>
-      </c>
-      <c r="E44" t="s">
-        <v>390</v>
-      </c>
-      <c r="F44" t="s">
-        <v>391</v>
-      </c>
-      <c r="I44" t="s">
-        <v>392</v>
-      </c>
-      <c r="K44" t="s">
-        <v>393</v>
-      </c>
-      <c r="L44" t="s">
-        <v>394</v>
-      </c>
-      <c r="M44" t="s">
-        <v>395</v>
-      </c>
-      <c r="N44" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B45" t="s">
-        <v>397</v>
-      </c>
-      <c r="E45" t="s">
         <v>398</v>
       </c>
+      <c r="E45" s="2" t="s">
+        <v>399</v>
+      </c>
       <c r="F45" t="s">
+        <v>400</v>
+      </c>
+      <c r="I45" t="s">
+        <v>401</v>
+      </c>
+      <c r="K45" t="s">
+        <v>402</v>
+      </c>
+      <c r="L45" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="I45" t="s">
-        <v>400</v>
-      </c>
-      <c r="K45" t="s">
-        <v>401</v>
-      </c>
-      <c r="L45" t="s">
-        <v>398</v>
-      </c>
       <c r="M45" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="N45" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:XFD1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:N12 A14:N45 A13:H13 J13:N13" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="45" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>403</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C1" s="1" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="B2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:D2" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="60" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>410</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C1" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="F1" t="s">
+      <c r="E1" s="1" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C2" t="s">
+        <v>419</v>
+      </c>
+      <c r="D2" t="s">
+        <v>420</v>
+      </c>
+      <c r="E2" t="s">
         <v>418</v>
       </c>
-      <c r="D2" t="s">
-        <v>419</v>
-      </c>
-      <c r="E2" t="s">
-        <v>417</v>
-      </c>
       <c r="F2" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C3" t="s">
+        <v>424</v>
+      </c>
+      <c r="D3" t="s">
+        <v>425</v>
+      </c>
+      <c r="E3" t="s">
         <v>423</v>
       </c>
-      <c r="D3" t="s">
-        <v>424</v>
-      </c>
-      <c r="E3" t="s">
-        <v>422</v>
-      </c>
       <c r="F3" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B4" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C4" t="s">
+        <v>429</v>
+      </c>
+      <c r="D4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E4" t="s">
         <v>428</v>
       </c>
-      <c r="D4" t="s">
-        <v>429</v>
-      </c>
-      <c r="E4" t="s">
-        <v>427</v>
-      </c>
       <c r="F4" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B5" t="s">
+        <v>433</v>
+      </c>
+      <c r="C5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D5" t="s">
+        <v>435</v>
+      </c>
+      <c r="E5" t="s">
+        <v>433</v>
+      </c>
+      <c r="F5" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>432</v>
       </c>
-      <c r="C5" t="s">
-        <v>433</v>
-      </c>
-      <c r="D5" t="s">
-        <v>434</v>
-      </c>
-      <c r="E5" t="s">
-        <v>432</v>
-      </c>
-      <c r="F5" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>431</v>
-      </c>
       <c r="B6" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C6" t="s">
+        <v>438</v>
+      </c>
+      <c r="D6" t="s">
+        <v>439</v>
+      </c>
+      <c r="E6" t="s">
         <v>437</v>
       </c>
-      <c r="D6" t="s">
-        <v>438</v>
-      </c>
-      <c r="E6" t="s">
-        <v>436</v>
-      </c>
       <c r="F6" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B7" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C7" t="s">
+        <v>443</v>
+      </c>
+      <c r="D7" t="s">
+        <v>444</v>
+      </c>
+      <c r="E7" t="s">
         <v>442</v>
       </c>
-      <c r="D7" t="s">
-        <v>443</v>
-      </c>
-      <c r="E7" t="s">
-        <v>441</v>
-      </c>
       <c r="F7" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B8" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C8" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" t="s">
+        <v>449</v>
+      </c>
+      <c r="E8" t="s">
         <v>447</v>
       </c>
-      <c r="D8" t="s">
-        <v>448</v>
-      </c>
-      <c r="E8" t="s">
-        <v>446</v>
-      </c>
       <c r="F8" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:F8" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="55" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>450</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="C1" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C2" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C3" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>458</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
         <v>459</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C2" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B3" t="s">
         <v>462</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>463</v>
-      </c>
-      <c r="B3" t="s">
-        <v>461</v>
-      </c>
       <c r="C3" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B4" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C4" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B5" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
-        <v>470</v>
-      </c>
-      <c r="C1" t="s">
-        <v>459</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="B1" s="1" t="s">
         <v>471</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="B2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D2" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>477</v>
+      </c>
+      <c r="B3" t="s">
+        <v>478</v>
+      </c>
+      <c r="C3" t="s">
+        <v>479</v>
+      </c>
+      <c r="D3" t="s">
         <v>476</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>477</v>
       </c>
-      <c r="C3" t="s">
-        <v>478</v>
-      </c>
-      <c r="D3" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>480</v>
+      </c>
+      <c r="C4" t="s">
+        <v>481</v>
+      </c>
+      <c r="D4" t="s">
         <v>476</v>
       </c>
-      <c r="B4" t="s">
-        <v>479</v>
-      </c>
-      <c r="C4" t="s">
-        <v>480</v>
-      </c>
-      <c r="D4" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="B5" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:D5" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>482</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B2" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B3" t="s">
         <v>485</v>
       </c>
-      <c r="B3" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="B4" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B5" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="B6" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B7" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>492</v>
+      </c>
+      <c r="B8" t="s">
         <v>491</v>
       </c>
-      <c r="B8" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B9" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="B10" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="B11" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B12" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="B15" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B17" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>503</v>
+      </c>
+      <c r="B18" t="s">
         <v>502</v>
       </c>
-      <c r="B18" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="B19" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B20" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>507</v>
+      </c>
+      <c r="B21" t="s">
         <v>506</v>
       </c>
-      <c r="B21" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B22" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B23" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B24" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>512</v>
+      </c>
+      <c r="B25" t="s">
         <v>511</v>
       </c>
-      <c r="B25" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B26" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B27" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B28" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B29" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>518</v>
+      </c>
+      <c r="B30" t="s">
         <v>517</v>
       </c>
-      <c r="B30" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="B31" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="B32" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B33" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>523</v>
+      </c>
+      <c r="B34" t="s">
         <v>522</v>
       </c>
-      <c r="B34" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="B35" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B36" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>527</v>
+      </c>
+      <c r="B37" t="s">
         <v>526</v>
       </c>
-      <c r="B37" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B38" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B39" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B40" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>532</v>
+      </c>
+      <c r="B41" t="s">
         <v>531</v>
       </c>
-      <c r="B41" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B42" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B43" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:B43" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update data, images, and manifest
- data.xlsx: content updates
- Lumen: rename/replace images, add logo.webp
- imaginmebnb: add logo.jpg, remove image58.jpg
- manifest.json: regenerated

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E4A1468-5AA1-4A71-A280-0CF8296820DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Profile" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Skills" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Project" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Contact" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Experience" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Education" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Certifications" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Awards" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Tools" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Playground" state="visible" r:id="rId13"/>
+    <sheet name="Profile" sheetId="1" r:id="rId1"/>
+    <sheet name="Skills" sheetId="2" r:id="rId2"/>
+    <sheet name="Project" sheetId="3" r:id="rId3"/>
+    <sheet name="Contact" sheetId="4" r:id="rId4"/>
+    <sheet name="Experience" sheetId="5" r:id="rId5"/>
+    <sheet name="Education" sheetId="6" r:id="rId6"/>
+    <sheet name="Certifications" sheetId="7" r:id="rId7"/>
+    <sheet name="Awards" sheetId="8" r:id="rId8"/>
+    <sheet name="Tools" sheetId="9" r:id="rId9"/>
+    <sheet name="Playground" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -67,7 +68,7 @@
     <t>QA Lead with 14+ years across game development and software testing. ISTQB CTFL certified, passionate about quality, automation, and growing teams.</t>
   </si>
   <si>
-    <t xml:space="preserve">I have over 10 years of experience in game development across various roles, including Production Manager, and more than 8 years in Quality Assurance with a current focus on software testing. While I am now primarily involved in non-gaming software projects, I maintain a strong passion for the gaming industry and bring a solid understanding of both game production pipelines and modern software development practices, including CI/CD processes.
+    <t>I have over 10 years of experience in game development across various roles, including Production Manager, and more than 8 years in Quality Assurance with a current focus on software testing. While I am now primarily involved in non-gaming software projects, I maintain a strong passion for the gaming industry and bring a solid understanding of both game production pipelines and modern software development practices, including CI/CD processes.
 In addition to my technical expertise, I actively mentor team members and take pride in sharing knowledge to help others grow. I believe in building strong, collaborative teams and creating an environment that supports continuous learning. I have been certified with ISTQB CTFL since 2019 and as an Agile Tester (AT) in 2024.</t>
   </si>
   <si>
@@ -83,7 +84,7 @@
     <t>QA Lead ที่คลุกคลีกับวงการพัฒนาเกมและทดสอบซอฟต์แวร์มากว่า 14 ปี ได้รับการรับรอง ISTQB CTFL ชอบงานที่เกี่ยวกับคุณภาพ ระบบทดสอบอัตโนมัติ และการพาทีมเติบโตไปด้วยกัน</t>
   </si>
   <si>
-    <t xml:space="preserve">ทำงานในวงการเกมมากว่า 10 ปี ผ่านหลายบทบาท รวมถึงตำแหน่ง Production Manager และมีประสบการณ์ด้าน QA อีกกว่า 8 ปี ปัจจุบันโฟกัสที่งานทดสอบซอฟต์แวร์เป็นหลัก แม้จะย้ายมาทำสายซอฟต์แวร์ทั่วไปแล้ว แต่ยังหลงรักวงการเกมอยู่เสมอ และเข้าใจทั้งกระบวนการผลิตเกมและการพัฒนาซอฟต์แวร์สมัยใหม่ รวมถึงงานสาย CI/CD เป็นอย่างดี
+    <t>ทำงานในวงการเกมมากว่า 10 ปี ผ่านหลายบทบาท รวมถึงตำแหน่ง Production Manager และมีประสบการณ์ด้าน QA อีกกว่า 8 ปี ปัจจุบันโฟกัสที่งานทดสอบซอฟต์แวร์เป็นหลัก แม้จะย้ายมาทำสายซอฟต์แวร์ทั่วไปแล้ว แต่ยังหลงรักวงการเกมอยู่เสมอ และเข้าใจทั้งกระบวนการผลิตเกมและการพัฒนาซอฟต์แวร์สมัยใหม่ รวมถึงงานสาย CI/CD เป็นอย่างดี
 นอกจากเรื่องเทคนิคแล้ว ยังชอบทำหน้าที่เป็น Mentor ให้น้องๆ ในทีม และยินดีแบ่งปันความรู้เพื่อให้ทุกคนเก่งขึ้นไปด้วยกัน เชื่อในเรื่องการสร้างทีมที่แข็งแรงและบรรยากาศที่เอื้อให้ทุกคนได้เรียนรู้ตลอดเวลา ได้รับการรับรอง ISTQB CTFL ตั้งแต่ปี 2019 และ Agile Tester (AT) ในปี 2024</t>
   </si>
   <si>
@@ -234,7 +235,7 @@
     <t>Lotus's is a major retail chain in Thailand, formerly known as Tesco Lotus, operating a wide range of store formats including hypermarkets, supermarkets, and convenience stores. Lotus's Web (Lotus's Shop Online) is their official online shopping platform, allowing customers to order groceries and household goods through its website or mobile app.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Manage products and inventory system to meet the requirements
+    <t>• Manage products and inventory system to meet the requirements
 • Manage test plan, design and execute test cases
 • Transfer knowledge and provide documents to team
 • Collaborate supporting between teams and investigate issue and root cause.</t>
@@ -252,7 +253,7 @@
     <t>Lotus's เป็นเชนค้าปลีกรายใหญ่ของไทย เดิมชื่อ Tesco Lotus มีร้านหลายรูปแบบ ทั้งไฮเปอร์มาร์เก็ต ซูเปอร์มาร์เก็ต และร้านสะดวกซื้อ ส่วน Lotus's Web (Lotus's Shop Online) คือแพลตฟอร์มช้อปออนไลน์อย่างเป็นทางการ ให้ลูกค้าสั่งของกินของใช้ผ่านเว็บไซต์หรือแอปได้สะดวกๆ</t>
   </si>
   <si>
-    <t xml:space="preserve">• ดูแลระบบสินค้าและสต็อกให้ตรงตามที่ทีมต้องการ
+    <t>• ดูแลระบบสินค้าและสต็อกให้ตรงตามที่ทีมต้องการ
 • วาง Test Plan ออกแบบและรัน Test Case
 • ถ่ายทอดความรู้และทำเอกสารให้ทีม
 • ประสานงานข้ามทีมและสืบหาต้นตอของปัญหา</t>
@@ -276,7 +277,7 @@
     <t>Manao Meals is a web and mobile application that allows company members to order lunch meals as a company benefit. Admins can assign restaurant details and menus, and employees use the app to order food, adjust add-ons, and submit to admin for processing to the restaurant.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Define test plan, approaches, template and strategy for test coverage
+    <t>• Define test plan, approaches, template and strategy for test coverage
 • Define automation test plan, template and contribute documentation
 • Perform functional test and test case design
 • Communicate between developer, QA and project owner.</t>
@@ -288,7 +289,7 @@
     <t>Manao Meals เป็นเว็บและแอปสำหรับสั่งข้าวกลางวันในออฟฟิศเป็นสวัสดิการพนักงาน แอดมินตั้งร้านและเมนูได้ พนักงานก็เข้าแอปไปสั่ง เลือก add-on แล้วส่งให้แอดมินรวบรวมไปสั่งร้านต่อ</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผน Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม
+    <t>• วางแผน Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม
 • วาง Automation Test Plan พร้อมเทมเพลตและช่วยทำเอกสาร
 • ทำ Functional Test และออกแบบ Test Case
 • ประสานงานระหว่าง Dev, QA และ Project Owner</t>
@@ -306,7 +307,7 @@
     <t>Seller Center is an E-commerce web application and inventory system that allows vendors (sellers) to join and manage their teams, orders, campaigns, and products. It separates into an admin site (managing other admins, sellers, and transactions) and a seller site (managing shop products and order transactions).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Manage and contribute documentation
+    <t>• Manage and contribute documentation
 • Define test plan, approaches, template and strategy for test coverage
 • Perform functional test and test case design
 • Communicate between developer, QA and project owner.</t>
@@ -318,7 +319,7 @@
     <t>Seller Center เป็นเว็บ E-commerce และระบบสต็อกที่ให้ผู้ขาย (Seller) เข้ามาจัดการทีม ออเดอร์ แคมเปญ และสินค้าได้ แบ่งเป็นฝั่ง Admin (จัดการแอดมินอื่น ผู้ขาย และธุรกรรม) กับฝั่ง Seller (จัดการสินค้าในร้านและออเดอร์)</t>
   </si>
   <si>
-    <t xml:space="preserve">• ดูแลและช่วยจัดทำเอกสาร
+    <t>• ดูแลและช่วยจัดทำเอกสาร
 • วาง Test Plan แนวทาง เทมเพลต และกลยุทธ์ให้ครอบคลุม
 • ทำ Functional Test และออกแบบ Test Case
 • ประสานงานระหว่าง Dev, QA และ Project Owner</t>
@@ -333,7 +334,7 @@
     <t>PTT Digital is a finance application for PTT, requiring Quality Assurance standards and DevSecOps processes to ensure secure and reliable transactions.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Contribute documentation for Standard Quality Assurance, covering DevSecOps process with user acceptance criteria
+    <t>• Contribute documentation for Standard Quality Assurance, covering DevSecOps process with user acceptance criteria
 • Communicate between developer, QA and project owner.</t>
   </si>
   <si>
@@ -343,7 +344,7 @@
     <t>PTT Digital เป็นแอปด้านการเงินของ ปตท. ที่ต้องการมาตรฐาน QA และกระบวนการ DevSecOps เพื่อให้ทุกธุรกรรมปลอดภัยและเชื่อถือได้</t>
   </si>
   <si>
-    <t xml:space="preserve">• จัดทำเอกสารมาตรฐาน QA ครอบคลุมกระบวนการ DevSecOps พร้อมเงื่อนไขการรับมอบงานจากผู้ใช้
+    <t>• จัดทำเอกสารมาตรฐาน QA ครอบคลุมกระบวนการ DevSecOps พร้อมเงื่อนไขการรับมอบงานจากผู้ใช้
 • ประสานงานระหว่าง Dev, QA และ Project Owner</t>
   </si>
   <si>
@@ -359,7 +360,7 @@
     <t>True Online Store is an E-commerce website by True Corporation, providing True products and services for customers and True membership.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Test planning, analysis and design to cover business requirements
+    <t>• Test planning, analysis and design to cover business requirements
 • Test case design and execution from day-to-day basis
 • Generate test data and test script for manual and automation testing
 • Perform static and dynamic testing to cover acceptances.</t>
@@ -371,7 +372,7 @@
     <t>True Online Store เป็นเว็บ E-commerce ของ True Corporation ขายสินค้าและบริการของทรู รวมถึงสิทธิประโยชน์สำหรับสมาชิก True</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผน วิเคราะห์ และออกแบบการทดสอบให้ครอบคลุม Business Requirement
+    <t>• วางแผน วิเคราะห์ และออกแบบการทดสอบให้ครอบคลุม Business Requirement
 • ออกแบบและรัน Test Case ในงานประจำวัน
 • เตรียม Test Data และเขียน Test Script ทั้งแบบ Manual และ Automation
 • ทำทั้ง Static และ Dynamic Testing เพื่อให้ผ่านเกณฑ์รับมอบ</t>
@@ -392,7 +393,7 @@
     <t>Linage W is a global scale MMORPG where players fight for their glories, set 150 years after the original Lineage story in the Aden World. Players can pick a story among lord, knight, fairy, and mage to explore a dark fantasy world.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Define test scope, plan, data and documentation to cover test standard
+    <t>• Define test scope, plan, data and documentation to cover test standard
 • Maintenance testing, investigate and analyze issues
 • Playthrough testing as end-user on production environment.</t>
   </si>
@@ -409,7 +410,7 @@
     <t>Lineage W เป็นเกม MMORPG ระดับโลก ซึ่งผู้เล่นต้องต่อสู้เพื่อชื่อเสียงของตัวเอง ดำเนินเรื่องหลังจาก Lineage ภาคแรก 150 ปี ในโลก Aden ผู้เล่นสามารถเลือกเล่นเป็นขุนนาง อัศวิน นางฟ้า หรือพ่อมด เพื่อผจญภัยในโลกแฟนตาซีลึกลับ</t>
   </si>
   <si>
-    <t xml:space="preserve">• กำหนดขอบเขตการทดสอบ Test Plan ข้อมูล และเอกสารให้ตรงตามมาตรฐาน
+    <t>• กำหนดขอบเขตการทดสอบ Test Plan ข้อมูล และเอกสารให้ตรงตามมาตรฐาน
 • ทำ Maintenance Testing ตรวจสอบและวิเคราะห์ปัญหา
 • เล่นจริงในมุมมองผู้ใช้งานบน Production</t>
   </si>
@@ -432,7 +433,7 @@
     <t>The project focused on the 'ALL member' 7-Eleven membership program via the 7App. This program allows users to get discounts, earn coupons, check, redeem, and transfer ALL points, and pay with credit cards via Truemoney Wallet at 7-Eleven stores, 7Delivery service, and All Online.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Supervision and coordinate between teams, developers, internal and external QA
+    <t>• Supervision and coordinate between teams, developers, internal and external QA
 • Test analysis, planning and management
 • Manage QA processes for new campaigns and features for each release
 • Transfer testing tool knowledge to teams.</t>
@@ -447,7 +448,7 @@
     <t>โปรเจกต์นี้เน้นที่ระบบสมาชิก 'ALL Member' ผ่านแอป 7App ผู้ใช้รับส่วนลด เก็บคูปอง เช็ค แลก และโอนคะแนน ALL Point รวมถึงจ่ายผ่านบัตรเครดิตผ่าน TrueMoney Wallet ที่ร้าน 7-Eleven, บริการ 7Delivery และ All Online</t>
   </si>
   <si>
-    <t xml:space="preserve">• ดูแลและประสานงานระหว่างทีม Dev และทีม QA ทั้งภายในและภายนอก
+    <t>• ดูแลและประสานงานระหว่างทีม Dev และทีม QA ทั้งภายในและภายนอก
 • วิเคราะห์ วางแผน และบริหารจัดการงานทดสอบ
 • ดูแลกระบวนการ QA สำหรับแคมเปญและฟีเจอร์ใหม่ในแต่ละ Release
 • ถ่ายทอดความรู้เรื่องเครื่องมือทดสอบให้ทีม</t>
@@ -465,7 +466,7 @@
     <t>Aliveunited is a digital platform that focuses on UI/UX design and system flow for end users, with consultation between project owner and design team.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Test planning, monitoring, analysis and design
+    <t>• Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers
 • Design, UI and UX consultant with Project Owner to analyze the whole system.</t>
@@ -477,7 +478,7 @@
     <t>Aliveunited เป็นแพลตฟอร์มดิจิทัลที่เน้นการออกแบบ UI/UX และ System Flow สำหรับผู้ใช้ ผ่านการปรึกษาระหว่าง Project Owner กับทีมดีไซน์</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
+    <t>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager
 • ให้คำปรึกษาด้าน Design, UI และ UX ร่วมกับ Project Owner เพื่อวิเคราะห์ระบบทั้งหมด</t>
@@ -495,7 +496,7 @@
     <t>The Curaprox App (iOS, Android) is designed to help users stay motivated in their daily dental routines, ensuring preventive dental care year-round. It allows connection with dental professionals and access to lectures, articles, and products.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Test planning, monitoring, analysis and design
+    <t>• Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers.</t>
   </si>
@@ -503,7 +504,7 @@
     <t>แอป Curaprox (iOS, Android) ช่วยสร้างแรงจูงใจในการดูแลสุขภาพฟันประจำวัน เพื่อการดูแลฟันเชิงป้องกันตลอดปี สามารถเชื่อมต่อกับทันตแพทย์ อ่านบทความ และเข้าถึงผลิตภัณฑ์ได้ผ่านแอป</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
+    <t>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับทีม Dev, Tester และ Manager</t>
   </si>
@@ -532,7 +533,7 @@
     <t>Hotel Life: A Resort Simulator is a simulation game where players build and manage their own resort, designing rooms, attractions, and services to attract guests.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Test planning, monitoring, analysis and design
+    <t>• Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers
 • Coordinated developer team to request test tools for game level testing and improve QA processes
@@ -545,7 +546,7 @@
     <t>Hotel Life: A Resort Simulator เป็นเกมแนวสร้างและบริหารรีสอร์ตของตัวเอง ผู้เล่นออกแบบห้องพัก สิ่งอำนวยความสะดวก และสถานที่ท่องเที่ยวต่างๆ เพื่อดึงดูดลูกค้า</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
+    <t>• วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager
 • ประสานกับทีม Dev ขอ Test Tools สำหรับทดสอบ Game Level และปรับปรุงกระบวนการ QA
@@ -558,7 +559,7 @@
     <t>Lumen.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lumen. is a puzzle game on Apple Arcade where players solve levels using lights lenses and mirrors
+    <t>Lumen. is a puzzle game on Apple Arcade where players solve levels using lights lenses and mirrors
   discovering a mysterious antique box.</t>
   </si>
   <si>
@@ -580,7 +581,7 @@
     <t>Pick is a mobile application that connects with hardware devices, allowing users to synchronize and control device functions through the app.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Coordinated with the external production and passed testing criteria to external tester teams
+    <t>• Coordinated with the external production and passed testing criteria to external tester teams
 • Functional, and API testing between software and hardware remotely to ensure app can synchronize as client acceptance.</t>
   </si>
   <si>
@@ -590,7 +591,7 @@
     <t>Pick เป็นแอปมือถือที่เชื่อมต่อกับ Hardware ผู้ใช้สามารถซิงโครไนซ์และควบคุมการทำงานของอุปกรณ์ผ่านแอปได้</t>
   </si>
   <si>
-    <t xml:space="preserve">• ประสานงานกับผู้ผลิตภายนอก และส่งต่อ Test Criteria ให้ทีม Tester ภายนอก
+    <t>• ประสานงานกับผู้ผลิตภายนอก และส่งต่อ Test Criteria ให้ทีม Tester ภายนอก
 • ทำ Functional Test และ API Test ระหว่าง Software กับ Hardware แบบ Remote เพื่อยืนยันว่าแอปซิงโครไนซ์ได้ตามที่ลูกค้าต้องการ</t>
   </si>
   <si>
@@ -606,7 +607,7 @@
     <t>City of Games is an app allowing free play of classic and no-commission baccarat modes, featuring 3D card squeezing, available on iOS, Android, and Chinese Android.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Release control, submit application to Apple and Google stores
+    <t>• Release control, submit application to Apple and Google stores
 • Test planning, monitoring, analysis and design
 • Functional and playthrough testing, collected requirements and passed on information to the tester team
 • Document review, managed test scenarios and coordinated with the developer team, tester team and managers
@@ -619,7 +620,7 @@
     <t>City of Games เป็นแอปที่ให้เล่นบาคาร่าแบบคลาสสิกและไร้ค่าคอมมิชชั่น ฟรี มีระบบเปิดไพ่สามมิติ รองรับทั้ง iOS, Android และ Android ของจีน</t>
   </si>
   <si>
-    <t xml:space="preserve">• ดูแล Release Control และ Submit แอปขึ้น Apple และ Google Store
+    <t>• ดูแล Release Control และ Submit แอปขึ้น Apple และ Google Store
 • วางแผน ติดตาม วิเคราะห์ และออกแบบการทดสอบ
 • ทำ Functional และ Playthrough Testing รวบรวม Requirement ส่งต่อให้ทีม Tester
 • รีวิวเอกสาร จัดการ Test Scenario และประสานกับ Dev, Tester และ Manager
@@ -638,7 +639,7 @@
     <t>Tint. is a mobile and console game available on iOS, MacOS, and TvOS, designed to work with and without peripheral game controllers.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Coordinated with the external production and passed testing criteria and other game information to external tester teams
+    <t>• Coordinated with the external production and passed testing criteria and other game information to external tester teams
 • Functional testing of new features and playthrough testing to ensure the game can progress correctly as expected with new integrated contents
 • Monitoring external teams closely from the regression process to cover client and store acceptance
 • Device coverage testing, to ensure app can work correctly on MacOS, TvOS and iOS devices with and without peripheral game controllers.</t>
@@ -650,7 +651,7 @@
     <t>Tint. เป็นเกมบนมือถือและคอนโซล รองรับทั้ง iOS, MacOS และ tvOS ออกแบบมาให้เล่นได้ทั้งแบบใช้และไม่ใช้ Game Controller เสริม</t>
   </si>
   <si>
-    <t xml:space="preserve">• ประสานงานกับผู้ผลิตภายนอก ส่งต่อ Test Criteria และข้อมูลเกมให้ทีม Tester ภายนอก
+    <t>• ประสานงานกับผู้ผลิตภายนอก ส่งต่อ Test Criteria และข้อมูลเกมให้ทีม Tester ภายนอก
 • Functional Test ฟีเจอร์ใหม่ และ Playthrough เพื่อให้มั่นใจว่าเกมเล่นได้ต่อเนื่องตามที่คาดหวังหลังรวม Content ใหม่
 • ติดตามทีมภายนอกอย่างใกล้ชิดตอนทำ Regression เพื่อรองรับรีควอเรมนต์ของลูกค้าและ Store
 • ทดสอบการรองรับอุปกรณ์ให้แอปทำงานได้บน MacOS, tvOS และ iOS ทั้งแบบใช้และไม่ใช้ Game Controller</t>
@@ -668,7 +669,7 @@
     <t>Panya is a mobile application designed to work reliably across various network conditions, with a focus on stability and performance for end users.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Test planning, gathered new requirements from clients directly and passed on information to the tester team
+    <t>• Test planning, gathered new requirements from clients directly and passed on information to the tester team
 • Test suite control, created, updated, prioritized and defined test cases from test suite for regression testing to reach client acceptance
 • Handled responsibility for test tools, implemented processes for automation to prepare test data, and created technical documents for internal purposes
 • Investigated network link conditions to perform stability testing, making sure the app works to various network status.</t>
@@ -680,7 +681,7 @@
     <t>Panya เป็นแอปมือถือที่ออกแบบมาให้ทำงานได้อย่างเสถียรบนสภาพเครือข่ายที่หลากหลาย มุ่งเน้นความเสถียรและประสิทธิภาพสำหรับผู้ใช้</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผนการทดสอบ รับ Requirement จากลูกค้าโดยตรงและส่งต่อให้ทีม Tester
+    <t>• วางแผนการทดสอบ รับ Requirement จากลูกค้าโดยตรงและส่งต่อให้ทีม Tester
 • จัดการ Test Suite — สร้าง อัปเดต จัดลำดับความสำคัญ และกำหนด Test Case สำหรับ Regression ให้ตรงตามที่ลูกค้ายอมรับ
 • ดูแล Test Tools วางแนวทาง Automation สำหรับจัดเตรียม Test Data พร้อมทำเอกสารทางเทคนิคภายใน
 • ตรวจสภาพเครือข่ายเพื่อทำ Stability Testing ให้มั่นใจว่าแอปทำงานได้ในทุกสภาพเน็ตเวิร์ก</t>
@@ -719,7 +720,7 @@
     <t>ImaginMe Beauty and the Beast is a personalized interactive storybook app where users customize their character to star in the Beauty and the Beast story, featuring mini-games and animated scenes.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
+    <t>• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
 • Art Asset management, designed specification, limitation and performed optimization for device coverage
 • Level designing with Unity to generate mini games and performed own unit, integration and system testing to meet requirements
 • Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing
@@ -732,7 +733,7 @@
     <t>เป็นแอปหนังสือนิทานส่วนตัวที่ผู้ใช้ปรับแต่งตัวละครได้เอง ร่วมผจญภัยในเรื่องโฉมงามกับเจ้าชายอสูร พร้อมมินิเกมและฉากแอนิเมชัน</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
+    <t>• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
 • จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย
 • ทำ Level Design ด้วย Unity สร้าง Mini Game พร้อม Unit, Integration และ System Test ของตัวเองให้ตรงตาม Requirement
 • ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop
@@ -748,7 +749,7 @@
     <t>ImaginMe Dragons is a personalized interactive storybook app where users customize their character to star in a dragon-themed adventure, featuring mini-games with patterns and obstacles.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
+    <t>• Built on client concepts to design control behaviours, character customization, game environment and mini games to meet client acceptance
 • Art Asset management, designed specification, limitation and performed optimization for device coverage
 • Level designing with Unity to generate pattern and obstacles and performed own unit, integration and system testing to meet requirements
 • Functional and playthrough testing with both manual and automation testing to ensure the app can perform proper game loop testing
@@ -761,7 +762,7 @@
     <t>หนังสือนิทานส่วนตัวธีมมังกร ที่ผู้ใช้ปรับแต่งตัวละครได้เอง ร่วมผจญภัยผ่านมินิเกมที่มีรูปแบบและอุปสรรคหลากหลาย</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
+    <t>• ออกแบบ Control, Character Customization, Game Environment และ Mini Game ตามคอนเซ็ปต์ของลูกค้า
 • จัดการ Art Asset ออกแบบ Spec และ Optimize ให้รองรับอุปกรณ์หลากหลาย
 • ทำ Level Design ด้วย Unity สร้างรูปแบบและอุปสรรค พร้อม Unit, Integration และ System Test
 • ทำ Functional และ Playthrough Testing ทั้ง Manual และ Automation รองรับ Game Loop
@@ -816,7 +817,7 @@
     <t>Tesco Lotus Shopping Spree is a promotional infinite running game for Tesco Lotus, designed for low-end mobile devices, where players run through stages to collect items and rewards.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Built on client concepts to design promotional infinite running games to meet client acceptance
+    <t>• Built on client concepts to design promotional infinite running games to meet client acceptance
 • Designed specification, limitation and optimization to cover low end devices
 • Level designing with Unity to generate stage patterns and perform own unit, integration and system testing
 • Handling responsibility for test tools and developing improvement processes.</t>
@@ -828,7 +829,7 @@
     <t>เกมประชาสัมพันธ์แนว Infinite Running ของเทสโก้โลตัส ทำงานได้บนมือถือสเป็กต่ำ ผู้เล่นวิ่งผ่านด่านต่างๆ เพื่อเก็บไอเท็มและรางวัล</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบเกม Promotional Infinite Running ตามคอนเซ็ปต์ของลูกค้า
+    <t>• ออกแบบเกม Promotional Infinite Running ตามคอนเซ็ปต์ของลูกค้า
 • ออกแบบ Spec ข้อจำกัด และ Optimize ให้รองรับมือถือ Spec ต่ำ
 • ทำ Level Design ด้วย Unity สร้าง Stage Pattern พร้อม Unit, Integration และ System Test
 • ดูแล Test Tools และพัฒนาปรับปรุงกระบวนการ</t>
@@ -846,7 +847,7 @@
     <t>Totem Defender is a free-to-play tower defense game for mobile, where players use totems to defend against waves of enemies across multiple stages and difficulty levels.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Project planning, built on client concepts to design games contents from scratch to be the final product to meet client acceptance
+    <t>• Project planning, built on client concepts to design games contents from scratch to be the final product to meet client acceptance
 • Researched and designed monetization for F2P games, targeted to both free and paid mobile users
 • Level designing with Unity to generate stage patterns, level progress, difficulty level and perform own unit, integration and system testing to cover low end devices
 • Coordinated with the production team closely and managed sprint goal planning.</t>
@@ -858,7 +859,7 @@
     <t>Totem Defender เป็นเกม Tower Defense แบบ Free-to-Play บนมือถือ ผู้เล่นใช้โทเท็มป้องกันศัตรูที่บุกเข้ามาเป็นระลอกไปในหลายด่านและหลายระดับความยาก</t>
   </si>
   <si>
-    <t xml:space="preserve">• วางแผนโปรเจกต์ ออกแบบเนื้อหาเกมตั้งแต่ต้นจนถึง Final Product ตามคอนเซ็ปต์ลูกค้า
+    <t>• วางแผนโปรเจกต์ ออกแบบเนื้อหาเกมตั้งแต่ต้นจนถึง Final Product ตามคอนเซ็ปต์ลูกค้า
 • วิจัยและออกแบบระบบ Monetization สำหรับเกม F2P รองรับทั้งผู้เล่นฟรีและจ่ายเงิน
 • ทำ Level Design ด้วย Unity สร้าง Stage Pattern, Level Progress และ Difficulty พร้อมทดสอบให้รองรับมือถือ Spec ต่ำ
 • ประสานงานกับทีม Production อย่างใกล้ชิด และจัดการ Sprint Goal Planning</t>
@@ -876,7 +877,7 @@
     <t>Mes Comptines for 3DS is a children's music game on Nintendo 3DS that combines karaoke and rhythm tap gameplay, helping kids sing along to French nursery rhymes.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Built on client concepts to design additional game play from karaoke to rhythm tap game to meet client acceptance
+    <t>• Built on client concepts to design additional game play from karaoke to rhythm tap game to meet client acceptance
 • Level designing, improved learning curve to cover more target players and replayability with various difficulty levels
 • Game version controlling and submitting game builds via Nintendo with LotCheck guidelines.</t>
   </si>
@@ -887,7 +888,7 @@
     <t>Mes Comptines for 3DS เป็นเกมดนตรีสำหรับเด็กบน Nintendo 3DS ผสมผสานระหว่างคาราโอเกะกับเกมจังหวะตามจังหวะ ช่วยให้เด็กร้องตามเพลงกล่อมเด็กภาษาฝรั่งเศส</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบ Gameplay เพิ่มเติมจากคาราโอเกะไปสู่เกมจังหวะตามจังหวะ ตามคอนเซ็ปต์ของลูกค้า
+    <t>• ออกแบบ Gameplay เพิ่มเติมจากคาราโอเกะไปสู่เกมจังหวะตามจังหวะ ตามคอนเซ็ปต์ของลูกค้า
 • ปรับปรุง Learning Curve ให้ครอบคลุมผู้เล่นหลายกลุ่ม และเพิ่ม Replayability ด้วยระดับความยากหลายระดับ
 • คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</t>
   </si>
@@ -946,7 +947,7 @@
     <t>Lolirock is a music and karaoke game based on the Lolirock animated series, featuring character and stage customization with mini-games synced to the show's vocal lines.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Level designing, design karaoke pitch level and synced to vocal line
+    <t>• Level designing, design karaoke pitch level and synced to vocal line
 • Functional and regression testing to mini game, character and stage customization.</t>
   </si>
   <si>
@@ -956,7 +957,7 @@
     <t>เกมดนตรีและคาราโอเกะที่อิงจากการ์ตูน Lolirock มี Mini Game ซิงกับเสียงร้อง พร้อมออกแบบตัวละครและเวที</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบ Karaoke Pitch Level ให้ซิงค์กับ Vocal
+    <t>• ออกแบบ Karaoke Pitch Level ให้ซิงค์กับ Vocal
 • ทำ Functional และ Regression Test ให้กับ Mini Game รวมถึงระบบตัวละครและเวที</t>
   </si>
   <si>
@@ -972,7 +973,7 @@
     <t>Meine ersten Mitsing-Lieder for WiiU is a children's karaoke game on Nintendo WiiU (remastered from the Wii version), featuring German nursery rhymes with peripheral device support.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Remastering from Wii to WiiU version, functional and regression testing with peripheral devices
+    <t>• Remastering from Wii to WiiU version, functional and regression testing with peripheral devices
 • Customer supporting and services
 • Game version controlling and submitting game builds via Nintendo with LotCheck guidelines.</t>
   </si>
@@ -983,7 +984,7 @@
     <t>เกมคาราโอเกะสำหรับเด็กบน Nintendo Wii U (ปรับจากเวอร์ชัน Wii) ร้องเพลงกล่อมเด็กภาษาเยอรมัน พร้อมรองรับอุปกรณ์เสริม</t>
   </si>
   <si>
-    <t xml:space="preserve">• ปรับ Wii ไปเป็นเวอร์ชัน Wii U พร้อมทำ Functional และ Regression Test ร่วมกับอุปกรณ์เสริม
+    <t>• ปรับ Wii ไปเป็นเวอร์ชัน Wii U พร้อมทำ Functional และ Regression Test ร่วมกับอุปกรณ์เสริม
 • สนับสนุนลูกค้า
 • คุม Game Version และ Submit Build ผ่าน Nintendo ตาม LotCheck Guideline</t>
   </si>
@@ -1042,7 +1043,7 @@
     <t>AeternoBlade for 3DS is a 2D side-scrolling action game on Nintendo 3DS where players control Freyja, who uses a magical blade to manipulate time and battle enemies across multiple stages.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Handling responsibility for test tools and QA improvement processes
+    <t>• Handling responsibility for test tools and QA improvement processes
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly
 • Handling responsibility for test tools and developing improvement processes for testing and generating game cutscenes
 • Level designing and difficulty control, fine tuning effects and particles
@@ -1056,7 +1057,7 @@
     <t>AeternoBlade for 3DS เป็นเกมแอ็กชั่นแบบ 2D Side-Scrolling บน Nintendo 3DS ผู้เล่นบังคับ Freyja ที่ใช้ดาบเวทมนต์บิดผันเวลาบุกออกต่อสู้ศัตรูผ่านหลายด่าน</t>
   </si>
   <si>
-    <t xml:space="preserve">• ดูแล Test Tools และปรับปรุงกระบวนการ QA
+    <t>• ดูแล Test Tools และปรับปรุงกระบวนการ QA
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตามที่ออกแบบไว้
 • พัฒนา Test Tools สำหรับทดสอบและสร้าง Cutscene ของเกม
 • ทำ Level Design และ Difficulty Control รวมถึง Fine-Tune Effect และ Particle
@@ -1076,7 +1077,7 @@
     <t>Deadly Premonition: The Director's Cut for Steam is a survival horror mystery game on Steam (built from the PS3 version), where players investigate a series of murders in a small American town.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Built on PS3 and Steam versions, designed additional contents, character control and customization to match with client, Steam submission requirements
+    <t>• Built on PS3 and Steam versions, designed additional contents, character control and customization to match with client, Steam submission requirements
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly as requirements.</t>
   </si>
   <si>
@@ -1086,7 +1087,7 @@
     <t>เกม Survival Horror แนวสืบสวนบน Steam (พอร์ตมาจากเวอร์ชัน PS3) ผู้เล่นสืบสวนคดีฝาต่อเนื่องในเมืองเล็กของอเมริกา</t>
   </si>
   <si>
-    <t xml:space="preserve">• พอร์ตจากเวอร์ชัน PS3 ไป Steam ออกแบบ Content เพิ่ม ระบบ Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Steam Submission
+    <t>• พอร์ตจากเวอร์ชัน PS3 ไป Steam ออกแบบ Content เพิ่ม ระบบ Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Steam Submission
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content ตาม Requirement</t>
   </si>
   <si>
@@ -1102,14 +1103,14 @@
     <t>Deadly Premonition: Director's Cut for PS3 is a survival horror mystery game on PlayStation 3 (remastered from Xbox 360), with added content, character controls, and customization.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Remastering from XBOX360 to PS3 version, designed additional contents, character control and customization to match with client, Sony submission requirements
+    <t>• Remastering from XBOX360 to PS3 version, designed additional contents, character control and customization to match with client, Sony submission requirements
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly as requirements.</t>
   </si>
   <si>
     <t>เกม Survival Horror แนวสืบสวนบน PlayStation 3 (รีมาสเตอร์จากเวอร์ชัน Xbox 360) เพิ่ม Content ระบบ Control และ Customization</t>
   </si>
   <si>
-    <t xml:space="preserve">• รีมาสเตอร์จาก Xbox 360 ไป PS3 ออกแบบ Content, Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Sony Submission
+    <t>• รีมาสเตอร์จาก Xbox 360 ไป PS3 ออกแบบ Content, Control และ Customization ให้ตรงตาม Requirement ของลูกค้าและ Sony Submission
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content</t>
   </si>
   <si>
@@ -1125,7 +1126,7 @@
     <t>Puzzle game for promotional purpose</t>
   </si>
   <si>
-    <t xml:space="preserve">• Created game design for promotional purposes
+    <t>• Created game design for promotional purposes
 • Functional, level design and regression testing</t>
   </si>
   <si>
@@ -1135,7 +1136,7 @@
     <t>เกมพัซเซิลใช้ในการโปรโมทสินค้า</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบเกมสำหรับ เพื่องานโปรโมต
+    <t>• ออกแบบเกมสำหรับ เพื่องานโปรโมต
 • ทำ Functional level design และ Regression Test</t>
   </si>
   <si>
@@ -1151,7 +1152,7 @@
     <t>Wicked Monster BLAST! for PS3 is a casual arcade shooting game on PlayStation 3, where players blast monsters across colorful stages with party-style multiplayer gameplay.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Game, level designing and art asset control, produced from the beginning to final product
+    <t>• Game, level designing and art asset control, produced from the beginning to final product
 • Functional, regression, playthrough testing to ensure the game can progress and unlock all contents as designed correctly
 • Game version controlling and submitting game builds and to Sony PlayStation.</t>
   </si>
@@ -1162,7 +1163,7 @@
     <t>เกมยิงปีศาจแนวอาร์เคดบน PlayStation 3 ผู้เล่นยิงมอนสเตอร์ผ่านสเตจสีสัน รองรับ Multiplayer สไตล์ปาร์ตี้</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบเกม Level Design และควบคุม Art Asset ตั้งแต่ต้นจน Final Product
+    <t>• ออกแบบเกม Level Design และควบคุม Art Asset ตั้งแต่ต้นจน Final Product
 • ทำ Functional, Regression และ Playthrough Testing รองรับลำดับเกมและการปลดล็อค Content
 • คุม Game Version และ Submit Build ไป Sony PlayStation</t>
   </si>
@@ -1179,7 +1180,7 @@
     <t>Crazy Strike Bowling for PS3 is a casual bowling game on PlayStation 3 released in US, EU, and Asia regions, featuring fun pin layouts, obstacles, and physics-based gameplay.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Functional, regression and playthrough testing to ensure player can go through to all area
+    <t>• Functional, regression and playthrough testing to ensure player can go through to all area
 • Handling responsibility for test tools and developing improvement processes for testing, pin, obstacle and physic editor
 • Game version controlling and submitting game builds Sony PlayStation US, EU, and Asia.</t>
   </si>
@@ -1190,7 +1191,7 @@
     <t>เกมโบวลิ่งแนวแคชวลบน PlayStation 3 วางจำหน่ายใน US, EU และ เอเชีย มีรูปแบบ Pin อุปสรรค และ Gameplay อิง Physic สนุกสนาน</t>
   </si>
   <si>
-    <t xml:space="preserve">• ทำ Functional, Regression และ Playthrough Testing ให้ผู้เล่นสามารถผ่านไปได้ทุกพื้นที่ของเกม
+    <t>• ทำ Functional, Regression และ Playthrough Testing ให้ผู้เล่นสามารถผ่านไปได้ทุกพื้นที่ของเกม
 • ดูแล Test Tools และพัฒนา Pin, Obstacle และ Physic Editor
 • คุม Game Version และ Submit Build ไป Sony PlayStation US, EU และ Asia</t>
   </si>
@@ -1207,7 +1208,7 @@
     <t>Wicked Monsters Type! is a Google HTML5 typing game made for promotional purposes, reusing art assets from the original Wicked Monsters shooting game in a typing-based format.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Created game design for promotional purposes as a Google HTML5 game
+    <t>• Created game design for promotional purposes as a Google HTML5 game
 • Transfer art assets from the original shooting game to typing game
 • Functional and regression testing to ensure the game meets google game acceptance.</t>
   </si>
@@ -1218,7 +1219,7 @@
     <t>เกมฝึกพิมพ์บน Google HTML5 สร้างขึ้นเพื่องานโปรโมต โดยนำ Art Asset จาก Wicked Monsters ต้นฉบับมาปรับให้เป็นเกมแนวพิมพ์ดีด</t>
   </si>
   <si>
-    <t xml:space="preserve">• ออกแบบเกมสำหรับ Google HTML5 เพื่องานโปรโมต
+    <t>• ออกแบบเกมสำหรับ Google HTML5 เพื่องานโปรโมต
 • ย้าย Art Asset จากเกมต้นฉบับมาสู่เกมแนวพิมพ์
 • ทำ Functional และ Regression Test ให้ผ่านตามมาตรฐานของ Google Game</t>
   </si>
@@ -1235,7 +1236,7 @@
     <t>B-Units: Build It! is a 2D casual construction game where players complete mini-games to build structures, featuring colorful characters and quick tasks. The project involved functional and playthrough testing, game level controlling, and handling test tools for process improvement.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Functional and playthrough testing and game level controlling
+    <t>• Functional and playthrough testing and game level controlling
 • Handling responsibility for test tools and developing improvement process for testing, managed script editor for level control.</t>
   </si>
   <si>
@@ -1245,7 +1246,7 @@
     <t>B-Units: Build It! เป็นเกมก่อสร้างแนวแคชวลแบบ 2D ผู้เล่นต้องผ่าน Mini Game เพื่อสร้างสิ่งปลูกสร้างต่างๆ มีตัวละครสีสันและภารกิจรวดเร็ว</t>
   </si>
   <si>
-    <t xml:space="preserve">• ทำ Functional และ Playthrough Testing พร้อมควบคุม Game Level
+    <t>• ทำ Functional และ Playthrough Testing พร้อมควบคุม Game Level
 • ดูแล Test Tools และพัฒนากระบวนการทดสอบ รวมถึง Script Editor สำหรับ Level Control</t>
   </si>
   <si>
@@ -1261,7 +1262,7 @@
     <t>Wicked Monsters BLAST! is a 2D casual shooting game developed by Thai studio Corecell Technology, supporting up to 4 players with fast-paced, arcade-style mini-games.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Level designer
+    <t>• Level designer
 • Quality assurance
 • Lead Tester
 • Release Control.</t>
@@ -1273,7 +1274,7 @@
     <t>Wicked Monsters BLAST! เป็นเกมยิงแนว 2D พัฒนาโดยสตูดิโอไทย Corecell Technology รองรับผู้เล่นสูงสุด 4 คน มาพร้อม Mini Game สไตล์อาร์เคดสนุกๆ</t>
   </si>
   <si>
-    <t xml:space="preserve">• Level Designer
+    <t>• Level Designer
 • Quality Assurance
 • Lead Tester
 • Release Control</t>
@@ -1327,7 +1328,7 @@
     <t>MegaXGame is a Thai gaming magazine known for its comprehensive coverage, expert walkthroughs, and deep dives into the gaming world.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Fast and simple updates on new releases.
+    <t>• Fast and simple updates on new releases.
 • Honest opinions and gameplay breakdowns.
 • Deep dives into combos and fighting mechanics.
 • Selecting visuals and engaging with the community.</t>
@@ -1342,14 +1343,11 @@
     <t>MegaXGame เป็นนิตยสารที่อยู่คู่เกมเมอร์ไทยมานาน เน้นเนื้อหาที่เข้มข้น ครบเครื่อง ทั้งข่าวสาร บทสรุป และบทวิเคราะห์ที่เข้าถึงง่าย</t>
   </si>
   <si>
-    <t xml:space="preserve">• สรุปข่าวเกมใหม่แบบสั้นง่าย ทันเหตุการณ์
+    <t>• สรุปข่าวเกมใหม่แบบสั้นง่าย ทันเหตุการณ์
 • รีวิวจากที่เล่นจริง บอกจุดดีจุดด้อยให้คนอ่าน
 • เจาะลึกสูตร คอมโบ และเทคนิคเฉพาะทางเกมต่อสู้</t>
   </si>
   <si>
-    <t>etc</t>
-  </si>
-  <si>
     <t>43</t>
   </si>
   <si>
@@ -1362,9 +1360,6 @@
     <t>localize from Japanese to Thai</t>
   </si>
   <si>
-    <t>localization</t>
-  </si>
-  <si>
     <t>แปลภาษา</t>
   </si>
   <si>
@@ -1380,7 +1375,7 @@
     <t>Website</t>
   </si>
   <si>
-    <t xml:space="preserve">Freshy Golf
+    <t>Freshy Golf
 Wicked Monster Blast
 Wicked Monster Type
 Crazy Strike Bowling</t>
@@ -1825,24 +1820,30 @@
   </si>
   <si>
     <t>Python, openpyxl, pandas, Jinja2, HTML, CSS</t>
+  </si>
+  <si>
+    <t>etc.</t>
+  </si>
+  <si>
+    <t>blazblue</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -2226,9 +2227,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
@@ -2241,7 +2242,7 @@
     <col min="11" max="11" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2276,7 +2277,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2312,15 +2313,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:K1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
@@ -2331,7 +2332,7 @@
     <col min="10" max="10" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>51</v>
       </c>
@@ -2363,63 +2364,63 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>533</v>
+      </c>
+      <c r="B2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C2" t="s">
         <v>535</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>536</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>537</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>538</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
         <v>539</v>
       </c>
-      <c r="F2" t="s">
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>540</v>
       </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="B3" t="s">
         <v>541</v>
       </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
+        <v>463</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
         <v>542</v>
       </c>
-      <c r="B3" t="s">
+      <c r="F3" t="s">
         <v>543</v>
       </c>
-      <c r="C3" t="s">
-        <v>465</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
         <v>544</v>
       </c>
-      <c r="F3" t="s">
-        <v>545</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>546</v>
-      </c>
       <c r="I3" t="s">
         <v>15</v>
       </c>
@@ -2428,15 +2429,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J1" xr:uid="{00000000-0009-0000-0000-000009000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -2445,7 +2446,7 @@
     <col min="5" max="5" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -2462,7 +2463,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -2479,7 +2480,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -2496,7 +2497,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -2513,7 +2514,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -2530,7 +2531,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -2547,7 +2548,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -2564,7 +2565,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -2581,7 +2582,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -2599,15 +2600,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:XFD45"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:N45"/>
+  <sheetFormatPr defaultColWidth="18" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -2621,10 +2622,10 @@
     <col min="11" max="11" width="32" customWidth="1"/>
     <col min="12" max="13" width="55" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
-    <col min="15" max="16384" width="18" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:16384" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
@@ -2668,7 +2669,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>64</v>
       </c>
@@ -2712,7 +2713,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" ht="220.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -2756,7 +2757,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" ht="189" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="189" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -2800,7 +2801,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -2844,7 +2845,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" ht="252" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="252" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -2888,7 +2889,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>108</v>
       </c>
@@ -2932,7 +2933,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>120</v>
       </c>
@@ -2976,7 +2977,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" ht="267.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="267.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>130</v>
       </c>
@@ -3020,7 +3021,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" ht="189" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="189" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>138</v>
       </c>
@@ -3064,7 +3065,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" ht="189" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="189" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>145</v>
       </c>
@@ -3108,7 +3109,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" ht="393.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" ht="393.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>149</v>
       </c>
@@ -3152,7 +3153,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="393.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" ht="393.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>157</v>
       </c>
@@ -3196,7 +3197,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" ht="173.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" ht="173.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -3240,7 +3241,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" ht="330.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="330.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>170</v>
       </c>
@@ -3284,7 +3285,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" ht="378" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="378" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>178</v>
       </c>
@@ -3328,7 +3329,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="17" ht="378" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" ht="378" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>186</v>
       </c>
@@ -3372,7 +3373,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" ht="110.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>194</v>
       </c>
@@ -3416,7 +3417,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="409.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>202</v>
       </c>
@@ -3460,7 +3461,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="20" ht="409.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>209</v>
       </c>
@@ -3504,7 +3505,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>216</v>
       </c>
@@ -3548,7 +3549,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>223</v>
       </c>
@@ -3592,7 +3593,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" ht="252" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" ht="252" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>228</v>
       </c>
@@ -3636,7 +3637,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" ht="330.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="330.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>236</v>
       </c>
@@ -3680,7 +3681,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>244</v>
       </c>
@@ -3724,7 +3725,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>252</v>
       </c>
@@ -3768,7 +3769,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="27" ht="47.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>260</v>
       </c>
@@ -3812,7 +3813,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="28" ht="126" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" ht="126" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>266</v>
       </c>
@@ -3856,7 +3857,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="29" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>274</v>
       </c>
@@ -3900,7 +3901,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>282</v>
       </c>
@@ -3944,7 +3945,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>288</v>
       </c>
@@ -3988,7 +3989,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" ht="393.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="393.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>296</v>
       </c>
@@ -4032,7 +4033,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="33" ht="236.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>304</v>
       </c>
@@ -4076,7 +4077,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="34" ht="220.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>312</v>
       </c>
@@ -4120,7 +4121,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="35" ht="78.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>319</v>
       </c>
@@ -4164,7 +4165,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="36" ht="204.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="204.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>327</v>
       </c>
@@ -4208,7 +4209,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="37" ht="204.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="204.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>335</v>
       </c>
@@ -4252,7 +4253,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="38" ht="157.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" ht="157.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>343</v>
       </c>
@@ -4296,7 +4297,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="39" ht="141.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>351</v>
       </c>
@@ -4340,7 +4341,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="40" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>359</v>
       </c>
@@ -4384,7 +4385,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="41" ht="94.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" ht="94.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>367</v>
       </c>
@@ -4428,7 +4429,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="42" ht="47.25" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>373</v>
       </c>
@@ -4472,7 +4473,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="43" ht="141.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>380</v>
       </c>
@@ -4498,77 +4499,77 @@
         <v>387</v>
       </c>
       <c r="N43" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="44" ht="31.5" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="B44" t="s">
         <v>389</v>
       </c>
-      <c r="B44" t="s">
+      <c r="E44" t="s">
         <v>390</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>391</v>
       </c>
-      <c r="F44" t="s">
+      <c r="I44" t="s">
+        <v>546</v>
+      </c>
+      <c r="K44" t="s">
         <v>392</v>
       </c>
-      <c r="I44" t="s">
+      <c r="L44" t="s">
         <v>393</v>
       </c>
-      <c r="K44" t="s">
+      <c r="M44" t="s">
         <v>394</v>
       </c>
-      <c r="L44" t="s">
+      <c r="N44" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>395</v>
       </c>
-      <c r="M44" t="s">
+      <c r="B45" t="s">
         <v>396</v>
       </c>
-      <c r="N44" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="45" ht="63" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="E45" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="B45" t="s">
+      <c r="F45" t="s">
         <v>398</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="I45" t="s">
         <v>399</v>
       </c>
-      <c r="F45" t="s">
+      <c r="K45" t="s">
         <v>400</v>
       </c>
-      <c r="I45" t="s">
+      <c r="L45" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="M45" t="s">
         <v>401</v>
       </c>
-      <c r="K45" t="s">
-        <v>402</v>
-      </c>
-      <c r="L45" s="2" t="s">
-        <v>399</v>
-      </c>
-      <c r="M45" t="s">
-        <v>403</v>
-      </c>
       <c r="N45" t="s">
-        <v>388</v>
+        <v>545</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:XFD1"/>
+  <autoFilter ref="A1:XFD1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -4576,44 +4577,44 @@
     <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>406</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>408</v>
       </c>
-      <c r="B2" t="s">
-        <v>409</v>
-      </c>
-      <c r="C2" t="s">
-        <v>410</v>
-      </c>
       <c r="D2" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:D1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
@@ -4622,296 +4623,296 @@
     <col min="6" max="6" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>411</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>413</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>415</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="B2" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>417</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>418</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>416</v>
+      </c>
+      <c r="F2" t="s">
         <v>419</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>420</v>
       </c>
-      <c r="E2" t="s">
-        <v>418</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="B3" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>422</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>423</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>421</v>
+      </c>
+      <c r="F3" t="s">
         <v>424</v>
       </c>
-      <c r="D3" t="s">
+    </row>
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>425</v>
       </c>
-      <c r="E3" t="s">
-        <v>423</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="B4" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>427</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>428</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
+        <v>426</v>
+      </c>
+      <c r="F4" t="s">
         <v>429</v>
       </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>430</v>
       </c>
-      <c r="E4" t="s">
-        <v>428</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="B5" t="s">
         <v>431</v>
       </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>432</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>433</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
+        <v>431</v>
+      </c>
+      <c r="F5" t="s">
         <v>434</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>430</v>
+      </c>
+      <c r="B6" t="s">
         <v>435</v>
       </c>
-      <c r="E5" t="s">
-        <v>433</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="C6" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>432</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>437</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>435</v>
+      </c>
+      <c r="F6" t="s">
         <v>438</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>439</v>
       </c>
-      <c r="E6" t="s">
-        <v>437</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="B7" t="s">
         <v>440</v>
       </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="C7" t="s">
         <v>441</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>442</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
+        <v>440</v>
+      </c>
+      <c r="F7" t="s">
         <v>443</v>
       </c>
-      <c r="D7" t="s">
+    </row>
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>444</v>
       </c>
-      <c r="E7" t="s">
-        <v>442</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="B8" t="s">
         <v>445</v>
       </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C8" t="s">
         <v>446</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
         <v>447</v>
       </c>
-      <c r="C8" t="s">
+      <c r="E8" t="s">
+        <v>445</v>
+      </c>
+      <c r="F8" t="s">
         <v>448</v>
       </c>
-      <c r="D8" t="s">
-        <v>449</v>
-      </c>
-      <c r="E8" t="s">
-        <v>447</v>
-      </c>
-      <c r="F8" t="s">
-        <v>450</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>451</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" t="s">
         <v>452</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>453</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>454</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
         <v>455</v>
       </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>456</v>
       </c>
-      <c r="B3" t="s">
-        <v>457</v>
-      </c>
-      <c r="C3" t="s">
-        <v>458</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1"/>
+  <autoFilter ref="A1:C1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>459</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
         <v>460</v>
       </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>461</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>462</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" t="s">
+        <v>460</v>
+      </c>
+      <c r="C3" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>464</v>
       </c>
-      <c r="B3" t="s">
-        <v>462</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
         <v>465</v>
       </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>466</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>467</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
         <v>468</v>
       </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>469</v>
-      </c>
-      <c r="B5" t="s">
-        <v>470</v>
-      </c>
       <c r="C5" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1"/>
+  <autoFilter ref="A1:C1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -4919,65 +4920,65 @@
     <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>471</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B2" t="s">
         <v>472</v>
       </c>
-    </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>473</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>474</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>475</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3" t="s">
         <v>476</v>
       </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>477</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>475</v>
+      </c>
+      <c r="B4" t="s">
         <v>478</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>479</v>
       </c>
-      <c r="D3" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>477</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>480</v>
-      </c>
-      <c r="C4" t="s">
-        <v>481</v>
-      </c>
-      <c r="D4" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>482</v>
       </c>
       <c r="B5" t="s">
         <v>368</v>
@@ -4986,370 +4987,370 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D1"/>
+  <autoFilter ref="A1:D1" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:B43"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>482</v>
+      </c>
+      <c r="B2" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>484</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>485</v>
       </c>
-    </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B4" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>486</v>
       </c>
-      <c r="B3" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B5" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>487</v>
       </c>
-      <c r="B4" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>488</v>
       </c>
-      <c r="B5" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B7" t="s">
         <v>489</v>
       </c>
-      <c r="B6" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>490</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B9" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>492</v>
       </c>
-      <c r="B8" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B10" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>493</v>
       </c>
-      <c r="B9" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="10" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B11" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>494</v>
       </c>
-      <c r="B10" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B12" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>495</v>
-      </c>
-      <c r="B11" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>496</v>
-      </c>
-      <c r="B12" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="13" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>497</v>
       </c>
       <c r="B13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="B15" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>499</v>
+      </c>
+      <c r="B17" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>501</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>502</v>
       </c>
-    </row>
-    <row r="18" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B19" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>503</v>
       </c>
-      <c r="B18" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="B20" t="s">
         <v>504</v>
       </c>
-      <c r="B19" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>505</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>506</v>
       </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B22" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>507</v>
       </c>
-      <c r="B21" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B23" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>508</v>
       </c>
-      <c r="B22" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B24" t="s">
         <v>509</v>
       </c>
-      <c r="B23" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>510</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B25" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B26" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>512</v>
       </c>
-      <c r="B25" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="B27" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>513</v>
       </c>
-      <c r="B26" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B28" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>514</v>
       </c>
-      <c r="B27" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B29" t="s">
         <v>515</v>
       </c>
-      <c r="B28" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    </row>
+    <row r="30" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>516</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>517</v>
       </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B31" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>518</v>
       </c>
-      <c r="B30" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B32" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>519</v>
       </c>
-      <c r="B31" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B33" t="s">
         <v>520</v>
       </c>
-      <c r="B32" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>521</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>522</v>
       </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B35" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>523</v>
       </c>
-      <c r="B34" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B36" t="s">
         <v>524</v>
       </c>
-      <c r="B35" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    </row>
+    <row r="37" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>525</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>526</v>
       </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B38" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>527</v>
       </c>
-      <c r="B37" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B39" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>528</v>
       </c>
-      <c r="B38" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B40" t="s">
         <v>529</v>
       </c>
-      <c r="B39" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>530</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B42" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>532</v>
       </c>
-      <c r="B41" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>533</v>
-      </c>
-      <c r="B42" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>534</v>
-      </c>
       <c r="B43" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1"/>
+  <autoFilter ref="A1:B1" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>